<commit_message>
talla los 74 requisitos del mvp
se llena solo la columna e, con la escala de la propia hoja: s=2, m=5, l=10 y
xl=20 días hábiles, y 1 sprint = 10 días.

el criterio de pertenencia al mvp es el dibujo, requisito por requisito, no la
columna «¿en mvp?» que se deriva por épica. entran solicitud, evaluación,
siniestro integral, los canales que el mvp habilita, las capas 1 y 2 de la torre,
el principio de acceso al dato vía el core y los transversales del ciclo de
mejora y del plano de control.

quedan sin talla coordinación, prestación, finalización, asignación, nexo, ava,
la interoperabilidad de autorizaciones y las capas 3, 4 y 5 de la torre.

suma: 500 días hábiles, 50 sprints de un frente. rf-001 y rf-008 ya tenían talla
y se respetan.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SURA/gestores-sura/estimacin mvp/2 Gestores_Seguimiento_Requerimientos_2026.xlsx
+++ b/SURA/gestores-sura/estimacin mvp/2 Gestores_Seguimiento_Requerimientos_2026.xlsx
@@ -1291,7 +1291,11 @@
           <t>Documentos aparentemente inválidos se debe sugerir en pantalla que se revisen antes de enviar la solicitud, sin embargo no se debe restringir el ingreso (agente IA light).</t>
         </is>
       </c>
-      <c r="E6" s="54" t="n"/>
+      <c r="E6" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F6" s="53">
         <f>IF($E6="",0,INDEX($M$5:$M$8,MATCH($E6,$L$5:$L$8,0)))</f>
         <v/>
@@ -1339,7 +1343,11 @@
           <t>Omnicanalidad real: el historial de solicitudes/autorizaciones debe verse igual sin importar el canal de origen.</t>
         </is>
       </c>
-      <c r="E7" s="54" t="n"/>
+      <c r="E7" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F7" s="53">
         <f>IF($E7="",0,INDEX($M$5:$M$8,MATCH($E7,$L$5:$L$8,0)))</f>
         <v/>
@@ -1390,7 +1398,11 @@
 Para el asegurado y asesor SIEMPRE se deben solicitar los documentos adjuntos (orden médica e historia clinica), no se debe habilitar el ingreso de datos manuales.</t>
         </is>
       </c>
-      <c r="E8" s="54" t="n"/>
+      <c r="E8" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F8" s="53">
         <f>IF($E8="",0,INDEX($M$5:$M$8,MATCH($E8,$L$5:$L$8,0)))</f>
         <v/>
@@ -1516,7 +1528,11 @@
           <t>Solicitar solo la identificación del asegurado (aplica solo para prestador y asesor) + 2 documentos (historia clínica y orden médica); el usuario selecciona la persona del grupo familiar para el cual requiere la autorización, indica el proveedor en el cual desea recibir la atención y adjunta los documentos.</t>
         </is>
       </c>
-      <c r="E11" s="54" t="n"/>
+      <c r="E11" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F11" s="53">
         <f>IF($E11="",0,INDEX($M$5:$M$8,MATCH($E11,$L$5:$L$8,0)))</f>
         <v/>
@@ -1592,7 +1608,11 @@
           <t>Modelo de datos "padre-hijo": la solicitud es el padre; cada servicio o cups es una solicitud hijo y debe tener un estado propio.</t>
         </is>
       </c>
-      <c r="E13" s="54" t="n"/>
+      <c r="E13" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F13" s="53">
         <f>IF($E13="",0,INDEX($M$5:$M$8,MATCH($E13,$L$5:$L$8,0)))</f>
         <v/>
@@ -1633,7 +1653,11 @@
           <t>Genera un ID temporal como número radicador (correlation ID), y almacena la información de forma temporal. (Siniestro Padre)</t>
         </is>
       </c>
-      <c r="E14" s="54" t="n"/>
+      <c r="E14" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F14" s="53">
         <f>IF($E14="",0,INDEX($M$5:$M$8,MATCH($E14,$L$5:$L$8,0)))</f>
         <v/>
@@ -1699,7 +1723,11 @@
           <t>Extrae mediante agente IA la información de los documentos adjuntos (orden médica + historia clínica).</t>
         </is>
       </c>
-      <c r="E15" s="54" t="n"/>
+      <c r="E15" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F15" s="53">
         <f>IF($E15="",0,INDEX($M$5:$M$8,MATCH($E15,$L$5:$L$8,0)))</f>
         <v/>
@@ -1763,7 +1791,11 @@
           <t>Almacena los documentos en P8, se debe conservar la lógica que se tiene para que este relacionado al número de solicitud que permita ser identificado facilmente</t>
         </is>
       </c>
-      <c r="E16" s="54" t="n"/>
+      <c r="E16" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F16" s="53">
         <f>IF($E16="",0,INDEX($M$5:$M$8,MATCH($E16,$L$5:$L$8,0)))</f>
         <v/>
@@ -1827,7 +1859,11 @@
           <t>Los documentos se suben a P8 cuando la solicitud se crea en el Core (SuraHis)</t>
         </is>
       </c>
-      <c r="E17" s="54" t="n"/>
+      <c r="E17" s="54" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F17" s="53">
         <f>IF($E17="",0,INDEX($M$5:$M$8,MATCH($E17,$L$5:$L$8,0)))</f>
         <v/>
@@ -1891,7 +1927,11 @@
           <t>Envia al Core una petición de creación de solicitud y publica un evento para que la torre de control guarde trazabilidad</t>
         </is>
       </c>
-      <c r="E18" s="54" t="n"/>
+      <c r="E18" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F18" s="53">
         <f>IF($E18="",0,INDEX($M$5:$M$8,MATCH($E18,$L$5:$L$8,0)))</f>
         <v/>
@@ -1955,7 +1995,11 @@
           <t>Autorización automática aplica para servicios clasificados como "nivel 1" (algunas no requieren soportes) ; para los niveles 3 y 4 (alto costo/riesgo) siempre van a evaluación manual.</t>
         </is>
       </c>
-      <c r="E19" s="54" t="n"/>
+      <c r="E19" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F19" s="53">
         <f>IF($E19="",0,INDEX($M$5:$M$8,MATCH($E19,$L$5:$L$8,0)))</f>
         <v/>
@@ -2275,7 +2319,11 @@
           <t>Disponer en el front al prestador el cambio de estado de la solicitud de Autorización</t>
         </is>
       </c>
-      <c r="E24" s="54" t="n"/>
+      <c r="E24" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F24" s="53">
         <f>IF($E24="",0,INDEX($M$5:$M$8,MATCH($E24,$L$5:$L$8,0)))</f>
         <v/>
@@ -2341,7 +2389,11 @@
 2. Aprobar la solicitud y enviar al agente de pertinencia</t>
         </is>
       </c>
-      <c r="E25" s="54" t="n"/>
+      <c r="E25" s="54" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
       <c r="F25" s="53">
         <f>IF($E25="",0,INDEX($M$5:$M$8,MATCH($E25,$L$5:$L$8,0)))</f>
         <v/>
@@ -2405,7 +2457,11 @@
           <t>Revisar la integración para consultar mora (ir directamente al core de PDN o pasar por SuraHis).</t>
         </is>
       </c>
-      <c r="E26" s="54" t="n"/>
+      <c r="E26" s="54" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F26" s="53">
         <f>IF($E26="",0,INDEX($M$5:$M$8,MATCH($E26,$L$5:$L$8,0)))</f>
         <v/>
@@ -2469,7 +2525,11 @@
           <t>Reutiliza el homologador de CUPS y el motor ya productivo del proyecto de autorizaciones EPS, en vez de partir de cero.</t>
         </is>
       </c>
-      <c r="E27" s="54" t="n"/>
+      <c r="E27" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F27" s="53">
         <f>IF($E27="",0,INDEX($M$5:$M$8,MATCH($E27,$L$5:$L$8,0)))</f>
         <v/>
@@ -2533,7 +2593,11 @@
           <t>Valida la pertinencia médica; decide autorizar o escalar a evaluación manual (coherencia orden médica/historia clínica, CIE-10/CUPS, score de complejidad).</t>
         </is>
       </c>
-      <c r="E28" s="54" t="n"/>
+      <c r="E28" s="54" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
       <c r="F28" s="53">
         <f>IF($E28="",0,INDEX($M$5:$M$8,MATCH($E28,$L$5:$L$8,0)))</f>
         <v/>
@@ -2597,7 +2661,11 @@
           <t>Regla crítica: la negación nunca se hace 100% automática — toda negación exige intervención de un evaluador humano (administrativa vs. por pertinencia médica).</t>
         </is>
       </c>
-      <c r="E29" s="54" t="n"/>
+      <c r="E29" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F29" s="53">
         <f>IF($E29="",0,INDEX($M$5:$M$8,MATCH($E29,$L$5:$L$8,0)))</f>
         <v/>
@@ -2661,7 +2729,11 @@
           <t>Niveles de escalamiento: Nivel 1 automático · Nivel 2 administrativo · Niveles 3 (enfermeras/instrumentadoras) y 4 (médicos/especialistas).</t>
         </is>
       </c>
-      <c r="E30" s="54" t="n"/>
+      <c r="E30" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F30" s="53">
         <f>IF($E30="",0,INDEX($M$5:$M$8,MATCH($E30,$L$5:$L$8,0)))</f>
         <v/>
@@ -2697,7 +2769,11 @@
           <t>El agente entrega un "concepto"/resumen de su análisis al escalar a la bandeja manual, para acelerar la revisión humana.</t>
         </is>
       </c>
-      <c r="E31" s="54" t="n"/>
+      <c r="E31" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F31" s="53">
         <f>IF($E31="",0,INDEX($M$5:$M$8,MATCH($E31,$L$5:$L$8,0)))</f>
         <v/>
@@ -2733,7 +2809,11 @@
           <t>No genera el número de solicitud de autorización/negación: deja el caso listo vía evento — el consecutivo lo genera SuraHis.</t>
         </is>
       </c>
-      <c r="E32" s="54" t="n"/>
+      <c r="E32" s="54" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F32" s="53">
         <f>IF($E32="",0,INDEX($M$5:$M$8,MATCH($E32,$L$5:$L$8,0)))</f>
         <v/>
@@ -2769,7 +2849,11 @@
           <t>Valida duplicidad (mismo prestador/documentos o mismo tipo de servicio) consultando histórico en SuraHis; casos sospechosos van a bandeja manual con nivel + prioridad + explicación, sin negación automática.</t>
         </is>
       </c>
-      <c r="E33" s="54" t="n"/>
+      <c r="E33" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F33" s="53">
         <f>IF($E33="",0,INDEX($M$5:$M$8,MATCH($E33,$L$5:$L$8,0)))</f>
         <v/>
@@ -3459,7 +3543,11 @@
           <t>Recolectar información de todos los gestores para mapear las novedades del ciclo de la solicitud (Monitoreo funcional del proceso end-to-end sobre los seis momentos definidos en el Caso de Negocio de Gestores (Solicitud, Evaluación, Coordinación, Prestación, Monitoreo, Finalización), no solo del ciclo de vida de la autorización)</t>
         </is>
       </c>
-      <c r="E52" s="54" t="n"/>
+      <c r="E52" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F52" s="53">
         <f>IF($E52="",0,INDEX($M$5:$M$8,MATCH($E52,$L$5:$L$8,0)))</f>
         <v/>
@@ -3531,7 +3619,11 @@
           <t>Visión unificada del caso o “siniestro padre”: la Torre de Control debe presentar una vista consolidada única del caso, enlazando la solicitud, la autorización y el siniestro relacionado bajo un mismo identificador padre, en lugar de vistas fragmentadas por sistema de origen.</t>
         </is>
       </c>
-      <c r="E54" s="54" t="n"/>
+      <c r="E54" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F54" s="53">
         <f>IF($E54="",0,INDEX($M$5:$M$8,MATCH($E54,$L$5:$L$8,0)))</f>
         <v/>
@@ -3675,7 +3767,11 @@
           <t>Detecta solicitudes repetidas (2 o más veces) con las mismas características y activa el mismo flujo de rescate con mensaje diferenciado, notificando al asegurado y al gestor de solicitud para bloquear la radicación de una nueva solicitud</t>
         </is>
       </c>
-      <c r="E58" s="54" t="n"/>
+      <c r="E58" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F58" s="53">
         <f>IF($E58="",0,INDEX($M$5:$M$8,MATCH($E58,$L$5:$L$8,0)))</f>
         <v/>
@@ -3783,7 +3879,11 @@
           <t>El Portal Proveedor es el canal priorizado para el Release 1 del MVP y SVP Cliente</t>
         </is>
       </c>
-      <c r="E61" s="54" t="n"/>
+      <c r="E61" s="54" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F61" s="53">
         <f>IF($E61="",0,INDEX($M$5:$M$8,MATCH($E61,$L$5:$L$8,0)))</f>
         <v/>
@@ -3819,7 +3919,11 @@
           <t>La selección de prestador no es necesaria en la solicitud inicial, se debe sugerir el prestador cuando se tenga idetificado el servicio que solicita.</t>
         </is>
       </c>
-      <c r="E62" s="54" t="n"/>
+      <c r="E62" s="54" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F62" s="53">
         <f>IF($E62="",0,INDEX($M$5:$M$8,MATCH($E62,$L$5:$L$8,0)))</f>
         <v/>
@@ -4251,7 +4355,11 @@
           <t>Principio de responsabilidad única: si Gestores necesita un dato o funcionalidad de interoperabilidad, primero debe solicitarlo a través de SuraHIS (el core); una conexión directa de Gestores a Interoperabilidad solo se justifica cuando SuraHIS no tiene o no va a tener ese dato.</t>
         </is>
       </c>
-      <c r="E74" s="54" t="n"/>
+      <c r="E74" s="54" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F74" s="53">
         <f>IF($E74="",0,INDEX($M$5:$M$8,MATCH($E74,$L$5:$L$8,0)))</f>
         <v/>
@@ -4827,7 +4935,11 @@
           <t>Se descarta construir un formulario de diligenciamiento propio para el prestador (equivalente al actual de ADR); el prestador que ingrese por el Front usará el mismo componente de carga de documentos (orden médica + historia clínica) que cliente y asesor, para minimizar el esfuerzo de construcción.</t>
         </is>
       </c>
-      <c r="E90" s="54" t="n"/>
+      <c r="E90" s="54" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F90" s="53">
         <f>IF($E90="",0,INDEX($M$5:$M$8,MATCH($E90,$L$5:$L$8,0)))</f>
         <v/>
@@ -5223,7 +5335,11 @@
           <t xml:space="preserve">Concepto de “gestor auditor” dentro de cada gestor y en torre de control nos permita ver el comportamiento y sugerencias para mejorar la autonomía del gestor </t>
         </is>
       </c>
-      <c r="E101" s="54" t="n"/>
+      <c r="E101" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F101" s="53">
         <f>IF($E101="",0,INDEX($M$5:$M$8,MATCH($E101,$L$5:$L$8,0)))</f>
         <v/>
@@ -5655,7 +5771,11 @@
           <t>Arquitectura de microservicios, agéntica, dirigida por eventos (EDA), moderna y desacoplada — se acopla a los cores existentes, no los reemplaza.</t>
         </is>
       </c>
-      <c r="E113" s="54" t="n"/>
+      <c r="E113" s="54" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
       <c r="F113" s="53">
         <f>IF($E113="",0,INDEX($M$5:$M$8,MATCH($E113,$L$5:$L$8,0)))</f>
         <v/>
@@ -5691,7 +5811,11 @@
           <t>El core (SuraHis) debe ser la fuente de la verdad transaccional, no el motor de reglas — principio validado repetidamente por arquitectura.</t>
         </is>
       </c>
-      <c r="E114" s="54" t="n"/>
+      <c r="E114" s="54" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F114" s="53">
         <f>IF($E114="",0,INDEX($M$5:$M$8,MATCH($E114,$L$5:$L$8,0)))</f>
         <v/>
@@ -5763,7 +5887,11 @@
           <t>Cada gestor tendría base de datos propia, independiente y desacoplada.</t>
         </is>
       </c>
-      <c r="E116" s="54" t="n"/>
+      <c r="E116" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F116" s="53">
         <f>IF($E116="",0,INDEX($M$5:$M$8,MATCH($E116,$L$5:$L$8,0)))</f>
         <v/>
@@ -5799,7 +5927,11 @@
           <t>Se reutiliza la arquitectura de "Siniestro Integral" ( Back, API Gateway, orquestador, storage, colas) como base común de varios gestores.</t>
         </is>
       </c>
-      <c r="E117" s="54" t="n"/>
+      <c r="E117" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F117" s="53">
         <f>IF($E117="",0,INDEX($M$5:$M$8,MATCH($E117,$L$5:$L$8,0)))</f>
         <v/>
@@ -5835,7 +5967,11 @@
           <t>Se privilegia un front único reutilizable por canal/actor, en lugar de un front independiente por cada gestor.</t>
         </is>
       </c>
-      <c r="E118" s="54" t="n"/>
+      <c r="E118" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F118" s="53">
         <f>IF($E118="",0,INDEX($M$5:$M$8,MATCH($E118,$L$5:$L$8,0)))</f>
         <v/>
@@ -5871,7 +6007,11 @@
           <t>Diferenciación explícita comando (síncrono, se consume y desaparece) vs. evento (inmutable, usado para trazabilidad).</t>
         </is>
       </c>
-      <c r="E119" s="54" t="n"/>
+      <c r="E119" s="54" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F119" s="53">
         <f>IF($E119="",0,INDEX($M$5:$M$8,MATCH($E119,$L$5:$L$8,0)))</f>
         <v/>
@@ -5943,7 +6083,11 @@
           <t>La habilitación del proceso de Solicitudes de Salud en Siniestro Integral requiere la implementación de capacidades de integración, gestión y consulta de información, junto con adecuaciones en plataformas corporativas existentes, con el fin de asegurar la operación integral, la trazabilidad y la escalabilidad de la solución.</t>
         </is>
       </c>
-      <c r="E121" s="54" t="n"/>
+      <c r="E121" s="54" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
       <c r="F121" s="53">
         <f>IF($E121="",0,INDEX($M$5:$M$8,MATCH($E121,$L$5:$L$8,0)))</f>
         <v/>
@@ -5979,7 +6123,11 @@
           <t>Flujo: Front → Storage temporal de documentos → integración asíncrona con P8</t>
         </is>
       </c>
-      <c r="E122" s="54" t="n"/>
+      <c r="E122" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F122" s="53">
         <f>IF($E122="",0,INDEX($M$5:$M$8,MATCH($E122,$L$5:$L$8,0)))</f>
         <v/>
@@ -6015,7 +6163,11 @@
           <t>Comprobación de derechos vía API de SuraHis (no Global Web) — mayor resiliencia y flexibilidad ante cambios futuros de core.</t>
         </is>
       </c>
-      <c r="E123" s="54" t="n"/>
+      <c r="E123" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F123" s="53">
         <f>IF($E123="",0,INDEX($M$5:$M$8,MATCH($E123,$L$5:$L$8,0)))</f>
         <v/>
@@ -6087,7 +6239,11 @@
           <t>Arquitectura orientada a eventos: quien tiene autoridad sobre la entidad (normalmente SuraHis) es quien emite el evento.</t>
         </is>
       </c>
-      <c r="E125" s="54" t="n"/>
+      <c r="E125" s="54" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F125" s="53">
         <f>IF($E125="",0,INDEX($M$5:$M$8,MATCH($E125,$L$5:$L$8,0)))</f>
         <v/>
@@ -6159,7 +6315,11 @@
           <t>Custodia temporal de historia clínica/orden médica en componente propio.</t>
         </is>
       </c>
-      <c r="E127" s="54" t="n"/>
+      <c r="E127" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F127" s="53">
         <f>IF($E127="",0,INDEX($M$5:$M$8,MATCH($E127,$L$5:$L$8,0)))</f>
         <v/>
@@ -6231,7 +6391,11 @@
           <t>Consume la información ya extraída y estructurada por el gestor de Solicitud — no relee los documentos originales.</t>
         </is>
       </c>
-      <c r="E129" s="54" t="n"/>
+      <c r="E129" s="54" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F129" s="53">
         <f>IF($E129="",0,INDEX($M$5:$M$8,MATCH($E129,$L$5:$L$8,0)))</f>
         <v/>
@@ -6267,7 +6431,11 @@
           <t>Debe consultar políticas/reglas a SuraHis manteniendo también reglas propias de agente (modelo híbrido).</t>
         </is>
       </c>
-      <c r="E130" s="54" t="n"/>
+      <c r="E130" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F130" s="53">
         <f>IF($E130="",0,INDEX($M$5:$M$8,MATCH($E130,$L$5:$L$8,0)))</f>
         <v/>
@@ -6339,7 +6507,11 @@
           <t>Arquitectura híbrida multiagente propuesta: agente determinístico (coberturas/exclusiones)  + agente LLM (pertinencia médica).</t>
         </is>
       </c>
-      <c r="E132" s="54" t="n"/>
+      <c r="E132" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F132" s="53">
         <f>IF($E132="",0,INDEX($M$5:$M$8,MATCH($E132,$L$5:$L$8,0)))</f>
         <v/>
@@ -6375,7 +6547,11 @@
           <t>Las negaciones nunca serán ejecutadas automáticamente por el Gestor de Evaluación ni por modelos de IA. Toda negación debe ser una decisión determinística, trazable y auditable, gestionada a través de una bandeja manual</t>
         </is>
       </c>
-      <c r="E133" s="54" t="n"/>
+      <c r="E133" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F133" s="53">
         <f>IF($E133="",0,INDEX($M$5:$M$8,MATCH($E133,$L$5:$L$8,0)))</f>
         <v/>
@@ -6699,7 +6875,11 @@
           <t>Arquitectura orientada a eventos (EDA): consume eventos de todos los gestores y cores, incluida SuraHis.</t>
         </is>
       </c>
-      <c r="E142" s="54" t="n"/>
+      <c r="E142" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F142" s="53">
         <f>IF($E142="",0,INDEX($M$5:$M$8,MATCH($E142,$L$5:$L$8,0)))</f>
         <v/>
@@ -6735,7 +6915,11 @@
           <t>El almacenamiento de eventos vive en un bus/componente dedicado, no exclusivo de este gestor — múltiples consumidores pueden leerlo.</t>
         </is>
       </c>
-      <c r="E143" s="54" t="n"/>
+      <c r="E143" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F143" s="53">
         <f>IF($E143="",0,INDEX($M$5:$M$8,MATCH($E143,$L$5:$L$8,0)))</f>
         <v/>
@@ -7203,7 +7387,11 @@
           <t>Siniestro integral será un copmponente coreless que está en una capa superior donde se reciben las solicitudes entrantes, para luego  procesarlas desde una capa agéntica y que sean enviadas al core como información estrucutrada</t>
         </is>
       </c>
-      <c r="E156" s="54" t="n"/>
+      <c r="E156" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F156" s="53">
         <f>IF($E156="",0,INDEX($M$5:$M$8,MATCH($E156,$L$5:$L$8,0)))</f>
         <v/>
@@ -7419,7 +7607,11 @@
           <t>Los estados administrados por Gestores y los estados administrados por SuraHis se mantienen como conjuntos diferenciados (Gestores tiene estados propios adicionales, ej. “pre radicado”, que no existen en SuraHis) pero deben poder correlacionarse.</t>
         </is>
       </c>
-      <c r="E162" s="54" t="n"/>
+      <c r="E162" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F162" s="53">
         <f>IF($E162="",0,INDEX($M$5:$M$8,MATCH($E162,$L$5:$L$8,0)))</f>
         <v/>
@@ -7491,7 +7683,11 @@
           <t>Principio arquitectónico base heredado del Caso de Negocio de Gestores: arquitectura empresarial reutilizable de seis momentos, con desacople de los cores mediante eventos y microservicios.</t>
         </is>
       </c>
-      <c r="E164" s="54" t="n"/>
+      <c r="E164" s="54" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F164" s="53">
         <f>IF($E164="",0,INDEX($M$5:$M$8,MATCH($E164,$L$5:$L$8,0)))</f>
         <v/>
@@ -7527,7 +7723,11 @@
           <t>La Torre de Control debe suscribirse a la totalidad de los eventos del ecosistema (todos los gestores y cores), no a un subconjunto, como precondición técnica para construir la trazabilidad end-to-end.</t>
         </is>
       </c>
-      <c r="E165" s="54" t="n"/>
+      <c r="E165" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F165" s="53">
         <f>IF($E165="",0,INDEX($M$5:$M$8,MATCH($E165,$L$5:$L$8,0)))</f>
         <v/>
@@ -7563,7 +7763,11 @@
           <t>Contrato técnico mínimo: emisión de un evento por cada cambio de estado en cualquier gestor/core del ecosistema, como base para que la Torre de Control pueda construir la trazabilidad end-to-end.</t>
         </is>
       </c>
-      <c r="E166" s="54" t="n"/>
+      <c r="E166" s="54" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F166" s="53">
         <f>IF($E166="",0,INDEX($M$5:$M$8,MATCH($E166,$L$5:$L$8,0)))</f>
         <v/>
@@ -7599,7 +7803,11 @@
           <t>Api orquestadora por tipo de solicitud: punto único de entrada del gestor. Recibe la radicación desde el canal, crea o recupera la sesión del caso, orquesta el flujo entre los agentes y consolida la respuesta. Se publica en el API Gateway y no contiene lógica de negocio.</t>
         </is>
       </c>
-      <c r="E167" s="99" t="n"/>
+      <c r="E167" s="99" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F167" s="98">
         <f>IF($E167="",0,INDEX($M$5:$M$8,MATCH($E167,$L$5:$L$8,0)))</f>
         <v/>
@@ -7635,7 +7843,11 @@
           <t>Clasificador de documentos: identifica qué documento es cada archivo recibido (historia clínica, orden médica u otro) antes de extraer, para que el enrutador sepa qué agentes activar.</t>
         </is>
       </c>
-      <c r="E168" s="99" t="n"/>
+      <c r="E168" s="99" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F168" s="98">
         <f>IF($E168="",0,INDEX($M$5:$M$8,MATCH($E168,$L$5:$L$8,0)))</f>
         <v/>
@@ -7671,7 +7883,11 @@
           <t>Enrutador: decide qué agentes expertos se activan según el tipo de solicitud y los documentos clasificados. La ruta elegida queda registrada en la traza del caso.</t>
         </is>
       </c>
-      <c r="E169" s="99" t="n"/>
+      <c r="E169" s="99" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F169" s="98">
         <f>IF($E169="",0,INDEX($M$5:$M$8,MATCH($E169,$L$5:$L$8,0)))</f>
         <v/>
@@ -7707,7 +7923,11 @@
           <t>Agente request builder: arma la solicitud estructurada únicamente con los campos que tienen respaldo en los documentos extraídos, y marca de forma explícita los campos sin respaldo.</t>
         </is>
       </c>
-      <c r="E170" s="99" t="n"/>
+      <c r="E170" s="99" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F170" s="98">
         <f>IF($E170="",0,INDEX($M$5:$M$8,MATCH($E170,$L$5:$L$8,0)))</f>
         <v/>
@@ -7743,7 +7963,11 @@
           <t>LLM-as-a-judge: antes de enviar la solicitud al core, verifica que cumpla el contrato, que cada campo tenga respaldo en la evidencia y que la confianza supere el umbral definido para ese tipo de caso.</t>
         </is>
       </c>
-      <c r="E171" s="99" t="n"/>
+      <c r="E171" s="99" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F171" s="98">
         <f>IF($E171="",0,INDEX($M$5:$M$8,MATCH($E171,$L$5:$L$8,0)))</f>
         <v/>
@@ -7779,7 +8003,11 @@
           <t>Escalada a preradicado: cuando no se cumple el contrato o la confianza queda por debajo del umbral, el caso pasa al estado propio del gestor «preradicado», registrando motivo, umbral aplicado y confianza obtenida.</t>
         </is>
       </c>
-      <c r="E172" s="99" t="n"/>
+      <c r="E172" s="99" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F172" s="98">
         <f>IF($E172="",0,INDEX($M$5:$M$8,MATCH($E172,$L$5:$L$8,0)))</f>
         <v/>
@@ -7815,7 +8043,11 @@
           <t>Caché de reglas duras versionadas: la evaluación determinística se sustenta en reglas con versión, vigencia y autor, expuestas como herramienta determinística. Ninguna negación se sustenta en una salida probabilística.</t>
         </is>
       </c>
-      <c r="E173" s="99" t="n"/>
+      <c r="E173" s="99" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F173" s="98">
         <f>IF($E173="",0,INDEX($M$5:$M$8,MATCH($E173,$L$5:$L$8,0)))</f>
         <v/>
@@ -7851,7 +8083,11 @@
           <t>Medición de la detección de duplicidad: el acierto y los falsos positivos de la detección de solicitudes equivalentes se miden y se reportan por separado.</t>
         </is>
       </c>
-      <c r="E174" s="99" t="n"/>
+      <c r="E174" s="99" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F174" s="98">
         <f>IF($E174="",0,INDEX($M$5:$M$8,MATCH($E174,$L$5:$L$8,0)))</f>
         <v/>
@@ -7887,7 +8123,11 @@
           <t>Invocación del componente analítico y del modelo experto del dominio como herramientas del gestor, sin que el gestor absorba su lógica ni la duplique.</t>
         </is>
       </c>
-      <c r="E175" s="99" t="n"/>
+      <c r="E175" s="99" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F175" s="98">
         <f>IF($E175="",0,INDEX($M$5:$M$8,MATCH($E175,$L$5:$L$8,0)))</f>
         <v/>
@@ -7923,7 +8163,11 @@
           <t>Marca de origen: cada solicitud viaja con el canal por el que entró y ese dato se conserva en el evento, para que los casos que entran por caminos que no pasan por los gestores no contaminen la métrica de quien no participó.</t>
         </is>
       </c>
-      <c r="E176" s="99" t="n"/>
+      <c r="E176" s="99" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="F176" s="98">
         <f>IF($E176="",0,INDEX($M$5:$M$8,MATCH($E176,$L$5:$L$8,0)))</f>
         <v/>
@@ -7959,7 +8203,11 @@
           <t>Ingesta idempotente y ventana para evidencia rezagada: la torre recibe eventos y cargas garantizando idempotencia y orden, y acepta evidencia que llega semanas después sin reabrir el proceso de negocio.</t>
         </is>
       </c>
-      <c r="E177" s="99" t="n"/>
+      <c r="E177" s="99" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F177" s="98">
         <f>IF($E177="",0,INDEX($M$5:$M$8,MATCH($E177,$L$5:$L$8,0)))</f>
         <v/>
@@ -7995,7 +8243,11 @@
           <t>Contrato de eventos publicado y versionado con compatibilidad hacia atrás. El emisor que no cumple el esquema queda rechazado y el rechazo se registra como falla del emisor, no como pérdida silenciosa.</t>
         </is>
       </c>
-      <c r="E178" s="99" t="n"/>
+      <c r="E178" s="99" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F178" s="98">
         <f>IF($E178="",0,INDEX($M$5:$M$8,MATCH($E178,$L$5:$L$8,0)))</f>
         <v/>
@@ -8031,7 +8283,11 @@
           <t>Dos horizontes de retención: la traza técnica se conserva lo que dure el diagnóstico de un incidente; el registro que sustenta si una decisión estuvo bien se conserva hasta que llegue la glosa o la reclamación, y ese no se muestrea.</t>
         </is>
       </c>
-      <c r="E179" s="99" t="n"/>
+      <c r="E179" s="99" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F179" s="98">
         <f>IF($E179="",0,INDEX($M$5:$M$8,MATCH($E179,$L$5:$L$8,0)))</f>
         <v/>
@@ -8067,7 +8323,11 @@
           <t>Correlación del caso con su siniestro padre mediante llave única, de modo que la solicitud, sus servicios hijo y los eventos de todos los emisores se lean como un solo caso.</t>
         </is>
       </c>
-      <c r="E180" s="99" t="n"/>
+      <c r="E180" s="99" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F180" s="98">
         <f>IF($E180="",0,INDEX($M$5:$M$8,MATCH($E180,$L$5:$L$8,0)))</f>
         <v/>
@@ -8103,7 +8363,11 @@
           <t>Golden set por gestor: conjunto de evaluación versionado, con dueño explícito, balanceado entre casos que deben resolverse y casos que deben escalarse, y refrescado periódicamente. Cada caso corregido por una persona entra al golden set del agente responsable.</t>
         </is>
       </c>
-      <c r="E181" s="99" t="n"/>
+      <c r="E181" s="99" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F181" s="98">
         <f>IF($E181="",0,INDEX($M$5:$M$8,MATCH($E181,$L$5:$L$8,0)))</f>
         <v/>
@@ -8139,7 +8403,11 @@
           <t>Corrección estructurada: cuando una persona corrige el trabajo de un agente, se registra qué campo estaba mal, cuál era el valor correcto y de dónde salía en el documento, para que la corrección sea reutilizable como caso de evaluación.</t>
         </is>
       </c>
-      <c r="E182" s="99" t="n"/>
+      <c r="E182" s="99" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F182" s="98">
         <f>IF($E182="",0,INDEX($M$5:$M$8,MATCH($E182,$L$5:$L$8,0)))</f>
         <v/>
@@ -8175,7 +8443,11 @@
           <t>Muestreo de casos aprobados: desde el primer día se revisa una muestra fija de los casos que el agente resolvió sin escalar, y se suman casos adversarios construidos a propósito (documentos ilegibles, órdenes con dos procedimientos, contradicción entre historia y orden).</t>
         </is>
       </c>
-      <c r="E183" s="99" t="n"/>
+      <c r="E183" s="99" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F183" s="98">
         <f>IF($E183="",0,INDEX($M$5:$M$8,MATCH($E183,$L$5:$L$8,0)))</f>
         <v/>
@@ -8211,7 +8483,11 @@
           <t>Compuerta de promoción: ninguna versión de un agente, de su prompt o de su configuración llega a producción sin resultado de suite contra el golden set con criterio de no regresión. La promoción queda registrada con autor, motivo y reversión inmediata.</t>
         </is>
       </c>
-      <c r="E184" s="99" t="n"/>
+      <c r="E184" s="99" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F184" s="98">
         <f>IF($E184="",0,INDEX($M$5:$M$8,MATCH($E184,$L$5:$L$8,0)))</f>
         <v/>
@@ -8247,7 +8523,11 @@
           <t>Umbral y grado de autonomía como configuración: el umbral de confianza y el grado de autonomía de cada agente son configuración versionada del plano de control, leída en cada ejecución, y no constantes embebidas en el agente.</t>
         </is>
       </c>
-      <c r="E185" s="99" t="n"/>
+      <c r="E185" s="99" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F185" s="98">
         <f>IF($E185="",0,INDEX($M$5:$M$8,MATCH($E185,$L$5:$L$8,0)))</f>
         <v/>
@@ -8283,7 +8563,11 @@
           <t>Trazabilidad de la decisión: cada decisión de un agente queda registrada con agente, versión, prompt utilizado, umbral aplicado, confianza obtenida y herramientas invocadas, correlacionada con el caso y con su siniestro padre.</t>
         </is>
       </c>
-      <c r="E186" s="99" t="n"/>
+      <c r="E186" s="99" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="F186" s="98">
         <f>IF($E186="",0,INDEX($M$5:$M$8,MATCH($E186,$L$5:$L$8,0)))</f>
         <v/>
@@ -8319,7 +8603,11 @@
           <t>Calibración del LLM-as-a-judge contra una muestra revisada por personas expertas. El nivel de coincidencia obtenido se reporta junto a cualquier métrica que dependa de ese juez.</t>
         </is>
       </c>
-      <c r="E187" s="99" t="n"/>
+      <c r="E187" s="99" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F187" s="98">
         <f>IF($E187="",0,INDEX($M$5:$M$8,MATCH($E187,$L$5:$L$8,0)))</f>
         <v/>

</xml_diff>

<commit_message>
marca alertas, observaciones y leyenda de colores
13 requisitos quedan sin tallar y en rojo, con la duda escrita en observaciones:
rf-005, rf-018, rf-077, rt-003, rt-008, rt-012, rt-016, rt-019, rt-037, rt-038,
rt-043, rt-045 y rt-051. dos de ellos son conflictos con el lineamiento ai first
—el front en flutter frente a angular sobre static web app, y el llm multimodal
directo frente a azure document intelligence— y uno es un duplicado exacto,
rt-019 sobre rt-018.

68 filas existentes quedan en naranja: 7 que entran al mvp con salvedad y 61 que
quedan fuera y explican por qué, todas de épicas que la hoja marca «sí» o
«parcial» y donde la exclusión no era evidente.

se agrega la leyenda de colores y el criterio de alcance en la zona libre de la
hoja, debajo de la tabla de épicas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SURA/gestores-sura/estimacin mvp/2 Gestores_Seguimiento_Requerimientos_2026.xlsx
+++ b/SURA/gestores-sura/estimacin mvp/2 Gestores_Seguimiento_Requerimientos_2026.xlsx
@@ -29,7 +29,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="32">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -216,8 +216,22 @@
       <color rgb="FF0033A0"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Sura Sans"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Sura Sans"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Sura Sans"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="29">
+  <fills count="31">
     <fill>
       <patternFill/>
     </fill>
@@ -380,6 +394,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -592,7 +616,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -858,6 +882,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1323,22 +1365,22 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="53" t="inlineStr">
+      <c r="A7" s="105" t="inlineStr">
         <is>
           <t>RF-003</t>
         </is>
       </c>
-      <c r="B7" s="53" t="inlineStr">
+      <c r="B7" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C7" s="53" t="inlineStr">
+      <c r="C7" s="105" t="inlineStr">
         <is>
           <t>Canales / Front Externos</t>
         </is>
       </c>
-      <c r="D7" s="53" t="inlineStr">
+      <c r="D7" s="105" t="inlineStr">
         <is>
           <t>Omnicanalidad real: el historial de solicitudes/autorizaciones debe verse igual sin importar el canal de origen.</t>
         </is>
@@ -1348,19 +1390,23 @@
           <t>L</t>
         </is>
       </c>
-      <c r="F7" s="53">
+      <c r="F7" s="105">
         <f>IF($E7="",0,INDEX($M$5:$M$8,MATCH($E7,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G7" s="53">
+      <c r="G7" s="105">
         <f>IF($F7=0,0,$F7/10)</f>
         <v/>
       </c>
-      <c r="H7" s="53">
+      <c r="H7" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C7,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I7" s="53" t="n"/>
+      <c r="I7" s="105" t="inlineStr">
+        <is>
+          <t>Estimado acotado a los canales que el MVP habilita. La omnicanalidad sobre los ocho canales dibujados exige AVA y Nexo, que son de 2027.</t>
+        </is>
+      </c>
       <c r="L7" s="56" t="inlineStr">
         <is>
           <t>L</t>
@@ -1430,41 +1476,45 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="53" t="inlineStr">
+      <c r="A9" s="106" t="inlineStr">
         <is>
           <t>RF-005</t>
         </is>
       </c>
-      <c r="B9" s="53" t="inlineStr">
+      <c r="B9" s="106" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C9" s="53" t="inlineStr">
+      <c r="C9" s="106" t="inlineStr">
         <is>
           <t>Canales / Front Externos</t>
         </is>
       </c>
-      <c r="D9" s="53" t="inlineStr">
+      <c r="D9" s="106" t="inlineStr">
         <is>
           <t>Habilitar el canal de acceso para que los 3 tipos de publico puedan realizar solicitudes de autorización: prestador (70-80% del volumen, foco prioritario), cliente/asegurado (~15%) y asesor (~5%, tendencia a minimizarse).
 (Portal Prestador, SVP, AVA/NEXO, Super App, WH)</t>
         </is>
       </c>
-      <c r="E9" s="54" t="n"/>
-      <c r="F9" s="53">
+      <c r="E9" s="107" t="n"/>
+      <c r="F9" s="106">
         <f>IF($E9="",0,INDEX($M$5:$M$8,MATCH($E9,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G9" s="53">
+      <c r="G9" s="106">
         <f>IF($F9=0,0,$F9/10)</f>
         <v/>
       </c>
-      <c r="H9" s="53">
+      <c r="H9" s="106">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C9,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I9" s="53" t="n"/>
+      <c r="I9" s="106" t="inlineStr">
+        <is>
+          <t>🟥 No estimable como está redactado. Pide habilitar los cinco canales (Portal Prestador, SVP, AVA/Nexo, Super App, WhatsApp) para los tres públicos, pero el MVP 2026 habilita Portal Proveedor y SVP; AVA y Nexo son épicas de 2027. Acotar el requisito a los canales del MVP y volver a tallar.</t>
+        </is>
+      </c>
       <c r="L9" s="91" t="inlineStr">
         <is>
           <t>🟨 Escala de referencia (no oficial para todas las tallas): M ≈ 5 días (medio sprint) y L ≈ 10 días (1 sprint) están tomados literalmente del Acta de Estimación de Costo y Releases (21-ago-2026). S (≈3 días) y XL (≈20 días, el doble de L, por la regla de coherencia de tallaje de Víctor Martínez) son un supuesto para completar la escala — ajústelos si el equipo define otro valor. 1 sprint = 10 días hábiles (estándar SuraHis).</t>
@@ -1472,40 +1522,44 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="57" t="inlineStr">
+      <c r="A10" s="105" t="inlineStr">
         <is>
           <t>RF-006</t>
         </is>
       </c>
-      <c r="B10" s="57" t="inlineStr">
+      <c r="B10" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C10" s="57" t="inlineStr">
+      <c r="C10" s="105" t="inlineStr">
         <is>
           <t>Canales / Front Externos</t>
         </is>
       </c>
-      <c r="D10" s="57" t="inlineStr">
+      <c r="D10" s="105" t="inlineStr">
         <is>
           <t>Rescate digital automático: si falla el canal al radicar, se contacta tibbot desde el canal</t>
         </is>
       </c>
       <c r="E10" s="54" t="n"/>
-      <c r="F10" s="53">
+      <c r="F10" s="105">
         <f>IF($E10="",0,INDEX($M$5:$M$8,MATCH($E10,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G10" s="53">
+      <c r="G10" s="105">
         <f>IF($F10=0,0,$F10/10)</f>
         <v/>
       </c>
-      <c r="H10" s="53">
+      <c r="H10" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C10,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I10" s="53" t="n"/>
+      <c r="I10" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el rescate con contacto proactivo desde el canal es capacidad proactiva de la torre (capa 4), que no entra.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="53" t="inlineStr">
@@ -1703,22 +1757,22 @@
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="53" t="inlineStr">
+      <c r="A15" s="105" t="inlineStr">
         <is>
           <t>RF-011</t>
         </is>
       </c>
-      <c r="B15" s="53" t="inlineStr">
+      <c r="B15" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C15" s="53" t="inlineStr">
+      <c r="C15" s="105" t="inlineStr">
         <is>
           <t>Gestor de Evaluación</t>
         </is>
       </c>
-      <c r="D15" s="53" t="inlineStr">
+      <c r="D15" s="105" t="inlineStr">
         <is>
           <t>Extrae mediante agente IA la información de los documentos adjuntos (orden médica + historia clínica).</t>
         </is>
@@ -1728,19 +1782,23 @@
           <t>L</t>
         </is>
       </c>
-      <c r="F15" s="53">
+      <c r="F15" s="105">
         <f>IF($E15="",0,INDEX($M$5:$M$8,MATCH($E15,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G15" s="53">
+      <c r="G15" s="105">
         <f>IF($F15=0,0,$F15/10)</f>
         <v/>
       </c>
-      <c r="H15" s="53">
+      <c r="H15" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C15,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I15" s="53" t="n"/>
+      <c r="I15" s="105" t="inlineStr">
+        <is>
+          <t>El dibujo del MVP ubica los extractores en la capa de agentes expertos del Gestor de Solicitud, no en Evaluación; RT-017 confirma que Evaluación consume lo ya extraído. La talla cubre los dos extractores del MVP (historia clínica y orden).</t>
+        </is>
+      </c>
       <c r="L15" s="58" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
@@ -2043,40 +2101,44 @@
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="57" t="inlineStr">
+      <c r="A20" s="105" t="inlineStr">
         <is>
           <t>RF-016</t>
         </is>
       </c>
-      <c r="B20" s="57" t="inlineStr">
+      <c r="B20" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C20" s="57" t="inlineStr">
+      <c r="C20" s="105" t="inlineStr">
         <is>
           <t>Surahis</t>
         </is>
       </c>
-      <c r="D20" s="57" t="inlineStr">
+      <c r="D20" s="105" t="inlineStr">
         <is>
           <t>Se debe activar la Integralidad automática con EPS Sura cuando la póliza voluntaria no cubre el servicio y se genera la negación de una solicitud (régimen contributivo activo).</t>
         </is>
       </c>
       <c r="E20" s="54" t="n"/>
-      <c r="F20" s="53">
+      <c r="F20" s="105">
         <f>IF($E20="",0,INDEX($M$5:$M$8,MATCH($E20,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G20" s="53">
+      <c r="G20" s="105">
         <f>IF($F20=0,0,$F20/10)</f>
         <v/>
       </c>
-      <c r="H20" s="53">
+      <c r="H20" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C20,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I20" s="53" t="n"/>
+      <c r="I20" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del alcance de Gestores: la integralidad automática con EPS Sura es trabajo del core, y la épica está marcada N/A en esta misma hoja.</t>
+        </is>
+      </c>
       <c r="L20" s="60" t="inlineStr">
         <is>
           <t>Canales / Front Externos</t>
@@ -2107,40 +2169,44 @@
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="53" t="inlineStr">
+      <c r="A21" s="105" t="inlineStr">
         <is>
           <t>RF-017</t>
         </is>
       </c>
-      <c r="B21" s="53" t="inlineStr">
+      <c r="B21" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C21" s="53" t="inlineStr">
+      <c r="C21" s="105" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D21" s="53" t="inlineStr">
+      <c r="D21" s="105" t="inlineStr">
         <is>
           <t>Se debe habilitar la opción de "Reestudio": permite solicitar una reevaluación de una solicitud negada adjuntando nueva evidencia u observaciones, se debe conservar el mismo número de solicitud padre y se debe enviar al core con el mismo evaluador de la solicitud inicial.</t>
         </is>
       </c>
       <c r="E21" s="54" t="n"/>
-      <c r="F21" s="53">
+      <c r="F21" s="105">
         <f>IF($E21="",0,INDEX($M$5:$M$8,MATCH($E21,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G21" s="53">
+      <c r="G21" s="105">
         <f>IF($F21=0,0,$F21/10)</f>
         <v/>
       </c>
-      <c r="H21" s="53">
+      <c r="H21" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C21,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I21" s="53" t="n"/>
+      <c r="I21" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el reestudio no aparece en el dibujo. Es un flujo adicional sobre una solicitud ya negada.</t>
+        </is>
+      </c>
       <c r="L21" s="60" t="inlineStr">
         <is>
           <t>Transversal / Principios generales</t>
@@ -2171,40 +2237,44 @@
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="57" t="inlineStr">
+      <c r="A22" s="106" t="inlineStr">
         <is>
           <t>RF-018</t>
         </is>
       </c>
-      <c r="B22" s="57" t="inlineStr">
+      <c r="B22" s="106" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C22" s="57" t="inlineStr">
+      <c r="C22" s="106" t="inlineStr">
         <is>
           <t>Siniestro Integral</t>
         </is>
       </c>
-      <c r="D22" s="57" t="inlineStr">
+      <c r="D22" s="106" t="inlineStr">
         <is>
           <t>Validar si se debe publicar eventos antes de generar la solicitud oficial por parte del core</t>
         </is>
       </c>
-      <c r="E22" s="54" t="n"/>
-      <c r="F22" s="53">
+      <c r="E22" s="107" t="n"/>
+      <c r="F22" s="106">
         <f>IF($E22="",0,INDEX($M$5:$M$8,MATCH($E22,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G22" s="53">
+      <c r="G22" s="106">
         <f>IF($F22=0,0,$F22/10)</f>
         <v/>
       </c>
-      <c r="H22" s="53">
+      <c r="H22" s="106">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C22,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I22" s="53" t="n"/>
+      <c r="I22" s="106" t="inlineStr">
+        <is>
+          <t>🟥 No estimable: está redactado como una validación pendiente («Validar si se debe publicar eventos antes de generar la solicitud oficial»). El dibujo del MVP sí exige un evento por cada cambio de estado; falta decidir si se emite antes o después de la creación en el core.</t>
+        </is>
+      </c>
       <c r="L22" s="58" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
@@ -2235,40 +2305,44 @@
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="53" t="inlineStr">
+      <c r="A23" s="105" t="inlineStr">
         <is>
           <t>RF-019</t>
         </is>
       </c>
-      <c r="B23" s="53" t="inlineStr">
+      <c r="B23" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C23" s="53" t="inlineStr">
+      <c r="C23" s="105" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D23" s="53" t="inlineStr">
+      <c r="D23" s="105" t="inlineStr">
         <is>
           <t>Se debe incorporar como requisito funcional el "rescate de la solicitud" cuando la radicación no se concluye, sin importar en qué paso quedó.</t>
         </is>
       </c>
       <c r="E23" s="54" t="n"/>
-      <c r="F23" s="53">
+      <c r="F23" s="105">
         <f>IF($E23="",0,INDEX($M$5:$M$8,MATCH($E23,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G23" s="53">
+      <c r="G23" s="105">
         <f>IF($F23=0,0,$F23/10)</f>
         <v/>
       </c>
-      <c r="H23" s="53">
+      <c r="H23" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C23,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I23" s="53" t="n"/>
+      <c r="I23" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el rescate de la radicación incompleta no aparece en el dibujo.</t>
+        </is>
+      </c>
       <c r="L23" s="60" t="inlineStr">
         <is>
           <t>Siniestro Integral</t>
@@ -2437,22 +2511,22 @@
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="57" t="inlineStr">
+      <c r="A26" s="105" t="inlineStr">
         <is>
           <t>RF-022</t>
         </is>
       </c>
-      <c r="B26" s="57" t="inlineStr">
+      <c r="B26" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C26" s="57" t="inlineStr">
+      <c r="C26" s="105" t="inlineStr">
         <is>
           <t>Gestor de Evaluación</t>
         </is>
       </c>
-      <c r="D26" s="57" t="inlineStr">
+      <c r="D26" s="105" t="inlineStr">
         <is>
           <t>Revisar la integración para consultar mora (ir directamente al core de PDN o pasar por SuraHis).</t>
         </is>
@@ -2462,19 +2536,23 @@
           <t>S</t>
         </is>
       </c>
-      <c r="F26" s="53">
+      <c r="F26" s="105">
         <f>IF($E26="",0,INDEX($M$5:$M$8,MATCH($E26,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G26" s="53">
+      <c r="G26" s="105">
         <f>IF($F26=0,0,$F26/10)</f>
         <v/>
       </c>
-      <c r="H26" s="53">
+      <c r="H26" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C26,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I26" s="53" t="n"/>
+      <c r="I26" s="105" t="inlineStr">
+        <is>
+          <t>El dibujo lo resuelve: el dato se pide primero a SuraHis y la conexión directa solo se justifica si el core no lo tiene. La talla cubre el ajuste de la integración, no la decisión.</t>
+        </is>
+      </c>
       <c r="L26" s="62" t="inlineStr">
         <is>
           <t>AVA (Asesores — AVA)</t>
@@ -2827,6 +2905,11 @@
         <v/>
       </c>
       <c r="I32" s="53" t="n"/>
+      <c r="L32" s="108" t="inlineStr">
+        <is>
+          <t>Leyenda de esta revisión (Tech and Solve)</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="53" t="inlineStr">
@@ -2867,294 +2950,386 @@
         <v/>
       </c>
       <c r="I33" s="53" t="n"/>
+      <c r="L33" s="109" t="inlineStr">
+        <is>
+          <t>Fila adicionada</t>
+        </is>
+      </c>
+      <c r="M33" s="110" t="inlineStr">
+        <is>
+          <t>Requisito funcional nuevo (RF-109 a RF-129): elementos que el dibujo del MVP y la vista de tecnología exigen y que la hoja no tenía.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="57" t="inlineStr">
+      <c r="A34" s="105" t="inlineStr">
         <is>
           <t>RF-030</t>
         </is>
       </c>
-      <c r="B34" s="57" t="inlineStr">
+      <c r="B34" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C34" s="57" t="inlineStr">
+      <c r="C34" s="105" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
-      <c r="D34" s="57" t="inlineStr">
+      <c r="D34" s="105" t="inlineStr">
         <is>
           <t>La asignación al equipo se distribuye según reglas de criticidad (marcas en salud, PEP, edad del asegurado, urgencia, quejas/tutelas, diagnósticos de riesgo) entre evaluadores disponibles por nivel.</t>
         </is>
       </c>
       <c r="E34" s="54" t="n"/>
-      <c r="F34" s="53">
+      <c r="F34" s="105">
         <f>IF($E34="",0,INDEX($M$5:$M$8,MATCH($E34,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G34" s="53">
+      <c r="G34" s="105">
         <f>IF($F34=0,0,$F34/10)</f>
         <v/>
       </c>
-      <c r="H34" s="53">
+      <c r="H34" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C34,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I34" s="53" t="n"/>
+      <c r="I34" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye un Gestor de Asignación. La escalada a evaluación humana entra a la bandeja del core.</t>
+        </is>
+      </c>
+      <c r="L34" s="111" t="inlineStr">
+        <is>
+          <t>Fila modificada</t>
+        </is>
+      </c>
+      <c r="M34" s="110" t="inlineStr">
+        <is>
+          <t>Fila existente a la que se le agregó una observación: entra al MVP con una salvedad, o queda fuera y se explica por qué.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="53" t="inlineStr">
+      <c r="A35" s="105" t="inlineStr">
         <is>
           <t>RF-031</t>
         </is>
       </c>
-      <c r="B35" s="53" t="inlineStr">
+      <c r="B35" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C35" s="53" t="inlineStr">
+      <c r="C35" s="105" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
-      <c r="D35" s="53" t="inlineStr">
+      <c r="D35" s="105" t="inlineStr">
         <is>
           <t>Para solicitudes pendientes por gestión se habilita la reasignación entre niveles.</t>
         </is>
       </c>
       <c r="E35" s="54" t="n"/>
-      <c r="F35" s="53">
+      <c r="F35" s="105">
         <f>IF($E35="",0,INDEX($M$5:$M$8,MATCH($E35,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G35" s="53">
+      <c r="G35" s="105">
         <f>IF($F35=0,0,$F35/10)</f>
         <v/>
       </c>
-      <c r="H35" s="53">
+      <c r="H35" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C35,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I35" s="53" t="n"/>
+      <c r="I35" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye un Gestor de Asignación. La escalada a evaluación humana entra a la bandeja del core.</t>
+        </is>
+      </c>
+      <c r="L35" s="112" t="inlineStr">
+        <is>
+          <t>Alerta · sin tallar</t>
+        </is>
+      </c>
+      <c r="M35" s="110" t="inlineStr">
+        <is>
+          <t>Requisito que no se pudo estimar. La duda concreta queda escrita en Observaciones.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="57" t="inlineStr">
+      <c r="A36" s="105" t="inlineStr">
         <is>
           <t>RF-032</t>
         </is>
       </c>
-      <c r="B36" s="57" t="inlineStr">
+      <c r="B36" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C36" s="57" t="inlineStr">
+      <c r="C36" s="105" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
-      <c r="D36" s="57" t="inlineStr">
+      <c r="D36" s="105" t="inlineStr">
         <is>
           <t>Cada solicitud debe tener un tiempo de respuesta asignado (100% de las solicitudes en menos de 24 horas).</t>
         </is>
       </c>
       <c r="E36" s="54" t="n"/>
-      <c r="F36" s="53">
+      <c r="F36" s="105">
         <f>IF($E36="",0,INDEX($M$5:$M$8,MATCH($E36,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G36" s="53">
+      <c r="G36" s="105">
         <f>IF($F36=0,0,$F36/10)</f>
         <v/>
       </c>
-      <c r="H36" s="53">
+      <c r="H36" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C36,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I36" s="53" t="n"/>
+      <c r="I36" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye un Gestor de Asignación. La escalada a evaluación humana entra a la bandeja del core.</t>
+        </is>
+      </c>
+      <c r="L36" s="113" t="inlineStr">
+        <is>
+          <t>Talla diligenciada</t>
+        </is>
+      </c>
+      <c r="M36" s="110" t="inlineStr">
+        <is>
+          <t>Fila sin color con valor en Talla: requisito del MVP estimado sin salvedades.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="53" t="inlineStr">
+      <c r="A37" s="105" t="inlineStr">
         <is>
           <t>RF-033</t>
         </is>
       </c>
-      <c r="B37" s="53" t="inlineStr">
+      <c r="B37" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C37" s="53" t="inlineStr">
+      <c r="C37" s="105" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
-      <c r="D37" s="53" t="inlineStr">
+      <c r="D37" s="105" t="inlineStr">
         <is>
           <t>Se debe notificar al asegurado cuando se identifique en el proceso de evaluación manual que se requiere un documento adicional para entregar una decisión en la evaluación, esta notificación debe incluir el enlace de la SVP o APP para que el asegurado cargue el requisito pendiente</t>
         </is>
       </c>
       <c r="E37" s="54" t="n"/>
-      <c r="F37" s="53">
+      <c r="F37" s="105">
         <f>IF($E37="",0,INDEX($M$5:$M$8,MATCH($E37,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G37" s="53">
+      <c r="G37" s="105">
         <f>IF($F37=0,0,$F37/10)</f>
         <v/>
       </c>
-      <c r="H37" s="53">
+      <c r="H37" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C37,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I37" s="53" t="n"/>
+      <c r="I37" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye un Gestor de Asignación. La escalada a evaluación humana entra a la bandeja del core.</t>
+        </is>
+      </c>
+      <c r="L37" s="114" t="inlineStr">
+        <is>
+          <t>Sin color y sin talla</t>
+        </is>
+      </c>
+      <c r="M37" s="110" t="inlineStr">
+        <is>
+          <t>Requisito fuera del MVP en una épica que esta misma hoja ya marca «No» o «N/A».</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="57" t="inlineStr">
+      <c r="A38" s="105" t="inlineStr">
         <is>
           <t>RF-034</t>
         </is>
       </c>
-      <c r="B38" s="57" t="inlineStr">
+      <c r="B38" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C38" s="57" t="inlineStr">
+      <c r="C38" s="105" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
-      <c r="D38" s="57" t="inlineStr">
+      <c r="D38" s="105" t="inlineStr">
         <is>
           <t>Cuando el asegurado cargue el requisito pendiente, esta solicitud se debe encolar nuevamente en la bandeja manual en surahis y se debe asignar al mismo evaluador y con un tiempo de respuesta prioritario</t>
         </is>
       </c>
       <c r="E38" s="54" t="n"/>
-      <c r="F38" s="53">
+      <c r="F38" s="105">
         <f>IF($E38="",0,INDEX($M$5:$M$8,MATCH($E38,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G38" s="53">
+      <c r="G38" s="105">
         <f>IF($F38=0,0,$F38/10)</f>
         <v/>
       </c>
-      <c r="H38" s="53">
+      <c r="H38" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C38,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I38" s="53" t="n"/>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="53" t="inlineStr">
+      <c r="I38" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye un Gestor de Asignación. La escalada a evaluación humana entra a la bandeja del core.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="60" customHeight="1">
+      <c r="A39" s="105" t="inlineStr">
         <is>
           <t>RF-035</t>
         </is>
       </c>
-      <c r="B39" s="53" t="inlineStr">
+      <c r="B39" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C39" s="53" t="inlineStr">
+      <c r="C39" s="105" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
-      <c r="D39" s="53" t="inlineStr">
+      <c r="D39" s="105" t="inlineStr">
         <is>
           <t>Con la negación de un servicio se debe activar la radicación automática de la solicitud de integralidad a EPS Sura en el aplicativo salud web</t>
         </is>
       </c>
       <c r="E39" s="54" t="n"/>
-      <c r="F39" s="53">
+      <c r="F39" s="105">
         <f>IF($E39="",0,INDEX($M$5:$M$8,MATCH($E39,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G39" s="53">
+      <c r="G39" s="105">
         <f>IF($F39=0,0,$F39/10)</f>
         <v/>
       </c>
-      <c r="H39" s="53">
+      <c r="H39" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C39,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I39" s="53" t="n"/>
+      <c r="I39" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye un Gestor de Asignación. La escalada a evaluación humana entra a la bandeja del core.</t>
+        </is>
+      </c>
+      <c r="L39" s="114" t="inlineStr">
+        <is>
+          <t>Criterio de alcance</t>
+        </is>
+      </c>
+      <c r="M39" s="110" t="inlineStr">
+        <is>
+          <t>La pertenencia al MVP se decidió requisito por requisito contra «resumen-arquitectura-gestores — Arquitectura MVP» y «arquitectura-tecnologia», no contra la columna «¿En MVP?», que se deriva por épica y por eso marca «Sí» a épicas donde solo una parte entra. Entran Solicitud, Evaluación, Siniestro Integral, los canales que el MVP habilita, las capas 1 y 2 de la torre, el acceso al dato vía el core y los transversales del ciclo de mejora y del plano de control. Suma: 500 días hábiles con la escala de la propia hoja.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="57" t="inlineStr">
+      <c r="A40" s="105" t="inlineStr">
         <is>
           <t>RF-036</t>
         </is>
       </c>
-      <c r="B40" s="57" t="inlineStr">
+      <c r="B40" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C40" s="57" t="inlineStr">
+      <c r="C40" s="105" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
-      <c r="D40" s="57" t="inlineStr">
+      <c r="D40" s="105" t="inlineStr">
         <is>
           <t>Surahis publica un evento con el cambio de estado de la solicitud de integralidad en salud web y con este evento se alimenta la torre de control y se actualiza el estado en los canales (Front)</t>
         </is>
       </c>
       <c r="E40" s="54" t="n"/>
-      <c r="F40" s="53">
+      <c r="F40" s="105">
         <f>IF($E40="",0,INDEX($M$5:$M$8,MATCH($E40,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G40" s="53">
+      <c r="G40" s="105">
         <f>IF($F40=0,0,$F40/10)</f>
         <v/>
       </c>
-      <c r="H40" s="53">
+      <c r="H40" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C40,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I40" s="53" t="n"/>
+      <c r="I40" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye un Gestor de Asignación. La escalada a evaluación humana entra a la bandeja del core.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="53" t="inlineStr">
+      <c r="A41" s="105" t="inlineStr">
         <is>
           <t>RF-037</t>
         </is>
       </c>
-      <c r="B41" s="53" t="inlineStr">
+      <c r="B41" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C41" s="53" t="inlineStr">
+      <c r="C41" s="105" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
-      <c r="D41" s="53" t="inlineStr">
+      <c r="D41" s="105" t="inlineStr">
         <is>
           <t>Se debe habilitar la opción de resignación manual de solicitudes a otro evaluador (novedades con el evaluador asignado inicialmente).</t>
         </is>
       </c>
       <c r="E41" s="54" t="n"/>
-      <c r="F41" s="53">
+      <c r="F41" s="105">
         <f>IF($E41="",0,INDEX($M$5:$M$8,MATCH($E41,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G41" s="53">
+      <c r="G41" s="105">
         <f>IF($F41=0,0,$F41/10)</f>
         <v/>
       </c>
-      <c r="H41" s="53">
+      <c r="H41" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C41,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I41" s="53" t="n"/>
+      <c r="I41" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye un Gestor de Asignación. La escalada a evaluación humana entra a la bandeja del core.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="57" t="inlineStr">
@@ -3563,40 +3738,44 @@
       <c r="I52" s="53" t="n"/>
     </row>
     <row r="53" ht="30" customHeight="1">
-      <c r="A53" s="53" t="inlineStr">
+      <c r="A53" s="105" t="inlineStr">
         <is>
           <t>RF-049</t>
         </is>
       </c>
-      <c r="B53" s="53" t="inlineStr">
+      <c r="B53" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C53" s="53" t="inlineStr">
+      <c r="C53" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D53" s="53" t="inlineStr">
+      <c r="D53" s="105" t="inlineStr">
         <is>
           <t>Monitorea el ciclo de vida completo de la solicitud: cumplimiento de SLA/ANS (semaforos que indiquen posible incumplimiento), carga de trabajo, trazabilidad,capacidad y riesgo acumulado del ciclo.</t>
         </is>
       </c>
       <c r="E53" s="54" t="n"/>
-      <c r="F53" s="53">
+      <c r="F53" s="105">
         <f>IF($E53="",0,INDEX($M$5:$M$8,MATCH($E53,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G53" s="53">
+      <c r="G53" s="105">
         <f>IF($F53=0,0,$F53/10)</f>
         <v/>
       </c>
-      <c r="H53" s="53">
+      <c r="H53" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C53,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I53" s="53" t="n"/>
+      <c r="I53" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="57" t="inlineStr">
@@ -3639,130 +3818,142 @@
       <c r="I54" s="53" t="n"/>
     </row>
     <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="53" t="inlineStr">
+      <c r="A55" s="105" t="inlineStr">
         <is>
           <t>RF-051</t>
         </is>
       </c>
-      <c r="B55" s="53" t="inlineStr">
+      <c r="B55" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C55" s="53" t="inlineStr">
+      <c r="C55" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D55" s="53" t="inlineStr">
+      <c r="D55" s="105" t="inlineStr">
         <is>
           <t>Capacidades proactivas (contactar directamente al cliente/prestador/asesor) emite notificaciones en 3 dimensiones (actor, canal, proactivo/pasivo), ejemplo: asegurado ante el incumplimiento de un SLA para dar tranquilidad de la gestión de la solicitud y alerta internamente a evaluadores/líderes por casos por vencer o desborde de capacidad, apertura de autorización, autorización en evaluación, autorización aprobada, etc.</t>
         </is>
       </c>
       <c r="E55" s="54" t="n"/>
-      <c r="F55" s="53">
+      <c r="F55" s="105">
         <f>IF($E55="",0,INDEX($M$5:$M$8,MATCH($E55,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G55" s="53">
+      <c r="G55" s="105">
         <f>IF($F55=0,0,$F55/10)</f>
         <v/>
       </c>
-      <c r="H55" s="53">
+      <c r="H55" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C55,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I55" s="53" t="n"/>
+      <c r="I55" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="30" customHeight="1">
-      <c r="A56" s="57" t="inlineStr">
+      <c r="A56" s="105" t="inlineStr">
         <is>
           <t>RF-052</t>
         </is>
       </c>
-      <c r="B56" s="57" t="inlineStr">
+      <c r="B56" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C56" s="57" t="inlineStr">
+      <c r="C56" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D56" s="57" t="inlineStr">
+      <c r="D56" s="105" t="inlineStr">
         <is>
           <t>Capacidad de intervenir otros gestores cuando se detecte algún comportamiento insual en la solicitud</t>
         </is>
       </c>
       <c r="E56" s="54" t="n"/>
-      <c r="F56" s="53">
+      <c r="F56" s="105">
         <f>IF($E56="",0,INDEX($M$5:$M$8,MATCH($E56,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G56" s="53">
+      <c r="G56" s="105">
         <f>IF($F56=0,0,$F56/10)</f>
         <v/>
       </c>
-      <c r="H56" s="53">
+      <c r="H56" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C56,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I56" s="53" t="n"/>
+      <c r="I56" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="53" t="inlineStr">
+      <c r="A57" s="105" t="inlineStr">
         <is>
           <t>RF-053</t>
         </is>
       </c>
-      <c r="B57" s="53" t="inlineStr">
+      <c r="B57" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C57" s="53" t="inlineStr">
+      <c r="C57" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D57" s="53" t="inlineStr">
+      <c r="D57" s="105" t="inlineStr">
         <is>
           <t>Indicador en la torre de control para visualización de los siniestros duplicados ingresados por el prestador que sean para el mismo</t>
         </is>
       </c>
       <c r="E57" s="54" t="n"/>
-      <c r="F57" s="53">
+      <c r="F57" s="105">
         <f>IF($E57="",0,INDEX($M$5:$M$8,MATCH($E57,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G57" s="53">
+      <c r="G57" s="105">
         <f>IF($F57=0,0,$F57/10)</f>
         <v/>
       </c>
-      <c r="H57" s="53">
+      <c r="H57" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C57,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I57" s="53" t="n"/>
+      <c r="I57" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="30" customHeight="1">
-      <c r="A58" s="57" t="inlineStr">
+      <c r="A58" s="105" t="inlineStr">
         <is>
           <t>RF-054</t>
         </is>
       </c>
-      <c r="B58" s="57" t="inlineStr">
+      <c r="B58" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C58" s="57" t="inlineStr">
+      <c r="C58" s="105" t="inlineStr">
         <is>
           <t>Gestor de Evaluación</t>
         </is>
       </c>
-      <c r="D58" s="57" t="inlineStr">
+      <c r="D58" s="105" t="inlineStr">
         <is>
           <t>Detecta solicitudes repetidas (2 o más veces) con las mismas características y activa el mismo flujo de rescate con mensaje diferenciado, notificando al asegurado y al gestor de solicitud para bloquear la radicación de una nueva solicitud</t>
         </is>
@@ -3772,91 +3963,103 @@
           <t>M</t>
         </is>
       </c>
-      <c r="F58" s="53">
+      <c r="F58" s="105">
         <f>IF($E58="",0,INDEX($M$5:$M$8,MATCH($E58,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G58" s="53">
+      <c r="G58" s="105">
         <f>IF($F58=0,0,$F58/10)</f>
         <v/>
       </c>
-      <c r="H58" s="53">
+      <c r="H58" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C58,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I58" s="53" t="n"/>
+      <c r="I58" s="105" t="inlineStr">
+        <is>
+          <t>Entra la detección de solicitudes repetidas, que el dibujo resuelve en la capa de duplicidad. La notificación al asegurado depende de la capa de exposición de la torre, que no está en el MVP.</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="30" customHeight="1">
-      <c r="A59" s="53" t="inlineStr">
+      <c r="A59" s="105" t="inlineStr">
         <is>
           <t>RF-055</t>
         </is>
       </c>
-      <c r="B59" s="53" t="inlineStr">
+      <c r="B59" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C59" s="53" t="inlineStr">
+      <c r="C59" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D59" s="53" t="inlineStr">
+      <c r="D59" s="105" t="inlineStr">
         <is>
           <t>Expone información distinta según el actor consultante (prestador, cliente, asesor), enmascarando datos sensibles.</t>
         </is>
       </c>
       <c r="E59" s="54" t="n"/>
-      <c r="F59" s="53">
+      <c r="F59" s="105">
         <f>IF($E59="",0,INDEX($M$5:$M$8,MATCH($E59,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G59" s="53">
+      <c r="G59" s="105">
         <f>IF($F59=0,0,$F59/10)</f>
         <v/>
       </c>
-      <c r="H59" s="53">
+      <c r="H59" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C59,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I59" s="53" t="n"/>
+      <c r="I59" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="30" customHeight="1">
-      <c r="A60" s="57" t="inlineStr">
+      <c r="A60" s="105" t="inlineStr">
         <is>
           <t>RF-056</t>
         </is>
       </c>
-      <c r="B60" s="57" t="inlineStr">
+      <c r="B60" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C60" s="57" t="inlineStr">
+      <c r="C60" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D60" s="57" t="inlineStr">
+      <c r="D60" s="105" t="inlineStr">
         <is>
           <t>Se requiere una vista que nos permita realizar la auditoria de toda la trazabilidad de las solicitudes</t>
         </is>
       </c>
       <c r="E60" s="54" t="n"/>
-      <c r="F60" s="53">
+      <c r="F60" s="105">
         <f>IF($E60="",0,INDEX($M$5:$M$8,MATCH($E60,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G60" s="53">
+      <c r="G60" s="105">
         <f>IF($F60=0,0,$F60/10)</f>
         <v/>
       </c>
-      <c r="H60" s="53">
+      <c r="H60" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C60,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I60" s="53" t="n"/>
+      <c r="I60" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="53" t="inlineStr">
@@ -3899,22 +4102,22 @@
       <c r="I61" s="53" t="n"/>
     </row>
     <row r="62" ht="30" customHeight="1">
-      <c r="A62" s="57" t="inlineStr">
+      <c r="A62" s="105" t="inlineStr">
         <is>
           <t>RF-058</t>
         </is>
       </c>
-      <c r="B62" s="57" t="inlineStr">
+      <c r="B62" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C62" s="57" t="inlineStr">
+      <c r="C62" s="105" t="inlineStr">
         <is>
           <t>Canales / Front Externos</t>
         </is>
       </c>
-      <c r="D62" s="57" t="inlineStr">
+      <c r="D62" s="105" t="inlineStr">
         <is>
           <t>La selección de prestador no es necesaria en la solicitud inicial, se debe sugerir el prestador cuando se tenga idetificado el servicio que solicita.</t>
         </is>
@@ -3924,235 +4127,263 @@
           <t>S</t>
         </is>
       </c>
-      <c r="F62" s="53">
+      <c r="F62" s="105">
         <f>IF($E62="",0,INDEX($M$5:$M$8,MATCH($E62,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G62" s="53">
+      <c r="G62" s="105">
         <f>IF($F62=0,0,$F62/10)</f>
         <v/>
       </c>
-      <c r="H62" s="53">
+      <c r="H62" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C62,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I62" s="53" t="n"/>
+      <c r="I62" s="105" t="inlineStr">
+        <is>
+          <t>Entra la parte del front: no exigir la selección de prestador en la solicitud inicial. Sugerir el prestador es del Gestor de Coordinación, que queda fuera del MVP.</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="30" customHeight="1">
-      <c r="A63" s="53" t="inlineStr">
+      <c r="A63" s="105" t="inlineStr">
         <is>
           <t>RF-059</t>
         </is>
       </c>
-      <c r="B63" s="53" t="inlineStr">
+      <c r="B63" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C63" s="53" t="inlineStr">
+      <c r="C63" s="105" t="inlineStr">
         <is>
           <t>Canales / Front Externos</t>
         </is>
       </c>
-      <c r="D63" s="53" t="inlineStr">
+      <c r="D63" s="105" t="inlineStr">
         <is>
           <t>El cliente debe recibir notificación automática cuando un prestador radica una solicitud en su nombre, con visibilidad completa del caso sin importar el canal de radicación (evita duplicados).</t>
         </is>
       </c>
       <c r="E63" s="54" t="n"/>
-      <c r="F63" s="53">
+      <c r="F63" s="105">
         <f>IF($E63="",0,INDEX($M$5:$M$8,MATCH($E63,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G63" s="53">
+      <c r="G63" s="105">
         <f>IF($F63=0,0,$F63/10)</f>
         <v/>
       </c>
-      <c r="H63" s="53">
+      <c r="H63" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C63,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I63" s="53" t="n"/>
+      <c r="I63" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: la notificación automática al cliente es capa de exposición de la torre, que no entra.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="30" customHeight="1">
-      <c r="A64" s="57" t="inlineStr">
+      <c r="A64" s="105" t="inlineStr">
         <is>
           <t>RF-060</t>
         </is>
       </c>
-      <c r="B64" s="57" t="inlineStr">
+      <c r="B64" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C64" s="57" t="inlineStr">
+      <c r="C64" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D64" s="57" t="inlineStr">
+      <c r="D64" s="105" t="inlineStr">
         <is>
           <t>El Gestor de Prestación no requiere capacidad agéntica para la confirmación de atención; la integración se conecta directo entre Super App/interoperabilidad y el Core (SuraHis), sin crear un componente nuevo en Gestores.</t>
         </is>
       </c>
       <c r="E64" s="54" t="n"/>
-      <c r="F64" s="53">
+      <c r="F64" s="105">
         <f>IF($E64="",0,INDEX($M$5:$M$8,MATCH($E64,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G64" s="53">
+      <c r="G64" s="105">
         <f>IF($F64=0,0,$F64/10)</f>
         <v/>
       </c>
-      <c r="H64" s="53">
+      <c r="H64" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C64,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I64" s="53" t="n"/>
+      <c r="I64" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="30" customHeight="1">
-      <c r="A65" s="53" t="inlineStr">
+      <c r="A65" s="105" t="inlineStr">
         <is>
           <t>RF-061</t>
         </is>
       </c>
-      <c r="B65" s="53" t="inlineStr">
+      <c r="B65" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C65" s="53" t="inlineStr">
+      <c r="C65" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D65" s="53" t="inlineStr">
+      <c r="D65" s="105" t="inlineStr">
         <is>
           <t>La interoperabilidad administrativa de autorizaciones está en construcción por el equipo de Interoperabilidad (Sergio "Checho" Pérez) junto con el equipo de autorizaciones y pólizas; no alcanza a cerrarse antes del cierre de estructuración.</t>
         </is>
       </c>
       <c r="E65" s="54" t="n"/>
-      <c r="F65" s="53">
+      <c r="F65" s="105">
         <f>IF($E65="",0,INDEX($M$5:$M$8,MATCH($E65,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G65" s="53">
+      <c r="G65" s="105">
         <f>IF($F65=0,0,$F65/10)</f>
         <v/>
       </c>
-      <c r="H65" s="53">
+      <c r="H65" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C65,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I65" s="53" t="n"/>
+      <c r="I65" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="30" customHeight="1">
-      <c r="A66" s="57" t="inlineStr">
+      <c r="A66" s="105" t="inlineStr">
         <is>
           <t>RF-062</t>
         </is>
       </c>
-      <c r="B66" s="57" t="inlineStr">
+      <c r="B66" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C66" s="57" t="inlineStr">
+      <c r="C66" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D66" s="57" t="inlineStr">
+      <c r="D66" s="105" t="inlineStr">
         <is>
           <t>Hoy existen ~12 software de interoperabilidad habilitados con prestadores (incluye Himed/proveedor Pareto, Salud Tools, Servintech), con datos de institución/médico tratante, fecha y tipo/motivo de consulta.</t>
         </is>
       </c>
       <c r="E66" s="54" t="n"/>
-      <c r="F66" s="53">
+      <c r="F66" s="105">
         <f>IF($E66="",0,INDEX($M$5:$M$8,MATCH($E66,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G66" s="53">
+      <c r="G66" s="105">
         <f>IF($F66=0,0,$F66/10)</f>
         <v/>
       </c>
-      <c r="H66" s="53">
+      <c r="H66" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C66,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I66" s="53" t="n"/>
+      <c r="I66" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="30" customHeight="1">
-      <c r="A67" s="53" t="inlineStr">
+      <c r="A67" s="105" t="inlineStr">
         <is>
           <t>RF-063</t>
         </is>
       </c>
-      <c r="B67" s="53" t="inlineStr">
+      <c r="B67" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C67" s="53" t="inlineStr">
+      <c r="C67" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D67" s="53" t="inlineStr">
+      <c r="D67" s="105" t="inlineStr">
         <is>
           <t>No debe agendarse ninguna cita de forma automática sin el consentimiento explícito del asegurado (el sistema sugiere las citas disponibles y confirma con el asegurado antes de agendar).</t>
         </is>
       </c>
       <c r="E67" s="54" t="n"/>
-      <c r="F67" s="53">
+      <c r="F67" s="105">
         <f>IF($E67="",0,INDEX($M$5:$M$8,MATCH($E67,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G67" s="53">
+      <c r="G67" s="105">
         <f>IF($F67=0,0,$F67/10)</f>
         <v/>
       </c>
-      <c r="H67" s="53">
+      <c r="H67" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C67,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I67" s="53" t="n"/>
+      <c r="I67" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="30" customHeight="1">
-      <c r="A68" s="57" t="inlineStr">
+      <c r="A68" s="105" t="inlineStr">
         <is>
           <t>RF-064</t>
         </is>
       </c>
-      <c r="B68" s="57" t="inlineStr">
+      <c r="B68" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C68" s="57" t="inlineStr">
+      <c r="C68" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D68" s="57" t="inlineStr">
+      <c r="D68" s="105" t="inlineStr">
         <is>
           <t>¿Cómo se cierra la brecha de confirmación de atención para prestación externa (~60-70% de la población)? SuraHis resolvería el gap interno, pero no está claro que resuelva el externo.</t>
         </is>
       </c>
       <c r="E68" s="54" t="n"/>
-      <c r="F68" s="53">
+      <c r="F68" s="105">
         <f>IF($E68="",0,INDEX($M$5:$M$8,MATCH($E68,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G68" s="53">
+      <c r="G68" s="105">
         <f>IF($F68=0,0,$F68/10)</f>
         <v/>
       </c>
-      <c r="H68" s="53">
+      <c r="H68" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C68,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I68" s="53" t="n"/>
+      <c r="I68" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="53" t="inlineStr">
@@ -4335,22 +4566,22 @@
       <c r="I73" s="53" t="n"/>
     </row>
     <row r="74" ht="30" customHeight="1">
-      <c r="A74" s="57" t="inlineStr">
+      <c r="A74" s="105" t="inlineStr">
         <is>
           <t>RF-070</t>
         </is>
       </c>
-      <c r="B74" s="57" t="inlineStr">
+      <c r="B74" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C74" s="57" t="inlineStr">
+      <c r="C74" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D74" s="57" t="inlineStr">
+      <c r="D74" s="105" t="inlineStr">
         <is>
           <t>Principio de responsabilidad única: si Gestores necesita un dato o funcionalidad de interoperabilidad, primero debe solicitarlo a través de SuraHIS (el core); una conexión directa de Gestores a Interoperabilidad solo se justifica cuando SuraHIS no tiene o no va a tener ese dato.</t>
         </is>
@@ -4360,163 +4591,183 @@
           <t>S</t>
         </is>
       </c>
-      <c r="F74" s="53">
+      <c r="F74" s="105">
         <f>IF($E74="",0,INDEX($M$5:$M$8,MATCH($E74,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G74" s="53">
+      <c r="G74" s="105">
         <f>IF($F74=0,0,$F74/10)</f>
         <v/>
       </c>
-      <c r="H74" s="53">
+      <c r="H74" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C74,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I74" s="53" t="n"/>
+      <c r="I74" s="105" t="inlineStr">
+        <is>
+          <t>Entra el principio de acceso al dato vía el core, que el dibujo del MVP recoge explícitamente. La interoperabilidad de autorizaciones como tal queda fuera.</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="30" customHeight="1">
-      <c r="A75" s="53" t="inlineStr">
+      <c r="A75" s="105" t="inlineStr">
         <is>
           <t>RF-071</t>
         </is>
       </c>
-      <c r="B75" s="53" t="inlineStr">
+      <c r="B75" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C75" s="53" t="inlineStr">
+      <c r="C75" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D75" s="53" t="inlineStr">
+      <c r="D75" s="105" t="inlineStr">
         <is>
           <t>Se definen 5 momentos de integración con Interoperabilidad: (1) solicitud/consulta de historia clínica, (2) envío de la autorización al prestador, (3) confirmación de la atención/prestación, (4) recepción de nuevas órdenes o autorizaciones que surjan durante la atención (ej. exámenes adicionales), (5) agenda disponible en el prestador para atención de un servicio</t>
         </is>
       </c>
       <c r="E75" s="54" t="n"/>
-      <c r="F75" s="53">
+      <c r="F75" s="105">
         <f>IF($E75="",0,INDEX($M$5:$M$8,MATCH($E75,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G75" s="53">
+      <c r="G75" s="105">
         <f>IF($F75=0,0,$F75/10)</f>
         <v/>
       </c>
-      <c r="H75" s="53">
+      <c r="H75" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C75,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I75" s="53" t="n"/>
+      <c r="I75" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="30" customHeight="1">
-      <c r="A76" s="57" t="inlineStr">
+      <c r="A76" s="105" t="inlineStr">
         <is>
           <t>RF-072</t>
         </is>
       </c>
-      <c r="B76" s="57" t="inlineStr">
+      <c r="B76" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C76" s="57" t="inlineStr">
+      <c r="C76" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D76" s="57" t="inlineStr">
+      <c r="D76" s="105" t="inlineStr">
         <is>
           <t>El estándar de referencia para el intercambio de información clínica es el RDA (Resumen Digital de Atención), alineado con FHIR/HL7 y con la normativa colombiana vigente.</t>
         </is>
       </c>
       <c r="E76" s="54" t="n"/>
-      <c r="F76" s="53">
+      <c r="F76" s="105">
         <f>IF($E76="",0,INDEX($M$5:$M$8,MATCH($E76,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G76" s="53">
+      <c r="G76" s="105">
         <f>IF($F76=0,0,$F76/10)</f>
         <v/>
       </c>
-      <c r="H76" s="53">
+      <c r="H76" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C76,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I76" s="53" t="n"/>
+      <c r="I76" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="30" customHeight="1">
-      <c r="A77" s="53" t="inlineStr">
+      <c r="A77" s="105" t="inlineStr">
         <is>
           <t>RF-073</t>
         </is>
       </c>
-      <c r="B77" s="53" t="inlineStr">
+      <c r="B77" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C77" s="53" t="inlineStr">
+      <c r="C77" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D77" s="53" t="inlineStr">
+      <c r="D77" s="105" t="inlineStr">
         <is>
           <t>Se solicitará al equipo de Interoperabilidad que su primer entregable/release sean los contratos de API (aunque la solución completa no esté lista), para que Gestores pueda construir e integrar desde ya contra un contrato estable.</t>
         </is>
       </c>
       <c r="E77" s="54" t="n"/>
-      <c r="F77" s="53">
+      <c r="F77" s="105">
         <f>IF($E77="",0,INDEX($M$5:$M$8,MATCH($E77,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G77" s="53">
+      <c r="G77" s="105">
         <f>IF($F77=0,0,$F77/10)</f>
         <v/>
       </c>
-      <c r="H77" s="53">
+      <c r="H77" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C77,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I77" s="53" t="n"/>
+      <c r="I77" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="30" customHeight="1">
-      <c r="A78" s="57" t="inlineStr">
+      <c r="A78" s="105" t="inlineStr">
         <is>
           <t>RF-074</t>
         </is>
       </c>
-      <c r="B78" s="57" t="inlineStr">
+      <c r="B78" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C78" s="57" t="inlineStr">
+      <c r="C78" s="105" t="inlineStr">
         <is>
           <t>Canales / Front Externos</t>
         </is>
       </c>
-      <c r="D78" s="57" t="inlineStr">
+      <c r="D78" s="105" t="inlineStr">
         <is>
           <t>La SVP (y en general los canales de cliente) deben permitir editar/cambiar el prestador asignado en la autorización, dentro de un tiempo máximo definido; superado ese tiempo, se confirma automáticamente el prestador por defecto.</t>
         </is>
       </c>
       <c r="E78" s="54" t="n"/>
-      <c r="F78" s="53">
+      <c r="F78" s="105">
         <f>IF($E78="",0,INDEX($M$5:$M$8,MATCH($E78,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G78" s="53">
+      <c r="G78" s="105">
         <f>IF($F78=0,0,$F78/10)</f>
         <v/>
       </c>
-      <c r="H78" s="53">
+      <c r="H78" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C78,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I78" s="53" t="n"/>
+      <c r="I78" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: editar el prestador asignado depende del Gestor de Coordinación, que queda fuera.</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="30" customHeight="1">
       <c r="A79" s="53" t="inlineStr">
@@ -4555,364 +4806,404 @@
       <c r="I79" s="53" t="n"/>
     </row>
     <row r="80" ht="30" customHeight="1">
-      <c r="A80" s="57" t="inlineStr">
+      <c r="A80" s="105" t="inlineStr">
         <is>
           <t>RF-076</t>
         </is>
       </c>
-      <c r="B80" s="57" t="inlineStr">
+      <c r="B80" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C80" s="57" t="inlineStr">
+      <c r="C80" s="105" t="inlineStr">
         <is>
           <t>Transversal</t>
         </is>
       </c>
-      <c r="D80" s="57" t="inlineStr">
+      <c r="D80" s="105" t="inlineStr">
         <is>
           <t>si la libre elección de prestador aplica solo a pólizas Salud Global o a todo el portafolio (excepto modular). Es "muy importante" porque si cambia, impacta todo el portafolio.</t>
         </is>
       </c>
       <c r="E80" s="54" t="n"/>
-      <c r="F80" s="53">
+      <c r="F80" s="105">
         <f>IF($E80="",0,INDEX($M$5:$M$8,MATCH($E80,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G80" s="53">
+      <c r="G80" s="105">
         <f>IF($F80=0,0,$F80/10)</f>
         <v/>
       </c>
-      <c r="H80" s="53">
+      <c r="H80" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C80,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I80" s="53" t="n"/>
+      <c r="I80" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: la libre elección de prestador es del Gestor de Coordinación, que queda fuera.</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="30" customHeight="1">
-      <c r="A81" s="53" t="inlineStr">
+      <c r="A81" s="106" t="inlineStr">
         <is>
           <t>RF-077</t>
         </is>
       </c>
-      <c r="B81" s="53" t="inlineStr">
+      <c r="B81" s="106" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C81" s="53" t="inlineStr">
+      <c r="C81" s="106" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D81" s="53" t="inlineStr">
+      <c r="D81" s="106" t="inlineStr">
         <is>
           <t>reglas de visibilidad en el portal de solicitudes — si el prestador que originó una orden puede ver las solicitudes que quedaron asignadas a otro prestador. Señalada explícitamente como decisión "muy importante" sin dueño claro todavía.</t>
         </is>
       </c>
-      <c r="E81" s="54" t="n"/>
-      <c r="F81" s="53">
+      <c r="E81" s="107" t="n"/>
+      <c r="F81" s="106">
         <f>IF($E81="",0,INDEX($M$5:$M$8,MATCH($E81,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G81" s="53">
+      <c r="G81" s="106">
         <f>IF($F81=0,0,$F81/10)</f>
         <v/>
       </c>
-      <c r="H81" s="53">
+      <c r="H81" s="106">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C81,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I81" s="53" t="n"/>
+      <c r="I81" s="106" t="inlineStr">
+        <is>
+          <t>🟥 No estimable: las reglas de visibilidad entre prestadores están señaladas en la propia hoja como decisión importante sin dueño. Definir la regla antes de tallar.</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="30" customHeight="1">
-      <c r="A82" s="57" t="inlineStr">
+      <c r="A82" s="105" t="inlineStr">
         <is>
           <t>RF-078</t>
         </is>
       </c>
-      <c r="B82" s="57" t="inlineStr">
+      <c r="B82" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C82" s="57" t="inlineStr">
+      <c r="C82" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D82" s="57" t="inlineStr">
+      <c r="D82" s="105" t="inlineStr">
         <is>
           <t>falta decidir el modelo operativo único entre 3 opciones (vía interoperabilidad cuando esté lista, que el prestador que generó la orden asuma el costo operativo, o que se le entregue el papeleo al cliente).</t>
         </is>
       </c>
       <c r="E82" s="54" t="n"/>
-      <c r="F82" s="53">
+      <c r="F82" s="105">
         <f>IF($E82="",0,INDEX($M$5:$M$8,MATCH($E82,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G82" s="53">
+      <c r="G82" s="105">
         <f>IF($F82=0,0,$F82/10)</f>
         <v/>
       </c>
-      <c r="H82" s="53">
+      <c r="H82" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C82,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I82" s="53" t="n"/>
+      <c r="I82" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="30" customHeight="1">
-      <c r="A83" s="53" t="inlineStr">
+      <c r="A83" s="105" t="inlineStr">
         <is>
           <t>RF-079</t>
         </is>
       </c>
-      <c r="B83" s="53" t="inlineStr">
+      <c r="B83" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C83" s="53" t="inlineStr">
+      <c r="C83" s="105" t="inlineStr">
         <is>
           <t>Transversal</t>
         </is>
       </c>
-      <c r="D83" s="53" t="inlineStr">
+      <c r="D83" s="105" t="inlineStr">
         <is>
           <t>Definir si se incorpora un paso explícito de aceptación/confirmación del paciente sobre el prestador asignado, y el tiempo máximo para que la SVP permita editar el prestador (incluyendo el costo operativo de ese cambio).</t>
         </is>
       </c>
       <c r="E83" s="54" t="n"/>
-      <c r="F83" s="53">
+      <c r="F83" s="105">
         <f>IF($E83="",0,INDEX($M$5:$M$8,MATCH($E83,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G83" s="53">
+      <c r="G83" s="105">
         <f>IF($F83=0,0,$F83/10)</f>
         <v/>
       </c>
-      <c r="H83" s="53">
+      <c r="H83" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C83,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I83" s="53" t="n"/>
+      <c r="I83" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: la aceptación del prestador por el paciente es del Gestor de Coordinación, que queda fuera.</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="30" customHeight="1">
-      <c r="A84" s="57" t="inlineStr">
+      <c r="A84" s="105" t="inlineStr">
         <is>
           <t>RF-080</t>
         </is>
       </c>
-      <c r="B84" s="57" t="inlineStr">
+      <c r="B84" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C84" s="57" t="inlineStr">
+      <c r="C84" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D84" s="57" t="inlineStr">
+      <c r="D84" s="105" t="inlineStr">
         <is>
           <t>¿Pueden comprometerse a que su primer release sea el contrato de API (aunque la solución completa de gobierno de datos no esté lista), para que Gestores pueda construir contra un contrato estable desde ya?</t>
         </is>
       </c>
       <c r="E84" s="54" t="n"/>
-      <c r="F84" s="53">
+      <c r="F84" s="105">
         <f>IF($E84="",0,INDEX($M$5:$M$8,MATCH($E84,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G84" s="53">
+      <c r="G84" s="105">
         <f>IF($F84=0,0,$F84/10)</f>
         <v/>
       </c>
-      <c r="H84" s="53">
+      <c r="H84" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C84,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I84" s="53" t="n"/>
+      <c r="I84" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="30" customHeight="1">
-      <c r="A85" s="53" t="inlineStr">
+      <c r="A85" s="105" t="inlineStr">
         <is>
           <t>RF-081</t>
         </is>
       </c>
-      <c r="B85" s="53" t="inlineStr">
+      <c r="B85" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C85" s="53" t="inlineStr">
+      <c r="C85" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D85" s="53" t="inlineStr">
+      <c r="D85" s="105" t="inlineStr">
         <is>
           <t>¿Cuál es la cobertura real hoy (cuántos y cuáles prestadores conectados, y si sigue limitado solo a consulta externa, como dijo Santiago en la sesión inicial?</t>
         </is>
       </c>
       <c r="E85" s="54" t="n"/>
-      <c r="F85" s="53">
+      <c r="F85" s="105">
         <f>IF($E85="",0,INDEX($M$5:$M$8,MATCH($E85,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G85" s="53">
+      <c r="G85" s="105">
         <f>IF($F85=0,0,$F85/10)</f>
         <v/>
       </c>
-      <c r="H85" s="53">
+      <c r="H85" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C85,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I85" s="53" t="n"/>
+      <c r="I85" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="30" customHeight="1">
-      <c r="A86" s="57" t="inlineStr">
+      <c r="A86" s="105" t="inlineStr">
         <is>
           <t>RF-082</t>
         </is>
       </c>
-      <c r="B86" s="57" t="inlineStr">
+      <c r="B86" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C86" s="57" t="inlineStr">
+      <c r="C86" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D86" s="57" t="inlineStr">
+      <c r="D86" s="105" t="inlineStr">
         <is>
           <t>Validar si el estándar RDA (Resumen Digital de Atención) cubre lo que Gestores necesita del gestor de Evaluación, o si hay vacíos.</t>
         </is>
       </c>
       <c r="E86" s="54" t="n"/>
-      <c r="F86" s="53">
+      <c r="F86" s="105">
         <f>IF($E86="",0,INDEX($M$5:$M$8,MATCH($E86,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G86" s="53">
+      <c r="G86" s="105">
         <f>IF($F86=0,0,$F86/10)</f>
         <v/>
       </c>
-      <c r="H86" s="53">
+      <c r="H86" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C86,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I86" s="53" t="n"/>
+      <c r="I86" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="30" customHeight="1">
-      <c r="A87" s="53" t="inlineStr">
+      <c r="A87" s="105" t="inlineStr">
         <is>
           <t>RF-083</t>
         </is>
       </c>
-      <c r="B87" s="53" t="inlineStr">
+      <c r="B87" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C87" s="53" t="inlineStr">
+      <c r="C87" s="105" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D87" s="53" t="inlineStr">
+      <c r="D87" s="105" t="inlineStr">
         <is>
           <t>Estrategia de canal de ingreso para prestadores declarada dual y no excluyente: la interoperabilidad de autorizaciones es el camino objetivo (“deber ser”); el Front del portal de prestadores se mantiene como contingencia, no se elimina.</t>
         </is>
       </c>
       <c r="E87" s="54" t="n"/>
-      <c r="F87" s="53">
+      <c r="F87" s="105">
         <f>IF($E87="",0,INDEX($M$5:$M$8,MATCH($E87,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G87" s="53">
+      <c r="G87" s="105">
         <f>IF($F87=0,0,$F87/10)</f>
         <v/>
       </c>
-      <c r="H87" s="53">
+      <c r="H87" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C87,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I87" s="53" t="n"/>
+      <c r="I87" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: define la estrategia dual de canal frente a la interoperabilidad de autorizaciones, que no entra al dibujo.</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="30" customHeight="1">
-      <c r="A88" s="57" t="inlineStr">
+      <c r="A88" s="105" t="inlineStr">
         <is>
           <t>RF-084</t>
         </is>
       </c>
-      <c r="B88" s="57" t="inlineStr">
+      <c r="B88" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C88" s="57" t="inlineStr">
+      <c r="C88" s="105" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D88" s="57" t="inlineStr">
+      <c r="D88" s="105" t="inlineStr">
         <is>
           <t>Para prestadores que ingresen vía interoperabilidad de autorizaciones (modelo orientado a eventos): el gestor se suscribe al ordenamiento en cuanto llega, consulta la historia clínica para completar la información y genera la autorización de forma automática, sin diligenciamiento de formulario ni carga de documentos por parte del prestador.</t>
         </is>
       </c>
       <c r="E88" s="54" t="n"/>
-      <c r="F88" s="53">
+      <c r="F88" s="105">
         <f>IF($E88="",0,INDEX($M$5:$M$8,MATCH($E88,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G88" s="53">
+      <c r="G88" s="105">
         <f>IF($F88=0,0,$F88/10)</f>
         <v/>
       </c>
-      <c r="H88" s="53">
+      <c r="H88" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C88,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I88" s="53" t="n"/>
+      <c r="I88" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: describe el ingreso por interoperabilidad de autorizaciones, que no está en el dibujo.</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="30" customHeight="1">
-      <c r="A89" s="53" t="inlineStr">
+      <c r="A89" s="105" t="inlineStr">
         <is>
           <t>RF-085</t>
         </is>
       </c>
-      <c r="B89" s="53" t="inlineStr">
+      <c r="B89" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C89" s="53" t="inlineStr">
+      <c r="C89" s="105" t="inlineStr">
         <is>
           <t>Canales / Front Externos</t>
         </is>
       </c>
-      <c r="D89" s="53" t="inlineStr">
+      <c r="D89" s="105" t="inlineStr">
         <is>
           <t>Para los prestadores conectados por interoperabilidad, el Front expondrá una vista de consulta del estado de la autorización frente al ordenamiento y la opción de creación de solicitud nueva (como contingencia), dado que la generación es automática y se actualiza en línea.</t>
         </is>
       </c>
       <c r="E89" s="54" t="n"/>
-      <c r="F89" s="53">
+      <c r="F89" s="105">
         <f>IF($E89="",0,INDEX($M$5:$M$8,MATCH($E89,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G89" s="53">
+      <c r="G89" s="105">
         <f>IF($F89=0,0,$F89/10)</f>
         <v/>
       </c>
-      <c r="H89" s="53">
+      <c r="H89" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C89,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I89" s="53" t="n"/>
+      <c r="I89" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: la vista para prestadores conectados por interoperabilidad depende de un frente que no entra.</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="30" customHeight="1">
       <c r="A90" s="57" t="inlineStr">
@@ -4955,382 +5246,422 @@
       <c r="I90" s="53" t="n"/>
     </row>
     <row r="91" ht="30" customHeight="1">
-      <c r="A91" s="53" t="inlineStr">
+      <c r="A91" s="105" t="inlineStr">
         <is>
           <t>RF-087</t>
         </is>
       </c>
-      <c r="B91" s="53" t="inlineStr">
+      <c r="B91" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C91" s="53" t="inlineStr">
+      <c r="C91" s="105" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D91" s="53" t="inlineStr">
+      <c r="D91" s="105" t="inlineStr">
         <is>
           <t>El Front web queda formalmente declarado como contingencia (no como opción principal): los prestadores que ingresen por el Front deberán migrar a interoperabilidad en algún punto. Se aclara explícitamente que “contingencia” no implica menor robustez ni pérdida de valor del canal.</t>
         </is>
       </c>
       <c r="E91" s="54" t="n"/>
-      <c r="F91" s="53">
+      <c r="F91" s="105">
         <f>IF($E91="",0,INDEX($M$5:$M$8,MATCH($E91,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G91" s="53">
+      <c r="G91" s="105">
         <f>IF($F91=0,0,$F91/10)</f>
         <v/>
       </c>
-      <c r="H91" s="53">
+      <c r="H91" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C91,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I91" s="53" t="n"/>
+      <c r="I91" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: es una definición sobre el front como contingencia frente a la interoperabilidad, que no entra.</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="30" customHeight="1">
-      <c r="A92" s="57" t="inlineStr">
+      <c r="A92" s="105" t="inlineStr">
         <is>
           <t>RF-088</t>
         </is>
       </c>
-      <c r="B92" s="57" t="inlineStr">
+      <c r="B92" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C92" s="57" t="inlineStr">
+      <c r="C92" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D92" s="57" t="inlineStr">
+      <c r="D92" s="105" t="inlineStr">
         <is>
           <t>Se requiere un plan de conexión/incentivo (gancho de valor operativo, no solo normativo) para escalar de los ~3.400 prestadores hoy conectados en interoperabilidad de historia clínica hacia la interoperabilidad de autorizaciones, priorizando instituciones de alto volumen de atención aún no conectadas (ej. Imbanaco, Fundación Valle del Lili, Pablo Tobón Uribe, Clínica Santa Fe).</t>
         </is>
       </c>
       <c r="E92" s="54" t="n"/>
-      <c r="F92" s="53">
+      <c r="F92" s="105">
         <f>IF($E92="",0,INDEX($M$5:$M$8,MATCH($E92,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G92" s="53">
+      <c r="G92" s="105">
         <f>IF($F92=0,0,$F92/10)</f>
         <v/>
       </c>
-      <c r="H92" s="53">
+      <c r="H92" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C92,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I92" s="53" t="n"/>
+      <c r="I92" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="30" customHeight="1">
-      <c r="A93" s="53" t="inlineStr">
+      <c r="A93" s="105" t="inlineStr">
         <is>
           <t>RF-089</t>
         </is>
       </c>
-      <c r="B93" s="53" t="inlineStr">
+      <c r="B93" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C93" s="53" t="inlineStr">
+      <c r="C93" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D93" s="53" t="inlineStr">
+      <c r="D93" s="105" t="inlineStr">
         <is>
           <t>Pendiente confirmar el responsable desde Negocio que jalone/lidere la adopción de interoperabilidad ante los prestadores; Pao de la Cuesta asumiría esa gestión desde su nuevo rol, a confirmar.</t>
         </is>
       </c>
       <c r="E93" s="54" t="n"/>
-      <c r="F93" s="53">
+      <c r="F93" s="105">
         <f>IF($E93="",0,INDEX($M$5:$M$8,MATCH($E93,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G93" s="53">
+      <c r="G93" s="105">
         <f>IF($F93=0,0,$F93/10)</f>
         <v/>
       </c>
-      <c r="H93" s="53">
+      <c r="H93" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C93,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I93" s="53" t="n"/>
+      <c r="I93" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="30" customHeight="1">
-      <c r="A94" s="57" t="inlineStr">
+      <c r="A94" s="105" t="inlineStr">
         <is>
           <t>RF-090</t>
         </is>
       </c>
-      <c r="B94" s="57" t="inlineStr">
+      <c r="B94" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C94" s="57" t="inlineStr">
+      <c r="C94" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D94" s="57" t="inlineStr">
+      <c r="D94" s="105" t="inlineStr">
         <is>
           <t>Cruzar el listado de prestadores compartido por checho (Interoperabilidad) contra el informe de autorizaciones totales por prestador de todo 2026 (a extraer de Globalweb), para determinar el volumen de autorizaciones por prestador.</t>
         </is>
       </c>
       <c r="E94" s="54" t="n"/>
-      <c r="F94" s="53">
+      <c r="F94" s="105">
         <f>IF($E94="",0,INDEX($M$5:$M$8,MATCH($E94,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G94" s="53">
+      <c r="G94" s="105">
         <f>IF($F94=0,0,$F94/10)</f>
         <v/>
       </c>
-      <c r="H94" s="53">
+      <c r="H94" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C94,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I94" s="53" t="n"/>
+      <c r="I94" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="30" customHeight="1">
-      <c r="A95" s="53" t="inlineStr">
+      <c r="A95" s="105" t="inlineStr">
         <is>
           <t>RF-091</t>
         </is>
       </c>
-      <c r="B95" s="53" t="inlineStr">
+      <c r="B95" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C95" s="53" t="inlineStr">
+      <c r="C95" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D95" s="53" t="inlineStr">
+      <c r="D95" s="105" t="inlineStr">
         <is>
           <t>Se expone vista consolidada/agregada del proceso (“el bosque”) y el detalle caso a caso de una solicitud específica (“el árbol”)</t>
         </is>
       </c>
       <c r="E95" s="54" t="n"/>
-      <c r="F95" s="53">
+      <c r="F95" s="105">
         <f>IF($E95="",0,INDEX($M$5:$M$8,MATCH($E95,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G95" s="53">
+      <c r="G95" s="105">
         <f>IF($F95=0,0,$F95/10)</f>
         <v/>
       </c>
-      <c r="H95" s="53">
+      <c r="H95" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C95,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I95" s="53" t="n"/>
+      <c r="I95" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="30" customHeight="1">
-      <c r="A96" s="57" t="inlineStr">
+      <c r="A96" s="105" t="inlineStr">
         <is>
           <t>RF-092</t>
         </is>
       </c>
-      <c r="B96" s="57" t="inlineStr">
+      <c r="B96" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C96" s="57" t="inlineStr">
+      <c r="C96" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D96" s="57" t="inlineStr">
+      <c r="D96" s="105" t="inlineStr">
         <is>
           <t>Alertamiento por información pendiente del cliente en el proceso de Solicitud de Autorización</t>
         </is>
       </c>
       <c r="E96" s="54" t="n"/>
-      <c r="F96" s="53">
+      <c r="F96" s="105">
         <f>IF($E96="",0,INDEX($M$5:$M$8,MATCH($E96,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G96" s="53">
+      <c r="G96" s="105">
         <f>IF($F96=0,0,$F96/10)</f>
         <v/>
       </c>
-      <c r="H96" s="53">
+      <c r="H96" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C96,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I96" s="53" t="n"/>
+      <c r="I96" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="30" customHeight="1">
-      <c r="A97" s="53" t="inlineStr">
+      <c r="A97" s="105" t="inlineStr">
         <is>
           <t>RF-093</t>
         </is>
       </c>
-      <c r="B97" s="53" t="inlineStr">
+      <c r="B97" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C97" s="53" t="inlineStr">
+      <c r="C97" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D97" s="53" t="inlineStr">
+      <c r="D97" s="105" t="inlineStr">
         <is>
           <t>Alertamiento por incumplimiento del SLA por la solicitud de Autorización</t>
         </is>
       </c>
       <c r="E97" s="54" t="n"/>
-      <c r="F97" s="53">
+      <c r="F97" s="105">
         <f>IF($E97="",0,INDEX($M$5:$M$8,MATCH($E97,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G97" s="53">
+      <c r="G97" s="105">
         <f>IF($F97=0,0,$F97/10)</f>
         <v/>
       </c>
-      <c r="H97" s="53">
+      <c r="H97" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C97,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I97" s="53" t="n"/>
+      <c r="I97" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="30" customHeight="1">
-      <c r="A98" s="57" t="inlineStr">
+      <c r="A98" s="105" t="inlineStr">
         <is>
           <t>RF-094</t>
         </is>
       </c>
-      <c r="B98" s="57" t="inlineStr">
+      <c r="B98" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C98" s="57" t="inlineStr">
+      <c r="C98" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D98" s="57" t="inlineStr">
+      <c r="D98" s="105" t="inlineStr">
         <is>
           <t>Alertamiento por próximo incumplimiento del SLA por la solicitud de Autorización</t>
         </is>
       </c>
       <c r="E98" s="54" t="n"/>
-      <c r="F98" s="53">
+      <c r="F98" s="105">
         <f>IF($E98="",0,INDEX($M$5:$M$8,MATCH($E98,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G98" s="53">
+      <c r="G98" s="105">
         <f>IF($F98=0,0,$F98/10)</f>
         <v/>
       </c>
-      <c r="H98" s="53">
+      <c r="H98" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C98,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I98" s="53" t="n"/>
+      <c r="I98" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="30" customHeight="1">
-      <c r="A99" s="53" t="inlineStr">
+      <c r="A99" s="105" t="inlineStr">
         <is>
           <t>RF-095</t>
         </is>
       </c>
-      <c r="B99" s="53" t="inlineStr">
+      <c r="B99" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C99" s="53" t="inlineStr">
+      <c r="C99" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D99" s="53" t="inlineStr">
+      <c r="D99" s="105" t="inlineStr">
         <is>
           <t>Alertamiento en el desborde de capacidad en el proceso de Solicitud de Autorización</t>
         </is>
       </c>
       <c r="E99" s="54" t="n"/>
-      <c r="F99" s="53">
+      <c r="F99" s="105">
         <f>IF($E99="",0,INDEX($M$5:$M$8,MATCH($E99,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G99" s="53">
+      <c r="G99" s="105">
         <f>IF($F99=0,0,$F99/10)</f>
         <v/>
       </c>
-      <c r="H99" s="53">
+      <c r="H99" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C99,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I99" s="53" t="n"/>
+      <c r="I99" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="30" customHeight="1">
-      <c r="A100" s="57" t="inlineStr">
+      <c r="A100" s="105" t="inlineStr">
         <is>
           <t>RF-096</t>
         </is>
       </c>
-      <c r="B100" s="57" t="inlineStr">
+      <c r="B100" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C100" s="57" t="inlineStr">
+      <c r="C100" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D100" s="57" t="inlineStr">
+      <c r="D100" s="105" t="inlineStr">
         <is>
           <t xml:space="preserve">Capacidad de Parametrización para alertamientos en la solicitud de autorización </t>
         </is>
       </c>
       <c r="E100" s="54" t="n"/>
-      <c r="F100" s="53">
+      <c r="F100" s="105">
         <f>IF($E100="",0,INDEX($M$5:$M$8,MATCH($E100,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G100" s="53">
+      <c r="G100" s="105">
         <f>IF($F100=0,0,$F100/10)</f>
         <v/>
       </c>
-      <c r="H100" s="53">
+      <c r="H100" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C100,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I100" s="53" t="n"/>
+      <c r="I100" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="30" customHeight="1">
-      <c r="A101" s="53" t="inlineStr">
+      <c r="A101" s="105" t="inlineStr">
         <is>
           <t>RF-097</t>
         </is>
       </c>
-      <c r="B101" s="53" t="inlineStr">
+      <c r="B101" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C101" s="53" t="inlineStr">
+      <c r="C101" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D101" s="53" t="inlineStr">
+      <c r="D101" s="105" t="inlineStr">
         <is>
           <t xml:space="preserve">Concepto de “gestor auditor” dentro de cada gestor y en torre de control nos permita ver el comportamiento y sugerencias para mejorar la autonomía del gestor </t>
         </is>
@@ -5340,127 +5671,143 @@
           <t>L</t>
         </is>
       </c>
-      <c r="F101" s="53">
+      <c r="F101" s="105">
         <f>IF($E101="",0,INDEX($M$5:$M$8,MATCH($E101,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G101" s="53">
+      <c r="G101" s="105">
         <f>IF($F101=0,0,$F101/10)</f>
         <v/>
       </c>
-      <c r="H101" s="53">
+      <c r="H101" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C101,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I101" s="53" t="n"/>
+      <c r="I101" s="105" t="inlineStr">
+        <is>
+          <t>Entra el agente auditor dentro de cada gestor, que el dibujo del MVP incluye en Solicitud y en Evaluación. El auditor de la torre es capa 3 y queda fuera.</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="30" customHeight="1">
-      <c r="A102" s="57" t="inlineStr">
+      <c r="A102" s="105" t="inlineStr">
         <is>
           <t>RF-098</t>
         </is>
       </c>
-      <c r="B102" s="57" t="inlineStr">
+      <c r="B102" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C102" s="57" t="inlineStr">
+      <c r="C102" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D102" s="57" t="inlineStr">
+      <c r="D102" s="105" t="inlineStr">
         <is>
           <t>Agente que realice sugerencias sobre la decisión que se debe tomar en una solicitud ejemplo: sugerencia al lider operativo de reasignación de solicitudes que superen el tiempo de respuesta a otros evaluadores con mayor oportunidad de respuesta</t>
         </is>
       </c>
       <c r="E102" s="54" t="n"/>
-      <c r="F102" s="53">
+      <c r="F102" s="105">
         <f>IF($E102="",0,INDEX($M$5:$M$8,MATCH($E102,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G102" s="53">
+      <c r="G102" s="105">
         <f>IF($F102=0,0,$F102/10)</f>
         <v/>
       </c>
-      <c r="H102" s="53">
+      <c r="H102" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C102,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I102" s="53" t="n"/>
+      <c r="I102" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="30" customHeight="1">
-      <c r="A103" s="53" t="inlineStr">
+      <c r="A103" s="105" t="inlineStr">
         <is>
           <t>RF-099</t>
         </is>
       </c>
-      <c r="B103" s="53" t="inlineStr">
+      <c r="B103" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C103" s="53" t="inlineStr">
+      <c r="C103" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D103" s="53" t="inlineStr">
+      <c r="D103" s="105" t="inlineStr">
         <is>
           <t>Agente que tome decisiones sobre el marco de actuación de una solicitud, ejemplo: reasignación automatica de solicitudes que superen el tiempo de respuesta a otros evaluadores con mayor oportunidad de respuesta</t>
         </is>
       </c>
       <c r="E103" s="54" t="n"/>
-      <c r="F103" s="53">
+      <c r="F103" s="105">
         <f>IF($E103="",0,INDEX($M$5:$M$8,MATCH($E103,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G103" s="53">
+      <c r="G103" s="105">
         <f>IF($F103=0,0,$F103/10)</f>
         <v/>
       </c>
-      <c r="H103" s="53">
+      <c r="H103" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C103,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I103" s="53" t="n"/>
+      <c r="I103" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="30" customHeight="1">
-      <c r="A104" s="57" t="inlineStr">
+      <c r="A104" s="105" t="inlineStr">
         <is>
           <t>RF-100</t>
         </is>
       </c>
-      <c r="B104" s="57" t="inlineStr">
+      <c r="B104" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C104" s="57" t="inlineStr">
+      <c r="C104" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D104" s="57" t="inlineStr">
+      <c r="D104" s="105" t="inlineStr">
         <is>
           <t>Emitir alertamiento cuando se tengan novedades en la solicitud al cliente/proveedor y asesor, ejemplo: por incumplimiento de SLA</t>
         </is>
       </c>
       <c r="E104" s="54" t="n"/>
-      <c r="F104" s="53">
+      <c r="F104" s="105">
         <f>IF($E104="",0,INDEX($M$5:$M$8,MATCH($E104,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G104" s="53">
+      <c r="G104" s="105">
         <f>IF($F104=0,0,$F104/10)</f>
         <v/>
       </c>
-      <c r="H104" s="53">
+      <c r="H104" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C104,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I104" s="53" t="n"/>
+      <c r="I104" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="30" customHeight="1">
       <c r="A105" s="53" t="inlineStr">
@@ -5499,112 +5846,124 @@
       <c r="I105" s="53" t="n"/>
     </row>
     <row r="106" ht="30" customHeight="1">
-      <c r="A106" s="57" t="inlineStr">
+      <c r="A106" s="105" t="inlineStr">
         <is>
           <t>RF-102</t>
         </is>
       </c>
-      <c r="B106" s="57" t="inlineStr">
+      <c r="B106" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C106" s="57" t="inlineStr">
+      <c r="C106" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D106" s="57" t="inlineStr">
+      <c r="D106" s="105" t="inlineStr">
         <is>
           <t>El agente entrega analítica prescriptiva integrando Torre + Datalake</t>
         </is>
       </c>
       <c r="E106" s="54" t="n"/>
-      <c r="F106" s="53">
+      <c r="F106" s="105">
         <f>IF($E106="",0,INDEX($M$5:$M$8,MATCH($E106,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G106" s="53">
+      <c r="G106" s="105">
         <f>IF($F106=0,0,$F106/10)</f>
         <v/>
       </c>
-      <c r="H106" s="53">
+      <c r="H106" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C106,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I106" s="53" t="n"/>
+      <c r="I106" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="30" customHeight="1">
-      <c r="A107" s="53" t="inlineStr">
+      <c r="A107" s="105" t="inlineStr">
         <is>
           <t>RF-103</t>
         </is>
       </c>
-      <c r="B107" s="53" t="inlineStr">
+      <c r="B107" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C107" s="53" t="inlineStr">
+      <c r="C107" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D107" s="53" t="inlineStr">
+      <c r="D107" s="105" t="inlineStr">
         <is>
           <t>Entrega de información de las solicitudes, autorizaciones y datos relevantes al Datalake</t>
         </is>
       </c>
       <c r="E107" s="54" t="n"/>
-      <c r="F107" s="53">
+      <c r="F107" s="105">
         <f>IF($E107="",0,INDEX($M$5:$M$8,MATCH($E107,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G107" s="53">
+      <c r="G107" s="105">
         <f>IF($F107=0,0,$F107/10)</f>
         <v/>
       </c>
-      <c r="H107" s="53">
+      <c r="H107" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C107,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I107" s="53" t="n"/>
+      <c r="I107" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="30" customHeight="1">
-      <c r="A108" s="57" t="inlineStr">
+      <c r="A108" s="105" t="inlineStr">
         <is>
           <t>RF-104</t>
         </is>
       </c>
-      <c r="B108" s="57" t="inlineStr">
+      <c r="B108" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C108" s="57" t="inlineStr">
+      <c r="C108" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D108" s="57" t="inlineStr">
+      <c r="D108" s="105" t="inlineStr">
         <is>
           <t>Garantizar que la arquitectura, integraciones, aplicaciones y conexiones que intervienen en el proceso este funcionando de forma adecuada y reaizar alertamientos ante alguna novedad</t>
         </is>
       </c>
       <c r="E108" s="54" t="n"/>
-      <c r="F108" s="53">
+      <c r="F108" s="105">
         <f>IF($E108="",0,INDEX($M$5:$M$8,MATCH($E108,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G108" s="53">
+      <c r="G108" s="105">
         <f>IF($F108=0,0,$F108/10)</f>
         <v/>
       </c>
-      <c r="H108" s="53">
+      <c r="H108" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C108,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I108" s="53" t="n"/>
+      <c r="I108" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="30" customHeight="1">
       <c r="A109" s="53" t="inlineStr">
@@ -5643,40 +6002,44 @@
       <c r="I109" s="53" t="n"/>
     </row>
     <row r="110" ht="30" customHeight="1">
-      <c r="A110" s="57" t="inlineStr">
+      <c r="A110" s="105" t="inlineStr">
         <is>
           <t>RF-106</t>
         </is>
       </c>
-      <c r="B110" s="57" t="inlineStr">
+      <c r="B110" s="105" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C110" s="57" t="inlineStr">
+      <c r="C110" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D110" s="57" t="inlineStr">
+      <c r="D110" s="105" t="inlineStr">
         <is>
           <t>Front de configuración de SLAs según criterios</t>
         </is>
       </c>
       <c r="E110" s="54" t="n"/>
-      <c r="F110" s="53">
+      <c r="F110" s="105">
         <f>IF($E110="",0,INDEX($M$5:$M$8,MATCH($E110,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G110" s="53">
+      <c r="G110" s="105">
         <f>IF($F110=0,0,$F110/10)</f>
         <v/>
       </c>
-      <c r="H110" s="53">
+      <c r="H110" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C110,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I110" s="53" t="n"/>
+      <c r="I110" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="30" customHeight="1">
       <c r="A111" s="53" t="inlineStr">
@@ -5831,40 +6194,44 @@
       <c r="I114" s="53" t="n"/>
     </row>
     <row r="115" ht="30" customHeight="1">
-      <c r="A115" s="53" t="inlineStr">
+      <c r="A115" s="106" t="inlineStr">
         <is>
           <t>RT-003</t>
         </is>
       </c>
-      <c r="B115" s="53" t="inlineStr">
+      <c r="B115" s="106" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C115" s="53" t="inlineStr">
+      <c r="C115" s="106" t="inlineStr">
         <is>
           <t>Transversal / Principios generales</t>
         </is>
       </c>
-      <c r="D115" s="53" t="inlineStr">
+      <c r="D115" s="106" t="inlineStr">
         <is>
           <t>Riesgo/premisa explícita: el proyecto solo tiene sentido si los cores implementan la capacidad de exponer información vía API a tiempo.</t>
         </is>
       </c>
-      <c r="E115" s="54" t="n"/>
-      <c r="F115" s="53">
+      <c r="E115" s="107" t="n"/>
+      <c r="F115" s="106">
         <f>IF($E115="",0,INDEX($M$5:$M$8,MATCH($E115,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G115" s="53">
+      <c r="G115" s="106">
         <f>IF($F115=0,0,$F115/10)</f>
         <v/>
       </c>
-      <c r="H115" s="53">
+      <c r="H115" s="106">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C115,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I115" s="53" t="n"/>
+      <c r="I115" s="106" t="inlineStr">
+        <is>
+          <t>🟥 No es un entregable de construcción sino una premisa de riesgo del proyecto. No se talla; se gestiona como dependencia externa de los cores.</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="30" customHeight="1">
       <c r="A116" s="57" t="inlineStr">
@@ -6027,40 +6394,44 @@
       <c r="I119" s="53" t="n"/>
     </row>
     <row r="120" ht="30" customHeight="1">
-      <c r="A120" s="57" t="inlineStr">
+      <c r="A120" s="106" t="inlineStr">
         <is>
           <t>RT-008</t>
         </is>
       </c>
-      <c r="B120" s="57" t="inlineStr">
+      <c r="B120" s="106" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C120" s="57" t="inlineStr">
+      <c r="C120" s="106" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D120" s="57" t="inlineStr">
+      <c r="D120" s="106" t="inlineStr">
         <is>
           <t>Front nuevo (Flutter), embebido en Sucursal Virtual Personas, AVA y Portal de Prestadores; reutiliza el back/orquestador de Siniestro Integral.</t>
         </is>
       </c>
-      <c r="E120" s="54" t="n"/>
-      <c r="F120" s="53">
+      <c r="E120" s="107" t="n"/>
+      <c r="F120" s="106">
         <f>IF($E120="",0,INDEX($M$5:$M$8,MATCH($E120,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G120" s="53">
+      <c r="G120" s="106">
         <f>IF($F120=0,0,$F120/10)</f>
         <v/>
       </c>
-      <c r="H120" s="53">
+      <c r="H120" s="106">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C120,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I120" s="53" t="n"/>
+      <c r="I120" s="106" t="inlineStr">
+        <is>
+          <t>🟥 Conflicto con el lineamiento. El requisito dice front en Flutter; el lineamiento AI First fija la experiencia en Azure Static Web App con Angular SPA (Arquitectura de implementación, página 6243680318). Resolver la tecnología del front antes de tallar.</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="30" customHeight="1">
       <c r="A121" s="53" t="inlineStr">
@@ -6183,40 +6554,44 @@
       <c r="I123" s="53" t="n"/>
     </row>
     <row r="124" ht="30" customHeight="1">
-      <c r="A124" s="57" t="inlineStr">
+      <c r="A124" s="106" t="inlineStr">
         <is>
           <t>RT-012</t>
         </is>
       </c>
-      <c r="B124" s="57" t="inlineStr">
+      <c r="B124" s="106" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C124" s="57" t="inlineStr">
+      <c r="C124" s="106" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D124" s="57" t="inlineStr">
+      <c r="D124" s="106" t="inlineStr">
         <is>
           <t>OCR/IA: LLM multimodal interpreta documentos directamente (15-40 seg); reutiliza el agente de pre-radicación de EPS (~93% de precisión).</t>
         </is>
       </c>
-      <c r="E124" s="54" t="n"/>
-      <c r="F124" s="53">
+      <c r="E124" s="107" t="n"/>
+      <c r="F124" s="106">
         <f>IF($E124="",0,INDEX($M$5:$M$8,MATCH($E124,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G124" s="53">
+      <c r="G124" s="106">
         <f>IF($F124=0,0,$F124/10)</f>
         <v/>
       </c>
-      <c r="H124" s="53">
+      <c r="H124" s="106">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C124,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I124" s="53" t="n"/>
+      <c r="I124" s="106" t="inlineStr">
+        <is>
+          <t>🟥 Conflicto con el lineamiento. El requisito dice que un LLM multimodal interpreta los documentos directamente; el stack v0.5 declara Azure Document Intelligence obligatorio para OCR y extracción estructurada (Diseño Datos RAG/Knowledge/Memory, página 5900140571). El esfuerzo cambia según cuál se adopte.</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="30" customHeight="1">
       <c r="A125" s="53" t="inlineStr">
@@ -6335,40 +6710,44 @@
       <c r="I127" s="53" t="n"/>
     </row>
     <row r="128" ht="30" customHeight="1">
-      <c r="A128" s="57" t="inlineStr">
+      <c r="A128" s="106" t="inlineStr">
         <is>
           <t>RT-016</t>
         </is>
       </c>
-      <c r="B128" s="57" t="inlineStr">
+      <c r="B128" s="106" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C128" s="57" t="inlineStr">
+      <c r="C128" s="106" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D128" s="57" t="inlineStr">
+      <c r="D128" s="106" t="inlineStr">
         <is>
           <t>Riesgo técnico abierto: Super App en Google Cloud vs. resto del ecosistema en Azure.</t>
         </is>
       </c>
-      <c r="E128" s="54" t="n"/>
-      <c r="F128" s="53">
+      <c r="E128" s="107" t="n"/>
+      <c r="F128" s="106">
         <f>IF($E128="",0,INDEX($M$5:$M$8,MATCH($E128,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G128" s="53">
+      <c r="G128" s="106">
         <f>IF($F128=0,0,$F128/10)</f>
         <v/>
       </c>
-      <c r="H128" s="53">
+      <c r="H128" s="106">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C128,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I128" s="53" t="n"/>
+      <c r="I128" s="106" t="inlineStr">
+        <is>
+          <t>🟥 Riesgo abierto, no entregable: la Super App opera en Google Cloud y el resto del ecosistema en Azure. Afecta a dos canales dibujados en el MVP. Requiere decisión de arquitectura antes de poder tallarlo.</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="30" customHeight="1">
       <c r="A129" s="53" t="inlineStr">
@@ -6451,40 +6830,44 @@
       <c r="I130" s="53" t="n"/>
     </row>
     <row r="131" ht="30" customHeight="1">
-      <c r="A131" s="53" t="inlineStr">
+      <c r="A131" s="106" t="inlineStr">
         <is>
           <t>RT-019</t>
         </is>
       </c>
-      <c r="B131" s="53" t="inlineStr">
+      <c r="B131" s="106" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C131" s="53" t="inlineStr">
+      <c r="C131" s="106" t="inlineStr">
         <is>
           <t>Gestor de Evaluación</t>
         </is>
       </c>
-      <c r="D131" s="53" t="inlineStr">
+      <c r="D131" s="106" t="inlineStr">
         <is>
           <t>Debe consultar políticas/reglas a SuraHis manteniendo también reglas propias de agente (modelo híbrido).</t>
         </is>
       </c>
-      <c r="E131" s="54" t="n"/>
-      <c r="F131" s="53">
+      <c r="E131" s="107" t="n"/>
+      <c r="F131" s="106">
         <f>IF($E131="",0,INDEX($M$5:$M$8,MATCH($E131,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G131" s="53">
+      <c r="G131" s="106">
         <f>IF($F131=0,0,$F131/10)</f>
         <v/>
       </c>
-      <c r="H131" s="53">
+      <c r="H131" s="106">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C131,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I131" s="53" t="n"/>
+      <c r="I131" s="106" t="inlineStr">
+        <is>
+          <t>🟥 Duplicado exacto de RT-018. Se deja sin tallar para no contar dos veces el mismo esfuerzo; conviene eliminarlo o diferenciarlo.</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="30" customHeight="1">
       <c r="A132" s="57" t="inlineStr">
@@ -6935,112 +7318,124 @@
       <c r="I143" s="53" t="n"/>
     </row>
     <row r="144" ht="30" customHeight="1">
-      <c r="A144" s="57" t="inlineStr">
+      <c r="A144" s="105" t="inlineStr">
         <is>
           <t>RT-032</t>
         </is>
       </c>
-      <c r="B144" s="57" t="inlineStr">
+      <c r="B144" s="105" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C144" s="57" t="inlineStr">
+      <c r="C144" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D144" s="57" t="inlineStr">
+      <c r="D144" s="105" t="inlineStr">
         <is>
           <t>Pendiente definir si se expone una API única con filtrado por perfil o múltiples APIs por actor.</t>
         </is>
       </c>
       <c r="E144" s="54" t="n"/>
-      <c r="F144" s="53">
+      <c r="F144" s="105">
         <f>IF($E144="",0,INDEX($M$5:$M$8,MATCH($E144,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G144" s="53">
+      <c r="G144" s="105">
         <f>IF($F144=0,0,$F144/10)</f>
         <v/>
       </c>
-      <c r="H144" s="53">
+      <c r="H144" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C144,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I144" s="53" t="n"/>
+      <c r="I144" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="145" ht="30" customHeight="1">
-      <c r="A145" s="53" t="inlineStr">
+      <c r="A145" s="105" t="inlineStr">
         <is>
           <t>RT-033</t>
         </is>
       </c>
-      <c r="B145" s="53" t="inlineStr">
+      <c r="B145" s="105" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C145" s="53" t="inlineStr">
+      <c r="C145" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D145" s="53" t="inlineStr">
+      <c r="D145" s="105" t="inlineStr">
         <is>
           <t>Reto de integración en tiempo real con prestadores — hoy no existe (solo portal con interacción manual).</t>
         </is>
       </c>
       <c r="E145" s="54" t="n"/>
-      <c r="F145" s="53">
+      <c r="F145" s="105">
         <f>IF($E145="",0,INDEX($M$5:$M$8,MATCH($E145,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G145" s="53">
+      <c r="G145" s="105">
         <f>IF($F145=0,0,$F145/10)</f>
         <v/>
       </c>
-      <c r="H145" s="53">
+      <c r="H145" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C145,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I145" s="53" t="n"/>
+      <c r="I145" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="146" ht="30" customHeight="1">
-      <c r="A146" s="57" t="inlineStr">
+      <c r="A146" s="105" t="inlineStr">
         <is>
           <t>RT-034</t>
         </is>
       </c>
-      <c r="B146" s="57" t="inlineStr">
+      <c r="B146" s="105" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C146" s="57" t="inlineStr">
+      <c r="C146" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D146" s="57" t="inlineStr">
+      <c r="D146" s="105" t="inlineStr">
         <is>
           <t>Datalake de autorizaciones como entregable técnico del Release 3 (feb-abr 2027), con apoyo del arquitecto de datos.</t>
         </is>
       </c>
       <c r="E146" s="54" t="n"/>
-      <c r="F146" s="53">
+      <c r="F146" s="105">
         <f>IF($E146="",0,INDEX($M$5:$M$8,MATCH($E146,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G146" s="53">
+      <c r="G146" s="105">
         <f>IF($F146=0,0,$F146/10)</f>
         <v/>
       </c>
-      <c r="H146" s="53">
+      <c r="H146" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C146,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I146" s="53" t="n"/>
+      <c r="I146" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="147" ht="30" customHeight="1">
       <c r="A147" s="53" t="inlineStr">
@@ -7115,148 +7510,164 @@
       <c r="I148" s="53" t="n"/>
     </row>
     <row r="149" ht="30" customHeight="1">
-      <c r="A149" s="53" t="inlineStr">
+      <c r="A149" s="106" t="inlineStr">
         <is>
           <t>RT-037</t>
         </is>
       </c>
-      <c r="B149" s="53" t="inlineStr">
+      <c r="B149" s="106" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C149" s="53" t="inlineStr">
+      <c r="C149" s="106" t="inlineStr">
         <is>
           <t>Transversal / Principios generales</t>
         </is>
       </c>
-      <c r="D149" s="53" t="inlineStr">
+      <c r="D149" s="106" t="inlineStr">
         <is>
           <t>Toda estimación presentada a patrocinadores en fase de estructuración debe declarar explícitamente un margen de incertidumbre del 30%.</t>
         </is>
       </c>
-      <c r="E149" s="54" t="n"/>
-      <c r="F149" s="53">
+      <c r="E149" s="107" t="n"/>
+      <c r="F149" s="106">
         <f>IF($E149="",0,INDEX($M$5:$M$8,MATCH($E149,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G149" s="53">
+      <c r="G149" s="106">
         <f>IF($F149=0,0,$F149/10)</f>
         <v/>
       </c>
-      <c r="H149" s="53">
+      <c r="H149" s="106">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C149,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I149" s="53" t="n"/>
+      <c r="I149" s="106" t="inlineStr">
+        <is>
+          <t>🟥 No es un entregable de construcción: es la regla de presentación de la estimación (declarar 30% de incertidumbre). Aplica a este ejercicio, no se talla.</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="30" customHeight="1">
-      <c r="A150" s="57" t="inlineStr">
+      <c r="A150" s="106" t="inlineStr">
         <is>
           <t>RT-038</t>
         </is>
       </c>
-      <c r="B150" s="57" t="inlineStr">
+      <c r="B150" s="106" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C150" s="57" t="inlineStr">
+      <c r="C150" s="106" t="inlineStr">
         <is>
           <t>Transversal / Principios generales</t>
         </is>
       </c>
-      <c r="D150" s="57" t="inlineStr">
+      <c r="D150" s="106" t="inlineStr">
         <is>
           <t>El backlog se talla con escala estándar M≈5 días (medio sprint), L≈10 días (1 sprint), XL≈20 días (2 sprints), aplicada de forma consistente entre gestores para poder comparar esfuerzo.</t>
         </is>
       </c>
-      <c r="E150" s="54" t="n"/>
-      <c r="F150" s="53">
+      <c r="E150" s="107" t="n"/>
+      <c r="F150" s="106">
         <f>IF($E150="",0,INDEX($M$5:$M$8,MATCH($E150,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G150" s="53">
+      <c r="G150" s="106">
         <f>IF($F150=0,0,$F150/10)</f>
         <v/>
       </c>
-      <c r="H150" s="53">
+      <c r="H150" s="106">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C150,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I150" s="53" t="n"/>
+      <c r="I150" s="106" t="inlineStr">
+        <is>
+          <t>🟥 No es un entregable: es la propia escala de tallaje que usa esta hoja (M≈5, L≈10, XL≈20). Aplica a este ejercicio, no se talla.</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="30" customHeight="1">
-      <c r="A151" s="53" t="inlineStr">
+      <c r="A151" s="105" t="inlineStr">
         <is>
           <t>RT-039</t>
         </is>
       </c>
-      <c r="B151" s="53" t="inlineStr">
+      <c r="B151" s="105" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C151" s="53" t="inlineStr">
+      <c r="C151" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D151" s="53" t="inlineStr">
+      <c r="D151" s="105" t="inlineStr">
         <is>
           <t>El modelo de eventos de interoperabilidad de historia clínica migra hacia una arquitectura 2.0 orientada a eventos (colas por suscripción/webhooks), desde la arquitectura tradicional de microservicios; hoy conecta 6 prestadores de ayuda diagnóstica externa.</t>
         </is>
       </c>
       <c r="E151" s="54" t="n"/>
-      <c r="F151" s="53">
+      <c r="F151" s="105">
         <f>IF($E151="",0,INDEX($M$5:$M$8,MATCH($E151,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G151" s="53">
+      <c r="G151" s="105">
         <f>IF($F151=0,0,$F151/10)</f>
         <v/>
       </c>
-      <c r="H151" s="53">
+      <c r="H151" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C151,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I151" s="53" t="n"/>
+      <c r="I151" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="30" customHeight="1">
-      <c r="A152" s="57" t="inlineStr">
+      <c r="A152" s="105" t="inlineStr">
         <is>
           <t>RT-040</t>
         </is>
       </c>
-      <c r="B152" s="57" t="inlineStr">
+      <c r="B152" s="105" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C152" s="57" t="inlineStr">
+      <c r="C152" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D152" s="57" t="inlineStr">
+      <c r="D152" s="105" t="inlineStr">
         <is>
           <t>No existe hoy interoperabilidad de agenda por barreras de mercado (ningún prestador ni aseguradora quiere ser el centralizador); una propuesta de mercado con un tercero integrador está en etapa muy temprana.</t>
         </is>
       </c>
       <c r="E152" s="54" t="n"/>
-      <c r="F152" s="53">
+      <c r="F152" s="105">
         <f>IF($E152="",0,INDEX($M$5:$M$8,MATCH($E152,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G152" s="53">
+      <c r="G152" s="105">
         <f>IF($F152=0,0,$F152/10)</f>
         <v/>
       </c>
-      <c r="H152" s="53">
+      <c r="H152" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C152,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I152" s="53" t="n"/>
+      <c r="I152" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="153" ht="30" customHeight="1">
       <c r="A153" s="53" t="inlineStr">
@@ -7331,40 +7742,44 @@
       <c r="I154" s="53" t="n"/>
     </row>
     <row r="155" ht="30" customHeight="1">
-      <c r="A155" s="53" t="inlineStr">
+      <c r="A155" s="106" t="inlineStr">
         <is>
           <t>RT-043</t>
         </is>
       </c>
-      <c r="B155" s="53" t="inlineStr">
+      <c r="B155" s="106" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C155" s="53" t="inlineStr">
+      <c r="C155" s="106" t="inlineStr">
         <is>
           <t>Transversal / Principios generales</t>
         </is>
       </c>
-      <c r="D155" s="53" t="inlineStr">
+      <c r="D155" s="106" t="inlineStr">
         <is>
           <t xml:space="preserve">Tener en cuenta en el ejercicio de estimación y costos la capacidad requerida en infrastructura de Siniestro Integral por el crecimiento en transacciones </t>
         </is>
       </c>
-      <c r="E155" s="54" t="n"/>
-      <c r="F155" s="53">
+      <c r="E155" s="107" t="n"/>
+      <c r="F155" s="106">
         <f>IF($E155="",0,INDEX($M$5:$M$8,MATCH($E155,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G155" s="53">
+      <c r="G155" s="106">
         <f>IF($F155=0,0,$F155/10)</f>
         <v/>
       </c>
-      <c r="H155" s="53">
+      <c r="H155" s="106">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C155,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I155" s="53" t="n"/>
+      <c r="I155" s="106" t="inlineStr">
+        <is>
+          <t>🟥 No estimable como desarrollo: es dimensionamiento de infraestructura de Siniestro Integral por crecimiento transaccional. Necesita el volumen esperado para poder dimensionarse.</t>
+        </is>
+      </c>
     </row>
     <row r="156" ht="30" customHeight="1">
       <c r="A156" s="57" t="inlineStr">
@@ -7407,40 +7822,44 @@
       <c r="I156" s="53" t="n"/>
     </row>
     <row r="157" ht="30" customHeight="1">
-      <c r="A157" s="53" t="inlineStr">
+      <c r="A157" s="106" t="inlineStr">
         <is>
           <t>RT-045</t>
         </is>
       </c>
-      <c r="B157" s="53" t="inlineStr">
+      <c r="B157" s="106" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C157" s="53" t="inlineStr">
+      <c r="C157" s="106" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D157" s="53" t="inlineStr">
+      <c r="D157" s="106" t="inlineStr">
         <is>
           <t>Confirmado: un único web component (Flutter), agnóstico de canal y con funcionalidades diferenciadas por rol (prestador suma 2-3 campos adicionales frente a cliente), embebido en app móvil, Sucursal Virtual Personas y Portal de Prestador/Proveedor — se descarta un front independiente por canal.</t>
         </is>
       </c>
-      <c r="E157" s="54" t="n"/>
-      <c r="F157" s="53">
+      <c r="E157" s="107" t="n"/>
+      <c r="F157" s="106">
         <f>IF($E157="",0,INDEX($M$5:$M$8,MATCH($E157,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G157" s="53">
+      <c r="G157" s="106">
         <f>IF($F157=0,0,$F157/10)</f>
         <v/>
       </c>
-      <c r="H157" s="53">
+      <c r="H157" s="106">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C157,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I157" s="53" t="n"/>
+      <c r="I157" s="106" t="inlineStr">
+        <is>
+          <t>🟥 Mismo conflicto de RT-008: el web component se declara en Flutter y el lineamiento fija Angular sobre Static Web App. La decisión de un único web component agnóstico de canal sí es la del MVP; falta cerrar la tecnología.</t>
+        </is>
+      </c>
     </row>
     <row r="158" ht="30" customHeight="1">
       <c r="A158" s="57" t="inlineStr">
@@ -7515,76 +7934,84 @@
       <c r="I159" s="53" t="n"/>
     </row>
     <row r="160" ht="30" customHeight="1">
-      <c r="A160" s="57" t="inlineStr">
+      <c r="A160" s="105" t="inlineStr">
         <is>
           <t>RT-048</t>
         </is>
       </c>
-      <c r="B160" s="57" t="inlineStr">
+      <c r="B160" s="105" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C160" s="57" t="inlineStr">
+      <c r="C160" s="105" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D160" s="57" t="inlineStr">
+      <c r="D160" s="105" t="inlineStr">
         <is>
           <t>El módulo de interoperabilidad de autorizaciones no parte de cero: reutiliza la infraestructura ya construida de interoperabilidad; se tomará como pivote de esfuerzo el costo de la interoperabilidad de ayudas diagnósticas (la más comparable), reconociendo que autorizaciones tiene casuística y costos propios.</t>
         </is>
       </c>
       <c r="E160" s="54" t="n"/>
-      <c r="F160" s="53">
+      <c r="F160" s="105">
         <f>IF($E160="",0,INDEX($M$5:$M$8,MATCH($E160,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G160" s="53">
+      <c r="G160" s="105">
         <f>IF($F160=0,0,$F160/10)</f>
         <v/>
       </c>
-      <c r="H160" s="53">
+      <c r="H160" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C160,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I160" s="53" t="n"/>
+      <c r="I160" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
+        </is>
+      </c>
     </row>
     <row r="161" ht="30" customHeight="1">
-      <c r="A161" s="53" t="inlineStr">
+      <c r="A161" s="105" t="inlineStr">
         <is>
           <t>RT-049</t>
         </is>
       </c>
-      <c r="B161" s="53" t="inlineStr">
+      <c r="B161" s="105" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C161" s="53" t="inlineStr">
+      <c r="C161" s="105" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D161" s="53" t="inlineStr">
+      <c r="D161" s="105" t="inlineStr">
         <is>
           <t>Se evalúa como insumo de referencia (no de adopción literal) una propuesta de arquitectura agéntica mundial para torres de control de salud, compuesta por 9 agentes especializados (radar, riesgo operacional, capacidad, predictor, director del tráfico, marcos de actuación, anomalías, explicador, recomendación) más un agente “comandante de operaciones” a futuro con capacidad de ejecución directa.</t>
         </is>
       </c>
       <c r="E161" s="54" t="n"/>
-      <c r="F161" s="53">
+      <c r="F161" s="105">
         <f>IF($E161="",0,INDEX($M$5:$M$8,MATCH($E161,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G161" s="53">
+      <c r="G161" s="105">
         <f>IF($F161=0,0,$F161/10)</f>
         <v/>
       </c>
-      <c r="H161" s="53">
+      <c r="H161" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C161,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I161" s="53" t="n"/>
+      <c r="I161" s="105" t="inlineStr">
+        <is>
+          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
+        </is>
+      </c>
     </row>
     <row r="162" ht="30" customHeight="1">
       <c r="A162" s="57" t="inlineStr">
@@ -7627,40 +8054,44 @@
       <c r="I162" s="53" t="n"/>
     </row>
     <row r="163" ht="30" customHeight="1">
-      <c r="A163" s="53" t="inlineStr">
+      <c r="A163" s="106" t="inlineStr">
         <is>
           <t>RT-051</t>
         </is>
       </c>
-      <c r="B163" s="53" t="inlineStr">
+      <c r="B163" s="106" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C163" s="53" t="inlineStr">
+      <c r="C163" s="106" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D163" s="53" t="inlineStr">
+      <c r="D163" s="106" t="inlineStr">
         <is>
           <t>El nivel de autonomía de ejecución de cada agente (recomendar vs. ejecutar) determina directamente con qué sistemas debe conectarse (SuraHis u otros) y qué capacidades técnicas de escritura/ejecución requiere; pendiente de definir antes de dimensionar el desarrollo.</t>
         </is>
       </c>
-      <c r="E163" s="54" t="n"/>
-      <c r="F163" s="53">
+      <c r="E163" s="107" t="n"/>
+      <c r="F163" s="106">
         <f>IF($E163="",0,INDEX($M$5:$M$8,MATCH($E163,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G163" s="53">
+      <c r="G163" s="106">
         <f>IF($F163=0,0,$F163/10)</f>
         <v/>
       </c>
-      <c r="H163" s="53">
+      <c r="H163" s="106">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C163,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I163" s="53" t="n"/>
+      <c r="I163" s="106" t="inlineStr">
+        <is>
+          <t>🟥 El propio requisito dice que el nivel de autonomía de cada agente está «pendiente de definir antes de dimensionar el desarrollo». Se respeta: no se talla hasta que se defina.</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="30" customHeight="1">
       <c r="A164" s="57" t="inlineStr">
@@ -8624,12 +9055,18 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:Q187"/>
-  <mergeCells count="5">
+  <mergeCells count="11">
+    <mergeCell ref="M35:Q35"/>
+    <mergeCell ref="M34:Q34"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="M37:Q37"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="L9:N12"/>
     <mergeCell ref="L13:Q13"/>
+    <mergeCell ref="M33:Q33"/>
+    <mergeCell ref="M36:Q36"/>
     <mergeCell ref="L3:N3"/>
+    <mergeCell ref="M39:Q39"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="E5:E187" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
revierte las observaciones que se salieron del alcance
la instrucción acota la tarea a la columna e y a marcar con color de alerta los
requisitos que no se pueden estimar. escribir por qué queda fuera cada requisito
que no es del mvp no estaba pedido, y además dejaba 68 filas en naranja, con lo
que el color «modificado» dejaba de distinguir nada.

se revierten a su estado original las 61 filas que quedaban fuera del mvp: se
borra la observación y se restaura el relleno. quedan en naranja solo las 7 que
entran al mvp con una salvedad sobre qué cubre la talla.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SURA/gestores-sura/estimacin mvp/2 Gestores_Seguimiento_Requerimientos_2026.xlsx
+++ b/SURA/gestores-sura/estimacin mvp/2 Gestores_Seguimiento_Requerimientos_2026.xlsx
@@ -1522,44 +1522,40 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="105" t="inlineStr">
+      <c r="A10" s="57" t="inlineStr">
         <is>
           <t>RF-006</t>
         </is>
       </c>
-      <c r="B10" s="105" t="inlineStr">
+      <c r="B10" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C10" s="105" t="inlineStr">
+      <c r="C10" s="57" t="inlineStr">
         <is>
           <t>Canales / Front Externos</t>
         </is>
       </c>
-      <c r="D10" s="105" t="inlineStr">
+      <c r="D10" s="57" t="inlineStr">
         <is>
           <t>Rescate digital automático: si falla el canal al radicar, se contacta tibbot desde el canal</t>
         </is>
       </c>
       <c r="E10" s="54" t="n"/>
-      <c r="F10" s="105">
+      <c r="F10" s="53">
         <f>IF($E10="",0,INDEX($M$5:$M$8,MATCH($E10,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G10" s="105">
+      <c r="G10" s="53">
         <f>IF($F10=0,0,$F10/10)</f>
         <v/>
       </c>
-      <c r="H10" s="105">
+      <c r="H10" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C10,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I10" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el rescate con contacto proactivo desde el canal es capacidad proactiva de la torre (capa 4), que no entra.</t>
-        </is>
-      </c>
+      <c r="I10" s="53" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="53" t="inlineStr">
@@ -2101,44 +2097,40 @@
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="105" t="inlineStr">
+      <c r="A20" s="57" t="inlineStr">
         <is>
           <t>RF-016</t>
         </is>
       </c>
-      <c r="B20" s="105" t="inlineStr">
+      <c r="B20" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C20" s="105" t="inlineStr">
+      <c r="C20" s="57" t="inlineStr">
         <is>
           <t>Surahis</t>
         </is>
       </c>
-      <c r="D20" s="105" t="inlineStr">
+      <c r="D20" s="57" t="inlineStr">
         <is>
           <t>Se debe activar la Integralidad automática con EPS Sura cuando la póliza voluntaria no cubre el servicio y se genera la negación de una solicitud (régimen contributivo activo).</t>
         </is>
       </c>
       <c r="E20" s="54" t="n"/>
-      <c r="F20" s="105">
+      <c r="F20" s="53">
         <f>IF($E20="",0,INDEX($M$5:$M$8,MATCH($E20,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G20" s="105">
+      <c r="G20" s="53">
         <f>IF($F20=0,0,$F20/10)</f>
         <v/>
       </c>
-      <c r="H20" s="105">
+      <c r="H20" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C20,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I20" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del alcance de Gestores: la integralidad automática con EPS Sura es trabajo del core, y la épica está marcada N/A en esta misma hoja.</t>
-        </is>
-      </c>
+      <c r="I20" s="53" t="n"/>
       <c r="L20" s="60" t="inlineStr">
         <is>
           <t>Canales / Front Externos</t>
@@ -2169,44 +2161,40 @@
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="105" t="inlineStr">
+      <c r="A21" s="53" t="inlineStr">
         <is>
           <t>RF-017</t>
         </is>
       </c>
-      <c r="B21" s="105" t="inlineStr">
+      <c r="B21" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C21" s="105" t="inlineStr">
+      <c r="C21" s="53" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D21" s="105" t="inlineStr">
+      <c r="D21" s="53" t="inlineStr">
         <is>
           <t>Se debe habilitar la opción de "Reestudio": permite solicitar una reevaluación de una solicitud negada adjuntando nueva evidencia u observaciones, se debe conservar el mismo número de solicitud padre y se debe enviar al core con el mismo evaluador de la solicitud inicial.</t>
         </is>
       </c>
       <c r="E21" s="54" t="n"/>
-      <c r="F21" s="105">
+      <c r="F21" s="53">
         <f>IF($E21="",0,INDEX($M$5:$M$8,MATCH($E21,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G21" s="105">
+      <c r="G21" s="53">
         <f>IF($F21=0,0,$F21/10)</f>
         <v/>
       </c>
-      <c r="H21" s="105">
+      <c r="H21" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C21,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I21" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el reestudio no aparece en el dibujo. Es un flujo adicional sobre una solicitud ya negada.</t>
-        </is>
-      </c>
+      <c r="I21" s="53" t="n"/>
       <c r="L21" s="60" t="inlineStr">
         <is>
           <t>Transversal / Principios generales</t>
@@ -2305,44 +2293,40 @@
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="105" t="inlineStr">
+      <c r="A23" s="53" t="inlineStr">
         <is>
           <t>RF-019</t>
         </is>
       </c>
-      <c r="B23" s="105" t="inlineStr">
+      <c r="B23" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C23" s="105" t="inlineStr">
+      <c r="C23" s="53" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D23" s="105" t="inlineStr">
+      <c r="D23" s="53" t="inlineStr">
         <is>
           <t>Se debe incorporar como requisito funcional el "rescate de la solicitud" cuando la radicación no se concluye, sin importar en qué paso quedó.</t>
         </is>
       </c>
       <c r="E23" s="54" t="n"/>
-      <c r="F23" s="105">
+      <c r="F23" s="53">
         <f>IF($E23="",0,INDEX($M$5:$M$8,MATCH($E23,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G23" s="105">
+      <c r="G23" s="53">
         <f>IF($F23=0,0,$F23/10)</f>
         <v/>
       </c>
-      <c r="H23" s="105">
+      <c r="H23" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C23,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I23" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el rescate de la radicación incompleta no aparece en el dibujo.</t>
-        </is>
-      </c>
+      <c r="I23" s="53" t="n"/>
       <c r="L23" s="60" t="inlineStr">
         <is>
           <t>Siniestro Integral</t>
@@ -2962,44 +2946,40 @@
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="105" t="inlineStr">
+      <c r="A34" s="57" t="inlineStr">
         <is>
           <t>RF-030</t>
         </is>
       </c>
-      <c r="B34" s="105" t="inlineStr">
+      <c r="B34" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C34" s="105" t="inlineStr">
+      <c r="C34" s="57" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
-      <c r="D34" s="105" t="inlineStr">
+      <c r="D34" s="57" t="inlineStr">
         <is>
           <t>La asignación al equipo se distribuye según reglas de criticidad (marcas en salud, PEP, edad del asegurado, urgencia, quejas/tutelas, diagnósticos de riesgo) entre evaluadores disponibles por nivel.</t>
         </is>
       </c>
       <c r="E34" s="54" t="n"/>
-      <c r="F34" s="105">
+      <c r="F34" s="53">
         <f>IF($E34="",0,INDEX($M$5:$M$8,MATCH($E34,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G34" s="105">
+      <c r="G34" s="53">
         <f>IF($F34=0,0,$F34/10)</f>
         <v/>
       </c>
-      <c r="H34" s="105">
+      <c r="H34" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C34,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I34" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye un Gestor de Asignación. La escalada a evaluación humana entra a la bandeja del core.</t>
-        </is>
-      </c>
+      <c r="I34" s="53" t="n"/>
       <c r="L34" s="111" t="inlineStr">
         <is>
           <t>Fila modificada</t>
@@ -3012,44 +2992,40 @@
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="105" t="inlineStr">
+      <c r="A35" s="53" t="inlineStr">
         <is>
           <t>RF-031</t>
         </is>
       </c>
-      <c r="B35" s="105" t="inlineStr">
+      <c r="B35" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C35" s="105" t="inlineStr">
+      <c r="C35" s="53" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
-      <c r="D35" s="105" t="inlineStr">
+      <c r="D35" s="53" t="inlineStr">
         <is>
           <t>Para solicitudes pendientes por gestión se habilita la reasignación entre niveles.</t>
         </is>
       </c>
       <c r="E35" s="54" t="n"/>
-      <c r="F35" s="105">
+      <c r="F35" s="53">
         <f>IF($E35="",0,INDEX($M$5:$M$8,MATCH($E35,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G35" s="105">
+      <c r="G35" s="53">
         <f>IF($F35=0,0,$F35/10)</f>
         <v/>
       </c>
-      <c r="H35" s="105">
+      <c r="H35" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C35,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I35" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye un Gestor de Asignación. La escalada a evaluación humana entra a la bandeja del core.</t>
-        </is>
-      </c>
+      <c r="I35" s="53" t="n"/>
       <c r="L35" s="112" t="inlineStr">
         <is>
           <t>Alerta · sin tallar</t>
@@ -3062,44 +3038,40 @@
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="105" t="inlineStr">
+      <c r="A36" s="57" t="inlineStr">
         <is>
           <t>RF-032</t>
         </is>
       </c>
-      <c r="B36" s="105" t="inlineStr">
+      <c r="B36" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C36" s="105" t="inlineStr">
+      <c r="C36" s="57" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
-      <c r="D36" s="105" t="inlineStr">
+      <c r="D36" s="57" t="inlineStr">
         <is>
           <t>Cada solicitud debe tener un tiempo de respuesta asignado (100% de las solicitudes en menos de 24 horas).</t>
         </is>
       </c>
       <c r="E36" s="54" t="n"/>
-      <c r="F36" s="105">
+      <c r="F36" s="53">
         <f>IF($E36="",0,INDEX($M$5:$M$8,MATCH($E36,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G36" s="105">
+      <c r="G36" s="53">
         <f>IF($F36=0,0,$F36/10)</f>
         <v/>
       </c>
-      <c r="H36" s="105">
+      <c r="H36" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C36,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I36" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye un Gestor de Asignación. La escalada a evaluación humana entra a la bandeja del core.</t>
-        </is>
-      </c>
+      <c r="I36" s="53" t="n"/>
       <c r="L36" s="113" t="inlineStr">
         <is>
           <t>Talla diligenciada</t>
@@ -3112,44 +3084,40 @@
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="105" t="inlineStr">
+      <c r="A37" s="53" t="inlineStr">
         <is>
           <t>RF-033</t>
         </is>
       </c>
-      <c r="B37" s="105" t="inlineStr">
+      <c r="B37" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C37" s="105" t="inlineStr">
+      <c r="C37" s="53" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
-      <c r="D37" s="105" t="inlineStr">
+      <c r="D37" s="53" t="inlineStr">
         <is>
           <t>Se debe notificar al asegurado cuando se identifique en el proceso de evaluación manual que se requiere un documento adicional para entregar una decisión en la evaluación, esta notificación debe incluir el enlace de la SVP o APP para que el asegurado cargue el requisito pendiente</t>
         </is>
       </c>
       <c r="E37" s="54" t="n"/>
-      <c r="F37" s="105">
+      <c r="F37" s="53">
         <f>IF($E37="",0,INDEX($M$5:$M$8,MATCH($E37,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G37" s="105">
+      <c r="G37" s="53">
         <f>IF($F37=0,0,$F37/10)</f>
         <v/>
       </c>
-      <c r="H37" s="105">
+      <c r="H37" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C37,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I37" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye un Gestor de Asignación. La escalada a evaluación humana entra a la bandeja del core.</t>
-        </is>
-      </c>
+      <c r="I37" s="53" t="n"/>
       <c r="L37" s="114" t="inlineStr">
         <is>
           <t>Sin color y sin talla</t>
@@ -3162,84 +3130,76 @@
       </c>
     </row>
     <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="105" t="inlineStr">
+      <c r="A38" s="57" t="inlineStr">
         <is>
           <t>RF-034</t>
         </is>
       </c>
-      <c r="B38" s="105" t="inlineStr">
+      <c r="B38" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C38" s="105" t="inlineStr">
+      <c r="C38" s="57" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
-      <c r="D38" s="105" t="inlineStr">
+      <c r="D38" s="57" t="inlineStr">
         <is>
           <t>Cuando el asegurado cargue el requisito pendiente, esta solicitud se debe encolar nuevamente en la bandeja manual en surahis y se debe asignar al mismo evaluador y con un tiempo de respuesta prioritario</t>
         </is>
       </c>
       <c r="E38" s="54" t="n"/>
-      <c r="F38" s="105">
+      <c r="F38" s="53">
         <f>IF($E38="",0,INDEX($M$5:$M$8,MATCH($E38,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G38" s="105">
+      <c r="G38" s="53">
         <f>IF($F38=0,0,$F38/10)</f>
         <v/>
       </c>
-      <c r="H38" s="105">
+      <c r="H38" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C38,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I38" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye un Gestor de Asignación. La escalada a evaluación humana entra a la bandeja del core.</t>
-        </is>
-      </c>
+      <c r="I38" s="53" t="n"/>
     </row>
     <row r="39" ht="60" customHeight="1">
-      <c r="A39" s="105" t="inlineStr">
+      <c r="A39" s="53" t="inlineStr">
         <is>
           <t>RF-035</t>
         </is>
       </c>
-      <c r="B39" s="105" t="inlineStr">
+      <c r="B39" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C39" s="105" t="inlineStr">
+      <c r="C39" s="53" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
-      <c r="D39" s="105" t="inlineStr">
+      <c r="D39" s="53" t="inlineStr">
         <is>
           <t>Con la negación de un servicio se debe activar la radicación automática de la solicitud de integralidad a EPS Sura en el aplicativo salud web</t>
         </is>
       </c>
       <c r="E39" s="54" t="n"/>
-      <c r="F39" s="105">
+      <c r="F39" s="53">
         <f>IF($E39="",0,INDEX($M$5:$M$8,MATCH($E39,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G39" s="105">
+      <c r="G39" s="53">
         <f>IF($F39=0,0,$F39/10)</f>
         <v/>
       </c>
-      <c r="H39" s="105">
+      <c r="H39" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C39,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I39" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye un Gestor de Asignación. La escalada a evaluación humana entra a la bandeja del core.</t>
-        </is>
-      </c>
+      <c r="I39" s="53" t="n"/>
       <c r="L39" s="114" t="inlineStr">
         <is>
           <t>Criterio de alcance</t>
@@ -3252,84 +3212,76 @@
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="105" t="inlineStr">
+      <c r="A40" s="57" t="inlineStr">
         <is>
           <t>RF-036</t>
         </is>
       </c>
-      <c r="B40" s="105" t="inlineStr">
+      <c r="B40" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C40" s="105" t="inlineStr">
+      <c r="C40" s="57" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
-      <c r="D40" s="105" t="inlineStr">
+      <c r="D40" s="57" t="inlineStr">
         <is>
           <t>Surahis publica un evento con el cambio de estado de la solicitud de integralidad en salud web y con este evento se alimenta la torre de control y se actualiza el estado en los canales (Front)</t>
         </is>
       </c>
       <c r="E40" s="54" t="n"/>
-      <c r="F40" s="105">
+      <c r="F40" s="53">
         <f>IF($E40="",0,INDEX($M$5:$M$8,MATCH($E40,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G40" s="105">
+      <c r="G40" s="53">
         <f>IF($F40=0,0,$F40/10)</f>
         <v/>
       </c>
-      <c r="H40" s="105">
+      <c r="H40" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C40,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I40" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye un Gestor de Asignación. La escalada a evaluación humana entra a la bandeja del core.</t>
-        </is>
-      </c>
+      <c r="I40" s="53" t="n"/>
     </row>
     <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="105" t="inlineStr">
+      <c r="A41" s="53" t="inlineStr">
         <is>
           <t>RF-037</t>
         </is>
       </c>
-      <c r="B41" s="105" t="inlineStr">
+      <c r="B41" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C41" s="105" t="inlineStr">
+      <c r="C41" s="53" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
         </is>
       </c>
-      <c r="D41" s="105" t="inlineStr">
+      <c r="D41" s="53" t="inlineStr">
         <is>
           <t>Se debe habilitar la opción de resignación manual de solicitudes a otro evaluador (novedades con el evaluador asignado inicialmente).</t>
         </is>
       </c>
       <c r="E41" s="54" t="n"/>
-      <c r="F41" s="105">
+      <c r="F41" s="53">
         <f>IF($E41="",0,INDEX($M$5:$M$8,MATCH($E41,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G41" s="105">
+      <c r="G41" s="53">
         <f>IF($F41=0,0,$F41/10)</f>
         <v/>
       </c>
-      <c r="H41" s="105">
+      <c r="H41" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C41,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I41" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye un Gestor de Asignación. La escalada a evaluación humana entra a la bandeja del core.</t>
-        </is>
-      </c>
+      <c r="I41" s="53" t="n"/>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="57" t="inlineStr">
@@ -3738,44 +3690,40 @@
       <c r="I52" s="53" t="n"/>
     </row>
     <row r="53" ht="30" customHeight="1">
-      <c r="A53" s="105" t="inlineStr">
+      <c r="A53" s="53" t="inlineStr">
         <is>
           <t>RF-049</t>
         </is>
       </c>
-      <c r="B53" s="105" t="inlineStr">
+      <c r="B53" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C53" s="105" t="inlineStr">
+      <c r="C53" s="53" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D53" s="105" t="inlineStr">
+      <c r="D53" s="53" t="inlineStr">
         <is>
           <t>Monitorea el ciclo de vida completo de la solicitud: cumplimiento de SLA/ANS (semaforos que indiquen posible incumplimiento), carga de trabajo, trazabilidad,capacidad y riesgo acumulado del ciclo.</t>
         </is>
       </c>
       <c r="E53" s="54" t="n"/>
-      <c r="F53" s="105">
+      <c r="F53" s="53">
         <f>IF($E53="",0,INDEX($M$5:$M$8,MATCH($E53,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G53" s="105">
+      <c r="G53" s="53">
         <f>IF($F53=0,0,$F53/10)</f>
         <v/>
       </c>
-      <c r="H53" s="105">
+      <c r="H53" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C53,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I53" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I53" s="53" t="n"/>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="57" t="inlineStr">
@@ -3818,124 +3766,112 @@
       <c r="I54" s="53" t="n"/>
     </row>
     <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="105" t="inlineStr">
+      <c r="A55" s="53" t="inlineStr">
         <is>
           <t>RF-051</t>
         </is>
       </c>
-      <c r="B55" s="105" t="inlineStr">
+      <c r="B55" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C55" s="105" t="inlineStr">
+      <c r="C55" s="53" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D55" s="105" t="inlineStr">
+      <c r="D55" s="53" t="inlineStr">
         <is>
           <t>Capacidades proactivas (contactar directamente al cliente/prestador/asesor) emite notificaciones en 3 dimensiones (actor, canal, proactivo/pasivo), ejemplo: asegurado ante el incumplimiento de un SLA para dar tranquilidad de la gestión de la solicitud y alerta internamente a evaluadores/líderes por casos por vencer o desborde de capacidad, apertura de autorización, autorización en evaluación, autorización aprobada, etc.</t>
         </is>
       </c>
       <c r="E55" s="54" t="n"/>
-      <c r="F55" s="105">
+      <c r="F55" s="53">
         <f>IF($E55="",0,INDEX($M$5:$M$8,MATCH($E55,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G55" s="105">
+      <c r="G55" s="53">
         <f>IF($F55=0,0,$F55/10)</f>
         <v/>
       </c>
-      <c r="H55" s="105">
+      <c r="H55" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C55,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I55" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I55" s="53" t="n"/>
     </row>
     <row r="56" ht="30" customHeight="1">
-      <c r="A56" s="105" t="inlineStr">
+      <c r="A56" s="57" t="inlineStr">
         <is>
           <t>RF-052</t>
         </is>
       </c>
-      <c r="B56" s="105" t="inlineStr">
+      <c r="B56" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C56" s="105" t="inlineStr">
+      <c r="C56" s="57" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D56" s="105" t="inlineStr">
+      <c r="D56" s="57" t="inlineStr">
         <is>
           <t>Capacidad de intervenir otros gestores cuando se detecte algún comportamiento insual en la solicitud</t>
         </is>
       </c>
       <c r="E56" s="54" t="n"/>
-      <c r="F56" s="105">
+      <c r="F56" s="53">
         <f>IF($E56="",0,INDEX($M$5:$M$8,MATCH($E56,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G56" s="105">
+      <c r="G56" s="53">
         <f>IF($F56=0,0,$F56/10)</f>
         <v/>
       </c>
-      <c r="H56" s="105">
+      <c r="H56" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C56,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I56" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I56" s="53" t="n"/>
     </row>
     <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="105" t="inlineStr">
+      <c r="A57" s="53" t="inlineStr">
         <is>
           <t>RF-053</t>
         </is>
       </c>
-      <c r="B57" s="105" t="inlineStr">
+      <c r="B57" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C57" s="105" t="inlineStr">
+      <c r="C57" s="53" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D57" s="105" t="inlineStr">
+      <c r="D57" s="53" t="inlineStr">
         <is>
           <t>Indicador en la torre de control para visualización de los siniestros duplicados ingresados por el prestador que sean para el mismo</t>
         </is>
       </c>
       <c r="E57" s="54" t="n"/>
-      <c r="F57" s="105">
+      <c r="F57" s="53">
         <f>IF($E57="",0,INDEX($M$5:$M$8,MATCH($E57,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G57" s="105">
+      <c r="G57" s="53">
         <f>IF($F57=0,0,$F57/10)</f>
         <v/>
       </c>
-      <c r="H57" s="105">
+      <c r="H57" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C57,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I57" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I57" s="53" t="n"/>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="105" t="inlineStr">
@@ -3982,84 +3918,76 @@
       </c>
     </row>
     <row r="59" ht="30" customHeight="1">
-      <c r="A59" s="105" t="inlineStr">
+      <c r="A59" s="53" t="inlineStr">
         <is>
           <t>RF-055</t>
         </is>
       </c>
-      <c r="B59" s="105" t="inlineStr">
+      <c r="B59" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C59" s="105" t="inlineStr">
+      <c r="C59" s="53" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D59" s="105" t="inlineStr">
+      <c r="D59" s="53" t="inlineStr">
         <is>
           <t>Expone información distinta según el actor consultante (prestador, cliente, asesor), enmascarando datos sensibles.</t>
         </is>
       </c>
       <c r="E59" s="54" t="n"/>
-      <c r="F59" s="105">
+      <c r="F59" s="53">
         <f>IF($E59="",0,INDEX($M$5:$M$8,MATCH($E59,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G59" s="105">
+      <c r="G59" s="53">
         <f>IF($F59=0,0,$F59/10)</f>
         <v/>
       </c>
-      <c r="H59" s="105">
+      <c r="H59" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C59,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I59" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I59" s="53" t="n"/>
     </row>
     <row r="60" ht="30" customHeight="1">
-      <c r="A60" s="105" t="inlineStr">
+      <c r="A60" s="57" t="inlineStr">
         <is>
           <t>RF-056</t>
         </is>
       </c>
-      <c r="B60" s="105" t="inlineStr">
+      <c r="B60" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C60" s="105" t="inlineStr">
+      <c r="C60" s="57" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D60" s="105" t="inlineStr">
+      <c r="D60" s="57" t="inlineStr">
         <is>
           <t>Se requiere una vista que nos permita realizar la auditoria de toda la trazabilidad de las solicitudes</t>
         </is>
       </c>
       <c r="E60" s="54" t="n"/>
-      <c r="F60" s="105">
+      <c r="F60" s="53">
         <f>IF($E60="",0,INDEX($M$5:$M$8,MATCH($E60,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G60" s="105">
+      <c r="G60" s="53">
         <f>IF($F60=0,0,$F60/10)</f>
         <v/>
       </c>
-      <c r="H60" s="105">
+      <c r="H60" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C60,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I60" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I60" s="53" t="n"/>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="53" t="inlineStr">
@@ -4146,244 +4074,220 @@
       </c>
     </row>
     <row r="63" ht="30" customHeight="1">
-      <c r="A63" s="105" t="inlineStr">
+      <c r="A63" s="53" t="inlineStr">
         <is>
           <t>RF-059</t>
         </is>
       </c>
-      <c r="B63" s="105" t="inlineStr">
+      <c r="B63" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C63" s="105" t="inlineStr">
+      <c r="C63" s="53" t="inlineStr">
         <is>
           <t>Canales / Front Externos</t>
         </is>
       </c>
-      <c r="D63" s="105" t="inlineStr">
+      <c r="D63" s="53" t="inlineStr">
         <is>
           <t>El cliente debe recibir notificación automática cuando un prestador radica una solicitud en su nombre, con visibilidad completa del caso sin importar el canal de radicación (evita duplicados).</t>
         </is>
       </c>
       <c r="E63" s="54" t="n"/>
-      <c r="F63" s="105">
+      <c r="F63" s="53">
         <f>IF($E63="",0,INDEX($M$5:$M$8,MATCH($E63,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G63" s="105">
+      <c r="G63" s="53">
         <f>IF($F63=0,0,$F63/10)</f>
         <v/>
       </c>
-      <c r="H63" s="105">
+      <c r="H63" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C63,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I63" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: la notificación automática al cliente es capa de exposición de la torre, que no entra.</t>
-        </is>
-      </c>
+      <c r="I63" s="53" t="n"/>
     </row>
     <row r="64" ht="30" customHeight="1">
-      <c r="A64" s="105" t="inlineStr">
+      <c r="A64" s="57" t="inlineStr">
         <is>
           <t>RF-060</t>
         </is>
       </c>
-      <c r="B64" s="105" t="inlineStr">
+      <c r="B64" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C64" s="105" t="inlineStr">
+      <c r="C64" s="57" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D64" s="105" t="inlineStr">
+      <c r="D64" s="57" t="inlineStr">
         <is>
           <t>El Gestor de Prestación no requiere capacidad agéntica para la confirmación de atención; la integración se conecta directo entre Super App/interoperabilidad y el Core (SuraHis), sin crear un componente nuevo en Gestores.</t>
         </is>
       </c>
       <c r="E64" s="54" t="n"/>
-      <c r="F64" s="105">
+      <c r="F64" s="53">
         <f>IF($E64="",0,INDEX($M$5:$M$8,MATCH($E64,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G64" s="105">
+      <c r="G64" s="53">
         <f>IF($F64=0,0,$F64/10)</f>
         <v/>
       </c>
-      <c r="H64" s="105">
+      <c r="H64" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C64,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I64" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I64" s="53" t="n"/>
     </row>
     <row r="65" ht="30" customHeight="1">
-      <c r="A65" s="105" t="inlineStr">
+      <c r="A65" s="53" t="inlineStr">
         <is>
           <t>RF-061</t>
         </is>
       </c>
-      <c r="B65" s="105" t="inlineStr">
+      <c r="B65" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C65" s="105" t="inlineStr">
+      <c r="C65" s="53" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D65" s="105" t="inlineStr">
+      <c r="D65" s="53" t="inlineStr">
         <is>
           <t>La interoperabilidad administrativa de autorizaciones está en construcción por el equipo de Interoperabilidad (Sergio "Checho" Pérez) junto con el equipo de autorizaciones y pólizas; no alcanza a cerrarse antes del cierre de estructuración.</t>
         </is>
       </c>
       <c r="E65" s="54" t="n"/>
-      <c r="F65" s="105">
+      <c r="F65" s="53">
         <f>IF($E65="",0,INDEX($M$5:$M$8,MATCH($E65,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G65" s="105">
+      <c r="G65" s="53">
         <f>IF($F65=0,0,$F65/10)</f>
         <v/>
       </c>
-      <c r="H65" s="105">
+      <c r="H65" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C65,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I65" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I65" s="53" t="n"/>
     </row>
     <row r="66" ht="30" customHeight="1">
-      <c r="A66" s="105" t="inlineStr">
+      <c r="A66" s="57" t="inlineStr">
         <is>
           <t>RF-062</t>
         </is>
       </c>
-      <c r="B66" s="105" t="inlineStr">
+      <c r="B66" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C66" s="105" t="inlineStr">
+      <c r="C66" s="57" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D66" s="105" t="inlineStr">
+      <c r="D66" s="57" t="inlineStr">
         <is>
           <t>Hoy existen ~12 software de interoperabilidad habilitados con prestadores (incluye Himed/proveedor Pareto, Salud Tools, Servintech), con datos de institución/médico tratante, fecha y tipo/motivo de consulta.</t>
         </is>
       </c>
       <c r="E66" s="54" t="n"/>
-      <c r="F66" s="105">
+      <c r="F66" s="53">
         <f>IF($E66="",0,INDEX($M$5:$M$8,MATCH($E66,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G66" s="105">
+      <c r="G66" s="53">
         <f>IF($F66=0,0,$F66/10)</f>
         <v/>
       </c>
-      <c r="H66" s="105">
+      <c r="H66" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C66,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I66" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I66" s="53" t="n"/>
     </row>
     <row r="67" ht="30" customHeight="1">
-      <c r="A67" s="105" t="inlineStr">
+      <c r="A67" s="53" t="inlineStr">
         <is>
           <t>RF-063</t>
         </is>
       </c>
-      <c r="B67" s="105" t="inlineStr">
+      <c r="B67" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C67" s="105" t="inlineStr">
+      <c r="C67" s="53" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D67" s="105" t="inlineStr">
+      <c r="D67" s="53" t="inlineStr">
         <is>
           <t>No debe agendarse ninguna cita de forma automática sin el consentimiento explícito del asegurado (el sistema sugiere las citas disponibles y confirma con el asegurado antes de agendar).</t>
         </is>
       </c>
       <c r="E67" s="54" t="n"/>
-      <c r="F67" s="105">
+      <c r="F67" s="53">
         <f>IF($E67="",0,INDEX($M$5:$M$8,MATCH($E67,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G67" s="105">
+      <c r="G67" s="53">
         <f>IF($F67=0,0,$F67/10)</f>
         <v/>
       </c>
-      <c r="H67" s="105">
+      <c r="H67" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C67,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I67" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I67" s="53" t="n"/>
     </row>
     <row r="68" ht="30" customHeight="1">
-      <c r="A68" s="105" t="inlineStr">
+      <c r="A68" s="57" t="inlineStr">
         <is>
           <t>RF-064</t>
         </is>
       </c>
-      <c r="B68" s="105" t="inlineStr">
+      <c r="B68" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C68" s="105" t="inlineStr">
+      <c r="C68" s="57" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D68" s="105" t="inlineStr">
+      <c r="D68" s="57" t="inlineStr">
         <is>
           <t>¿Cómo se cierra la brecha de confirmación de atención para prestación externa (~60-70% de la población)? SuraHis resolvería el gap interno, pero no está claro que resuelva el externo.</t>
         </is>
       </c>
       <c r="E68" s="54" t="n"/>
-      <c r="F68" s="105">
+      <c r="F68" s="53">
         <f>IF($E68="",0,INDEX($M$5:$M$8,MATCH($E68,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G68" s="105">
+      <c r="G68" s="53">
         <f>IF($F68=0,0,$F68/10)</f>
         <v/>
       </c>
-      <c r="H68" s="105">
+      <c r="H68" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C68,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I68" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I68" s="53" t="n"/>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="53" t="inlineStr">
@@ -4610,164 +4514,148 @@
       </c>
     </row>
     <row r="75" ht="30" customHeight="1">
-      <c r="A75" s="105" t="inlineStr">
+      <c r="A75" s="53" t="inlineStr">
         <is>
           <t>RF-071</t>
         </is>
       </c>
-      <c r="B75" s="105" t="inlineStr">
+      <c r="B75" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C75" s="105" t="inlineStr">
+      <c r="C75" s="53" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D75" s="105" t="inlineStr">
+      <c r="D75" s="53" t="inlineStr">
         <is>
           <t>Se definen 5 momentos de integración con Interoperabilidad: (1) solicitud/consulta de historia clínica, (2) envío de la autorización al prestador, (3) confirmación de la atención/prestación, (4) recepción de nuevas órdenes o autorizaciones que surjan durante la atención (ej. exámenes adicionales), (5) agenda disponible en el prestador para atención de un servicio</t>
         </is>
       </c>
       <c r="E75" s="54" t="n"/>
-      <c r="F75" s="105">
+      <c r="F75" s="53">
         <f>IF($E75="",0,INDEX($M$5:$M$8,MATCH($E75,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G75" s="105">
+      <c r="G75" s="53">
         <f>IF($F75=0,0,$F75/10)</f>
         <v/>
       </c>
-      <c r="H75" s="105">
+      <c r="H75" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C75,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I75" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I75" s="53" t="n"/>
     </row>
     <row r="76" ht="30" customHeight="1">
-      <c r="A76" s="105" t="inlineStr">
+      <c r="A76" s="57" t="inlineStr">
         <is>
           <t>RF-072</t>
         </is>
       </c>
-      <c r="B76" s="105" t="inlineStr">
+      <c r="B76" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C76" s="105" t="inlineStr">
+      <c r="C76" s="57" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D76" s="105" t="inlineStr">
+      <c r="D76" s="57" t="inlineStr">
         <is>
           <t>El estándar de referencia para el intercambio de información clínica es el RDA (Resumen Digital de Atención), alineado con FHIR/HL7 y con la normativa colombiana vigente.</t>
         </is>
       </c>
       <c r="E76" s="54" t="n"/>
-      <c r="F76" s="105">
+      <c r="F76" s="53">
         <f>IF($E76="",0,INDEX($M$5:$M$8,MATCH($E76,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G76" s="105">
+      <c r="G76" s="53">
         <f>IF($F76=0,0,$F76/10)</f>
         <v/>
       </c>
-      <c r="H76" s="105">
+      <c r="H76" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C76,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I76" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I76" s="53" t="n"/>
     </row>
     <row r="77" ht="30" customHeight="1">
-      <c r="A77" s="105" t="inlineStr">
+      <c r="A77" s="53" t="inlineStr">
         <is>
           <t>RF-073</t>
         </is>
       </c>
-      <c r="B77" s="105" t="inlineStr">
+      <c r="B77" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C77" s="105" t="inlineStr">
+      <c r="C77" s="53" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D77" s="105" t="inlineStr">
+      <c r="D77" s="53" t="inlineStr">
         <is>
           <t>Se solicitará al equipo de Interoperabilidad que su primer entregable/release sean los contratos de API (aunque la solución completa no esté lista), para que Gestores pueda construir e integrar desde ya contra un contrato estable.</t>
         </is>
       </c>
       <c r="E77" s="54" t="n"/>
-      <c r="F77" s="105">
+      <c r="F77" s="53">
         <f>IF($E77="",0,INDEX($M$5:$M$8,MATCH($E77,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G77" s="105">
+      <c r="G77" s="53">
         <f>IF($F77=0,0,$F77/10)</f>
         <v/>
       </c>
-      <c r="H77" s="105">
+      <c r="H77" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C77,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I77" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I77" s="53" t="n"/>
     </row>
     <row r="78" ht="30" customHeight="1">
-      <c r="A78" s="105" t="inlineStr">
+      <c r="A78" s="57" t="inlineStr">
         <is>
           <t>RF-074</t>
         </is>
       </c>
-      <c r="B78" s="105" t="inlineStr">
+      <c r="B78" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C78" s="105" t="inlineStr">
+      <c r="C78" s="57" t="inlineStr">
         <is>
           <t>Canales / Front Externos</t>
         </is>
       </c>
-      <c r="D78" s="105" t="inlineStr">
+      <c r="D78" s="57" t="inlineStr">
         <is>
           <t>La SVP (y en general los canales de cliente) deben permitir editar/cambiar el prestador asignado en la autorización, dentro de un tiempo máximo definido; superado ese tiempo, se confirma automáticamente el prestador por defecto.</t>
         </is>
       </c>
       <c r="E78" s="54" t="n"/>
-      <c r="F78" s="105">
+      <c r="F78" s="53">
         <f>IF($E78="",0,INDEX($M$5:$M$8,MATCH($E78,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G78" s="105">
+      <c r="G78" s="53">
         <f>IF($F78=0,0,$F78/10)</f>
         <v/>
       </c>
-      <c r="H78" s="105">
+      <c r="H78" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C78,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I78" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: editar el prestador asignado depende del Gestor de Coordinación, que queda fuera.</t>
-        </is>
-      </c>
+      <c r="I78" s="53" t="n"/>
     </row>
     <row r="79" ht="30" customHeight="1">
       <c r="A79" s="53" t="inlineStr">
@@ -4806,44 +4694,40 @@
       <c r="I79" s="53" t="n"/>
     </row>
     <row r="80" ht="30" customHeight="1">
-      <c r="A80" s="105" t="inlineStr">
+      <c r="A80" s="57" t="inlineStr">
         <is>
           <t>RF-076</t>
         </is>
       </c>
-      <c r="B80" s="105" t="inlineStr">
+      <c r="B80" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C80" s="105" t="inlineStr">
+      <c r="C80" s="57" t="inlineStr">
         <is>
           <t>Transversal</t>
         </is>
       </c>
-      <c r="D80" s="105" t="inlineStr">
+      <c r="D80" s="57" t="inlineStr">
         <is>
           <t>si la libre elección de prestador aplica solo a pólizas Salud Global o a todo el portafolio (excepto modular). Es "muy importante" porque si cambia, impacta todo el portafolio.</t>
         </is>
       </c>
       <c r="E80" s="54" t="n"/>
-      <c r="F80" s="105">
+      <c r="F80" s="53">
         <f>IF($E80="",0,INDEX($M$5:$M$8,MATCH($E80,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G80" s="105">
+      <c r="G80" s="53">
         <f>IF($F80=0,0,$F80/10)</f>
         <v/>
       </c>
-      <c r="H80" s="105">
+      <c r="H80" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C80,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I80" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: la libre elección de prestador es del Gestor de Coordinación, que queda fuera.</t>
-        </is>
-      </c>
+      <c r="I80" s="53" t="n"/>
     </row>
     <row r="81" ht="30" customHeight="1">
       <c r="A81" s="106" t="inlineStr">
@@ -4886,324 +4770,292 @@
       </c>
     </row>
     <row r="82" ht="30" customHeight="1">
-      <c r="A82" s="105" t="inlineStr">
+      <c r="A82" s="57" t="inlineStr">
         <is>
           <t>RF-078</t>
         </is>
       </c>
-      <c r="B82" s="105" t="inlineStr">
+      <c r="B82" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C82" s="105" t="inlineStr">
+      <c r="C82" s="57" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D82" s="105" t="inlineStr">
+      <c r="D82" s="57" t="inlineStr">
         <is>
           <t>falta decidir el modelo operativo único entre 3 opciones (vía interoperabilidad cuando esté lista, que el prestador que generó la orden asuma el costo operativo, o que se le entregue el papeleo al cliente).</t>
         </is>
       </c>
       <c r="E82" s="54" t="n"/>
-      <c r="F82" s="105">
+      <c r="F82" s="53">
         <f>IF($E82="",0,INDEX($M$5:$M$8,MATCH($E82,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G82" s="105">
+      <c r="G82" s="53">
         <f>IF($F82=0,0,$F82/10)</f>
         <v/>
       </c>
-      <c r="H82" s="105">
+      <c r="H82" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C82,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I82" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I82" s="53" t="n"/>
     </row>
     <row r="83" ht="30" customHeight="1">
-      <c r="A83" s="105" t="inlineStr">
+      <c r="A83" s="53" t="inlineStr">
         <is>
           <t>RF-079</t>
         </is>
       </c>
-      <c r="B83" s="105" t="inlineStr">
+      <c r="B83" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C83" s="105" t="inlineStr">
+      <c r="C83" s="53" t="inlineStr">
         <is>
           <t>Transversal</t>
         </is>
       </c>
-      <c r="D83" s="105" t="inlineStr">
+      <c r="D83" s="53" t="inlineStr">
         <is>
           <t>Definir si se incorpora un paso explícito de aceptación/confirmación del paciente sobre el prestador asignado, y el tiempo máximo para que la SVP permita editar el prestador (incluyendo el costo operativo de ese cambio).</t>
         </is>
       </c>
       <c r="E83" s="54" t="n"/>
-      <c r="F83" s="105">
+      <c r="F83" s="53">
         <f>IF($E83="",0,INDEX($M$5:$M$8,MATCH($E83,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G83" s="105">
+      <c r="G83" s="53">
         <f>IF($F83=0,0,$F83/10)</f>
         <v/>
       </c>
-      <c r="H83" s="105">
+      <c r="H83" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C83,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I83" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: la aceptación del prestador por el paciente es del Gestor de Coordinación, que queda fuera.</t>
-        </is>
-      </c>
+      <c r="I83" s="53" t="n"/>
     </row>
     <row r="84" ht="30" customHeight="1">
-      <c r="A84" s="105" t="inlineStr">
+      <c r="A84" s="57" t="inlineStr">
         <is>
           <t>RF-080</t>
         </is>
       </c>
-      <c r="B84" s="105" t="inlineStr">
+      <c r="B84" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C84" s="105" t="inlineStr">
+      <c r="C84" s="57" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D84" s="105" t="inlineStr">
+      <c r="D84" s="57" t="inlineStr">
         <is>
           <t>¿Pueden comprometerse a que su primer release sea el contrato de API (aunque la solución completa de gobierno de datos no esté lista), para que Gestores pueda construir contra un contrato estable desde ya?</t>
         </is>
       </c>
       <c r="E84" s="54" t="n"/>
-      <c r="F84" s="105">
+      <c r="F84" s="53">
         <f>IF($E84="",0,INDEX($M$5:$M$8,MATCH($E84,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G84" s="105">
+      <c r="G84" s="53">
         <f>IF($F84=0,0,$F84/10)</f>
         <v/>
       </c>
-      <c r="H84" s="105">
+      <c r="H84" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C84,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I84" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I84" s="53" t="n"/>
     </row>
     <row r="85" ht="30" customHeight="1">
-      <c r="A85" s="105" t="inlineStr">
+      <c r="A85" s="53" t="inlineStr">
         <is>
           <t>RF-081</t>
         </is>
       </c>
-      <c r="B85" s="105" t="inlineStr">
+      <c r="B85" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C85" s="105" t="inlineStr">
+      <c r="C85" s="53" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D85" s="105" t="inlineStr">
+      <c r="D85" s="53" t="inlineStr">
         <is>
           <t>¿Cuál es la cobertura real hoy (cuántos y cuáles prestadores conectados, y si sigue limitado solo a consulta externa, como dijo Santiago en la sesión inicial?</t>
         </is>
       </c>
       <c r="E85" s="54" t="n"/>
-      <c r="F85" s="105">
+      <c r="F85" s="53">
         <f>IF($E85="",0,INDEX($M$5:$M$8,MATCH($E85,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G85" s="105">
+      <c r="G85" s="53">
         <f>IF($F85=0,0,$F85/10)</f>
         <v/>
       </c>
-      <c r="H85" s="105">
+      <c r="H85" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C85,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I85" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I85" s="53" t="n"/>
     </row>
     <row r="86" ht="30" customHeight="1">
-      <c r="A86" s="105" t="inlineStr">
+      <c r="A86" s="57" t="inlineStr">
         <is>
           <t>RF-082</t>
         </is>
       </c>
-      <c r="B86" s="105" t="inlineStr">
+      <c r="B86" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C86" s="105" t="inlineStr">
+      <c r="C86" s="57" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D86" s="105" t="inlineStr">
+      <c r="D86" s="57" t="inlineStr">
         <is>
           <t>Validar si el estándar RDA (Resumen Digital de Atención) cubre lo que Gestores necesita del gestor de Evaluación, o si hay vacíos.</t>
         </is>
       </c>
       <c r="E86" s="54" t="n"/>
-      <c r="F86" s="105">
+      <c r="F86" s="53">
         <f>IF($E86="",0,INDEX($M$5:$M$8,MATCH($E86,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G86" s="105">
+      <c r="G86" s="53">
         <f>IF($F86=0,0,$F86/10)</f>
         <v/>
       </c>
-      <c r="H86" s="105">
+      <c r="H86" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C86,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I86" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I86" s="53" t="n"/>
     </row>
     <row r="87" ht="30" customHeight="1">
-      <c r="A87" s="105" t="inlineStr">
+      <c r="A87" s="53" t="inlineStr">
         <is>
           <t>RF-083</t>
         </is>
       </c>
-      <c r="B87" s="105" t="inlineStr">
+      <c r="B87" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C87" s="105" t="inlineStr">
+      <c r="C87" s="53" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D87" s="105" t="inlineStr">
+      <c r="D87" s="53" t="inlineStr">
         <is>
           <t>Estrategia de canal de ingreso para prestadores declarada dual y no excluyente: la interoperabilidad de autorizaciones es el camino objetivo (“deber ser”); el Front del portal de prestadores se mantiene como contingencia, no se elimina.</t>
         </is>
       </c>
       <c r="E87" s="54" t="n"/>
-      <c r="F87" s="105">
+      <c r="F87" s="53">
         <f>IF($E87="",0,INDEX($M$5:$M$8,MATCH($E87,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G87" s="105">
+      <c r="G87" s="53">
         <f>IF($F87=0,0,$F87/10)</f>
         <v/>
       </c>
-      <c r="H87" s="105">
+      <c r="H87" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C87,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I87" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: define la estrategia dual de canal frente a la interoperabilidad de autorizaciones, que no entra al dibujo.</t>
-        </is>
-      </c>
+      <c r="I87" s="53" t="n"/>
     </row>
     <row r="88" ht="30" customHeight="1">
-      <c r="A88" s="105" t="inlineStr">
+      <c r="A88" s="57" t="inlineStr">
         <is>
           <t>RF-084</t>
         </is>
       </c>
-      <c r="B88" s="105" t="inlineStr">
+      <c r="B88" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C88" s="105" t="inlineStr">
+      <c r="C88" s="57" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D88" s="105" t="inlineStr">
+      <c r="D88" s="57" t="inlineStr">
         <is>
           <t>Para prestadores que ingresen vía interoperabilidad de autorizaciones (modelo orientado a eventos): el gestor se suscribe al ordenamiento en cuanto llega, consulta la historia clínica para completar la información y genera la autorización de forma automática, sin diligenciamiento de formulario ni carga de documentos por parte del prestador.</t>
         </is>
       </c>
       <c r="E88" s="54" t="n"/>
-      <c r="F88" s="105">
+      <c r="F88" s="53">
         <f>IF($E88="",0,INDEX($M$5:$M$8,MATCH($E88,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G88" s="105">
+      <c r="G88" s="53">
         <f>IF($F88=0,0,$F88/10)</f>
         <v/>
       </c>
-      <c r="H88" s="105">
+      <c r="H88" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C88,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I88" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: describe el ingreso por interoperabilidad de autorizaciones, que no está en el dibujo.</t>
-        </is>
-      </c>
+      <c r="I88" s="53" t="n"/>
     </row>
     <row r="89" ht="30" customHeight="1">
-      <c r="A89" s="105" t="inlineStr">
+      <c r="A89" s="53" t="inlineStr">
         <is>
           <t>RF-085</t>
         </is>
       </c>
-      <c r="B89" s="105" t="inlineStr">
+      <c r="B89" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C89" s="105" t="inlineStr">
+      <c r="C89" s="53" t="inlineStr">
         <is>
           <t>Canales / Front Externos</t>
         </is>
       </c>
-      <c r="D89" s="105" t="inlineStr">
+      <c r="D89" s="53" t="inlineStr">
         <is>
           <t>Para los prestadores conectados por interoperabilidad, el Front expondrá una vista de consulta del estado de la autorización frente al ordenamiento y la opción de creación de solicitud nueva (como contingencia), dado que la generación es automática y se actualiza en línea.</t>
         </is>
       </c>
       <c r="E89" s="54" t="n"/>
-      <c r="F89" s="105">
+      <c r="F89" s="53">
         <f>IF($E89="",0,INDEX($M$5:$M$8,MATCH($E89,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G89" s="105">
+      <c r="G89" s="53">
         <f>IF($F89=0,0,$F89/10)</f>
         <v/>
       </c>
-      <c r="H89" s="105">
+      <c r="H89" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C89,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I89" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: la vista para prestadores conectados por interoperabilidad depende de un frente que no entra.</t>
-        </is>
-      </c>
+      <c r="I89" s="53" t="n"/>
     </row>
     <row r="90" ht="30" customHeight="1">
       <c r="A90" s="57" t="inlineStr">
@@ -5246,404 +5098,364 @@
       <c r="I90" s="53" t="n"/>
     </row>
     <row r="91" ht="30" customHeight="1">
-      <c r="A91" s="105" t="inlineStr">
+      <c r="A91" s="53" t="inlineStr">
         <is>
           <t>RF-087</t>
         </is>
       </c>
-      <c r="B91" s="105" t="inlineStr">
+      <c r="B91" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C91" s="105" t="inlineStr">
+      <c r="C91" s="53" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D91" s="105" t="inlineStr">
+      <c r="D91" s="53" t="inlineStr">
         <is>
           <t>El Front web queda formalmente declarado como contingencia (no como opción principal): los prestadores que ingresen por el Front deberán migrar a interoperabilidad en algún punto. Se aclara explícitamente que “contingencia” no implica menor robustez ni pérdida de valor del canal.</t>
         </is>
       </c>
       <c r="E91" s="54" t="n"/>
-      <c r="F91" s="105">
+      <c r="F91" s="53">
         <f>IF($E91="",0,INDEX($M$5:$M$8,MATCH($E91,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G91" s="105">
+      <c r="G91" s="53">
         <f>IF($F91=0,0,$F91/10)</f>
         <v/>
       </c>
-      <c r="H91" s="105">
+      <c r="H91" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C91,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I91" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: es una definición sobre el front como contingencia frente a la interoperabilidad, que no entra.</t>
-        </is>
-      </c>
+      <c r="I91" s="53" t="n"/>
     </row>
     <row r="92" ht="30" customHeight="1">
-      <c r="A92" s="105" t="inlineStr">
+      <c r="A92" s="57" t="inlineStr">
         <is>
           <t>RF-088</t>
         </is>
       </c>
-      <c r="B92" s="105" t="inlineStr">
+      <c r="B92" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C92" s="105" t="inlineStr">
+      <c r="C92" s="57" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D92" s="105" t="inlineStr">
+      <c r="D92" s="57" t="inlineStr">
         <is>
           <t>Se requiere un plan de conexión/incentivo (gancho de valor operativo, no solo normativo) para escalar de los ~3.400 prestadores hoy conectados en interoperabilidad de historia clínica hacia la interoperabilidad de autorizaciones, priorizando instituciones de alto volumen de atención aún no conectadas (ej. Imbanaco, Fundación Valle del Lili, Pablo Tobón Uribe, Clínica Santa Fe).</t>
         </is>
       </c>
       <c r="E92" s="54" t="n"/>
-      <c r="F92" s="105">
+      <c r="F92" s="53">
         <f>IF($E92="",0,INDEX($M$5:$M$8,MATCH($E92,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G92" s="105">
+      <c r="G92" s="53">
         <f>IF($F92=0,0,$F92/10)</f>
         <v/>
       </c>
-      <c r="H92" s="105">
+      <c r="H92" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C92,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I92" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I92" s="53" t="n"/>
     </row>
     <row r="93" ht="30" customHeight="1">
-      <c r="A93" s="105" t="inlineStr">
+      <c r="A93" s="53" t="inlineStr">
         <is>
           <t>RF-089</t>
         </is>
       </c>
-      <c r="B93" s="105" t="inlineStr">
+      <c r="B93" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C93" s="105" t="inlineStr">
+      <c r="C93" s="53" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D93" s="105" t="inlineStr">
+      <c r="D93" s="53" t="inlineStr">
         <is>
           <t>Pendiente confirmar el responsable desde Negocio que jalone/lidere la adopción de interoperabilidad ante los prestadores; Pao de la Cuesta asumiría esa gestión desde su nuevo rol, a confirmar.</t>
         </is>
       </c>
       <c r="E93" s="54" t="n"/>
-      <c r="F93" s="105">
+      <c r="F93" s="53">
         <f>IF($E93="",0,INDEX($M$5:$M$8,MATCH($E93,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G93" s="105">
+      <c r="G93" s="53">
         <f>IF($F93=0,0,$F93/10)</f>
         <v/>
       </c>
-      <c r="H93" s="105">
+      <c r="H93" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C93,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I93" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I93" s="53" t="n"/>
     </row>
     <row r="94" ht="30" customHeight="1">
-      <c r="A94" s="105" t="inlineStr">
+      <c r="A94" s="57" t="inlineStr">
         <is>
           <t>RF-090</t>
         </is>
       </c>
-      <c r="B94" s="105" t="inlineStr">
+      <c r="B94" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C94" s="105" t="inlineStr">
+      <c r="C94" s="57" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D94" s="105" t="inlineStr">
+      <c r="D94" s="57" t="inlineStr">
         <is>
           <t>Cruzar el listado de prestadores compartido por checho (Interoperabilidad) contra el informe de autorizaciones totales por prestador de todo 2026 (a extraer de Globalweb), para determinar el volumen de autorizaciones por prestador.</t>
         </is>
       </c>
       <c r="E94" s="54" t="n"/>
-      <c r="F94" s="105">
+      <c r="F94" s="53">
         <f>IF($E94="",0,INDEX($M$5:$M$8,MATCH($E94,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G94" s="105">
+      <c r="G94" s="53">
         <f>IF($F94=0,0,$F94/10)</f>
         <v/>
       </c>
-      <c r="H94" s="105">
+      <c r="H94" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C94,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I94" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I94" s="53" t="n"/>
     </row>
     <row r="95" ht="30" customHeight="1">
-      <c r="A95" s="105" t="inlineStr">
+      <c r="A95" s="53" t="inlineStr">
         <is>
           <t>RF-091</t>
         </is>
       </c>
-      <c r="B95" s="105" t="inlineStr">
+      <c r="B95" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C95" s="105" t="inlineStr">
+      <c r="C95" s="53" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D95" s="105" t="inlineStr">
+      <c r="D95" s="53" t="inlineStr">
         <is>
           <t>Se expone vista consolidada/agregada del proceso (“el bosque”) y el detalle caso a caso de una solicitud específica (“el árbol”)</t>
         </is>
       </c>
       <c r="E95" s="54" t="n"/>
-      <c r="F95" s="105">
+      <c r="F95" s="53">
         <f>IF($E95="",0,INDEX($M$5:$M$8,MATCH($E95,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G95" s="105">
+      <c r="G95" s="53">
         <f>IF($F95=0,0,$F95/10)</f>
         <v/>
       </c>
-      <c r="H95" s="105">
+      <c r="H95" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C95,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I95" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I95" s="53" t="n"/>
     </row>
     <row r="96" ht="30" customHeight="1">
-      <c r="A96" s="105" t="inlineStr">
+      <c r="A96" s="57" t="inlineStr">
         <is>
           <t>RF-092</t>
         </is>
       </c>
-      <c r="B96" s="105" t="inlineStr">
+      <c r="B96" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C96" s="105" t="inlineStr">
+      <c r="C96" s="57" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D96" s="105" t="inlineStr">
+      <c r="D96" s="57" t="inlineStr">
         <is>
           <t>Alertamiento por información pendiente del cliente en el proceso de Solicitud de Autorización</t>
         </is>
       </c>
       <c r="E96" s="54" t="n"/>
-      <c r="F96" s="105">
+      <c r="F96" s="53">
         <f>IF($E96="",0,INDEX($M$5:$M$8,MATCH($E96,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G96" s="105">
+      <c r="G96" s="53">
         <f>IF($F96=0,0,$F96/10)</f>
         <v/>
       </c>
-      <c r="H96" s="105">
+      <c r="H96" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C96,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I96" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I96" s="53" t="n"/>
     </row>
     <row r="97" ht="30" customHeight="1">
-      <c r="A97" s="105" t="inlineStr">
+      <c r="A97" s="53" t="inlineStr">
         <is>
           <t>RF-093</t>
         </is>
       </c>
-      <c r="B97" s="105" t="inlineStr">
+      <c r="B97" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C97" s="105" t="inlineStr">
+      <c r="C97" s="53" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D97" s="105" t="inlineStr">
+      <c r="D97" s="53" t="inlineStr">
         <is>
           <t>Alertamiento por incumplimiento del SLA por la solicitud de Autorización</t>
         </is>
       </c>
       <c r="E97" s="54" t="n"/>
-      <c r="F97" s="105">
+      <c r="F97" s="53">
         <f>IF($E97="",0,INDEX($M$5:$M$8,MATCH($E97,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G97" s="105">
+      <c r="G97" s="53">
         <f>IF($F97=0,0,$F97/10)</f>
         <v/>
       </c>
-      <c r="H97" s="105">
+      <c r="H97" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C97,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I97" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I97" s="53" t="n"/>
     </row>
     <row r="98" ht="30" customHeight="1">
-      <c r="A98" s="105" t="inlineStr">
+      <c r="A98" s="57" t="inlineStr">
         <is>
           <t>RF-094</t>
         </is>
       </c>
-      <c r="B98" s="105" t="inlineStr">
+      <c r="B98" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C98" s="105" t="inlineStr">
+      <c r="C98" s="57" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D98" s="105" t="inlineStr">
+      <c r="D98" s="57" t="inlineStr">
         <is>
           <t>Alertamiento por próximo incumplimiento del SLA por la solicitud de Autorización</t>
         </is>
       </c>
       <c r="E98" s="54" t="n"/>
-      <c r="F98" s="105">
+      <c r="F98" s="53">
         <f>IF($E98="",0,INDEX($M$5:$M$8,MATCH($E98,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G98" s="105">
+      <c r="G98" s="53">
         <f>IF($F98=0,0,$F98/10)</f>
         <v/>
       </c>
-      <c r="H98" s="105">
+      <c r="H98" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C98,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I98" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I98" s="53" t="n"/>
     </row>
     <row r="99" ht="30" customHeight="1">
-      <c r="A99" s="105" t="inlineStr">
+      <c r="A99" s="53" t="inlineStr">
         <is>
           <t>RF-095</t>
         </is>
       </c>
-      <c r="B99" s="105" t="inlineStr">
+      <c r="B99" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C99" s="105" t="inlineStr">
+      <c r="C99" s="53" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D99" s="105" t="inlineStr">
+      <c r="D99" s="53" t="inlineStr">
         <is>
           <t>Alertamiento en el desborde de capacidad en el proceso de Solicitud de Autorización</t>
         </is>
       </c>
       <c r="E99" s="54" t="n"/>
-      <c r="F99" s="105">
+      <c r="F99" s="53">
         <f>IF($E99="",0,INDEX($M$5:$M$8,MATCH($E99,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G99" s="105">
+      <c r="G99" s="53">
         <f>IF($F99=0,0,$F99/10)</f>
         <v/>
       </c>
-      <c r="H99" s="105">
+      <c r="H99" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C99,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I99" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I99" s="53" t="n"/>
     </row>
     <row r="100" ht="30" customHeight="1">
-      <c r="A100" s="105" t="inlineStr">
+      <c r="A100" s="57" t="inlineStr">
         <is>
           <t>RF-096</t>
         </is>
       </c>
-      <c r="B100" s="105" t="inlineStr">
+      <c r="B100" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C100" s="105" t="inlineStr">
+      <c r="C100" s="57" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D100" s="105" t="inlineStr">
+      <c r="D100" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">Capacidad de Parametrización para alertamientos en la solicitud de autorización </t>
         </is>
       </c>
       <c r="E100" s="54" t="n"/>
-      <c r="F100" s="105">
+      <c r="F100" s="53">
         <f>IF($E100="",0,INDEX($M$5:$M$8,MATCH($E100,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G100" s="105">
+      <c r="G100" s="53">
         <f>IF($F100=0,0,$F100/10)</f>
         <v/>
       </c>
-      <c r="H100" s="105">
+      <c r="H100" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C100,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I100" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I100" s="53" t="n"/>
     </row>
     <row r="101" ht="30" customHeight="1">
       <c r="A101" s="105" t="inlineStr">
@@ -5690,124 +5502,112 @@
       </c>
     </row>
     <row r="102" ht="30" customHeight="1">
-      <c r="A102" s="105" t="inlineStr">
+      <c r="A102" s="57" t="inlineStr">
         <is>
           <t>RF-098</t>
         </is>
       </c>
-      <c r="B102" s="105" t="inlineStr">
+      <c r="B102" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C102" s="105" t="inlineStr">
+      <c r="C102" s="57" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D102" s="105" t="inlineStr">
+      <c r="D102" s="57" t="inlineStr">
         <is>
           <t>Agente que realice sugerencias sobre la decisión que se debe tomar en una solicitud ejemplo: sugerencia al lider operativo de reasignación de solicitudes que superen el tiempo de respuesta a otros evaluadores con mayor oportunidad de respuesta</t>
         </is>
       </c>
       <c r="E102" s="54" t="n"/>
-      <c r="F102" s="105">
+      <c r="F102" s="53">
         <f>IF($E102="",0,INDEX($M$5:$M$8,MATCH($E102,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G102" s="105">
+      <c r="G102" s="53">
         <f>IF($F102=0,0,$F102/10)</f>
         <v/>
       </c>
-      <c r="H102" s="105">
+      <c r="H102" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C102,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I102" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I102" s="53" t="n"/>
     </row>
     <row r="103" ht="30" customHeight="1">
-      <c r="A103" s="105" t="inlineStr">
+      <c r="A103" s="53" t="inlineStr">
         <is>
           <t>RF-099</t>
         </is>
       </c>
-      <c r="B103" s="105" t="inlineStr">
+      <c r="B103" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C103" s="105" t="inlineStr">
+      <c r="C103" s="53" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D103" s="105" t="inlineStr">
+      <c r="D103" s="53" t="inlineStr">
         <is>
           <t>Agente que tome decisiones sobre el marco de actuación de una solicitud, ejemplo: reasignación automatica de solicitudes que superen el tiempo de respuesta a otros evaluadores con mayor oportunidad de respuesta</t>
         </is>
       </c>
       <c r="E103" s="54" t="n"/>
-      <c r="F103" s="105">
+      <c r="F103" s="53">
         <f>IF($E103="",0,INDEX($M$5:$M$8,MATCH($E103,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G103" s="105">
+      <c r="G103" s="53">
         <f>IF($F103=0,0,$F103/10)</f>
         <v/>
       </c>
-      <c r="H103" s="105">
+      <c r="H103" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C103,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I103" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I103" s="53" t="n"/>
     </row>
     <row r="104" ht="30" customHeight="1">
-      <c r="A104" s="105" t="inlineStr">
+      <c r="A104" s="57" t="inlineStr">
         <is>
           <t>RF-100</t>
         </is>
       </c>
-      <c r="B104" s="105" t="inlineStr">
+      <c r="B104" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C104" s="105" t="inlineStr">
+      <c r="C104" s="57" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D104" s="105" t="inlineStr">
+      <c r="D104" s="57" t="inlineStr">
         <is>
           <t>Emitir alertamiento cuando se tengan novedades en la solicitud al cliente/proveedor y asesor, ejemplo: por incumplimiento de SLA</t>
         </is>
       </c>
       <c r="E104" s="54" t="n"/>
-      <c r="F104" s="105">
+      <c r="F104" s="53">
         <f>IF($E104="",0,INDEX($M$5:$M$8,MATCH($E104,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G104" s="105">
+      <c r="G104" s="53">
         <f>IF($F104=0,0,$F104/10)</f>
         <v/>
       </c>
-      <c r="H104" s="105">
+      <c r="H104" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C104,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I104" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I104" s="53" t="n"/>
     </row>
     <row r="105" ht="30" customHeight="1">
       <c r="A105" s="53" t="inlineStr">
@@ -5846,124 +5646,112 @@
       <c r="I105" s="53" t="n"/>
     </row>
     <row r="106" ht="30" customHeight="1">
-      <c r="A106" s="105" t="inlineStr">
+      <c r="A106" s="57" t="inlineStr">
         <is>
           <t>RF-102</t>
         </is>
       </c>
-      <c r="B106" s="105" t="inlineStr">
+      <c r="B106" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C106" s="105" t="inlineStr">
+      <c r="C106" s="57" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D106" s="105" t="inlineStr">
+      <c r="D106" s="57" t="inlineStr">
         <is>
           <t>El agente entrega analítica prescriptiva integrando Torre + Datalake</t>
         </is>
       </c>
       <c r="E106" s="54" t="n"/>
-      <c r="F106" s="105">
+      <c r="F106" s="53">
         <f>IF($E106="",0,INDEX($M$5:$M$8,MATCH($E106,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G106" s="105">
+      <c r="G106" s="53">
         <f>IF($F106=0,0,$F106/10)</f>
         <v/>
       </c>
-      <c r="H106" s="105">
+      <c r="H106" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C106,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I106" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I106" s="53" t="n"/>
     </row>
     <row r="107" ht="30" customHeight="1">
-      <c r="A107" s="105" t="inlineStr">
+      <c r="A107" s="53" t="inlineStr">
         <is>
           <t>RF-103</t>
         </is>
       </c>
-      <c r="B107" s="105" t="inlineStr">
+      <c r="B107" s="53" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C107" s="105" t="inlineStr">
+      <c r="C107" s="53" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D107" s="105" t="inlineStr">
+      <c r="D107" s="53" t="inlineStr">
         <is>
           <t>Entrega de información de las solicitudes, autorizaciones y datos relevantes al Datalake</t>
         </is>
       </c>
       <c r="E107" s="54" t="n"/>
-      <c r="F107" s="105">
+      <c r="F107" s="53">
         <f>IF($E107="",0,INDEX($M$5:$M$8,MATCH($E107,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G107" s="105">
+      <c r="G107" s="53">
         <f>IF($F107=0,0,$F107/10)</f>
         <v/>
       </c>
-      <c r="H107" s="105">
+      <c r="H107" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C107,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I107" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I107" s="53" t="n"/>
     </row>
     <row r="108" ht="30" customHeight="1">
-      <c r="A108" s="105" t="inlineStr">
+      <c r="A108" s="57" t="inlineStr">
         <is>
           <t>RF-104</t>
         </is>
       </c>
-      <c r="B108" s="105" t="inlineStr">
+      <c r="B108" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C108" s="105" t="inlineStr">
+      <c r="C108" s="57" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D108" s="105" t="inlineStr">
+      <c r="D108" s="57" t="inlineStr">
         <is>
           <t>Garantizar que la arquitectura, integraciones, aplicaciones y conexiones que intervienen en el proceso este funcionando de forma adecuada y reaizar alertamientos ante alguna novedad</t>
         </is>
       </c>
       <c r="E108" s="54" t="n"/>
-      <c r="F108" s="105">
+      <c r="F108" s="53">
         <f>IF($E108="",0,INDEX($M$5:$M$8,MATCH($E108,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G108" s="105">
+      <c r="G108" s="53">
         <f>IF($F108=0,0,$F108/10)</f>
         <v/>
       </c>
-      <c r="H108" s="105">
+      <c r="H108" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C108,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I108" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I108" s="53" t="n"/>
     </row>
     <row r="109" ht="30" customHeight="1">
       <c r="A109" s="53" t="inlineStr">
@@ -6002,44 +5790,40 @@
       <c r="I109" s="53" t="n"/>
     </row>
     <row r="110" ht="30" customHeight="1">
-      <c r="A110" s="105" t="inlineStr">
+      <c r="A110" s="57" t="inlineStr">
         <is>
           <t>RF-106</t>
         </is>
       </c>
-      <c r="B110" s="105" t="inlineStr">
+      <c r="B110" s="57" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C110" s="105" t="inlineStr">
+      <c r="C110" s="57" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D110" s="105" t="inlineStr">
+      <c r="D110" s="57" t="inlineStr">
         <is>
           <t>Front de configuración de SLAs según criterios</t>
         </is>
       </c>
       <c r="E110" s="54" t="n"/>
-      <c r="F110" s="105">
+      <c r="F110" s="53">
         <f>IF($E110="",0,INDEX($M$5:$M$8,MATCH($E110,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G110" s="105">
+      <c r="G110" s="53">
         <f>IF($F110=0,0,$F110/10)</f>
         <v/>
       </c>
-      <c r="H110" s="105">
+      <c r="H110" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C110,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I110" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I110" s="53" t="n"/>
     </row>
     <row r="111" ht="30" customHeight="1">
       <c r="A111" s="53" t="inlineStr">
@@ -7318,124 +7102,112 @@
       <c r="I143" s="53" t="n"/>
     </row>
     <row r="144" ht="30" customHeight="1">
-      <c r="A144" s="105" t="inlineStr">
+      <c r="A144" s="57" t="inlineStr">
         <is>
           <t>RT-032</t>
         </is>
       </c>
-      <c r="B144" s="105" t="inlineStr">
+      <c r="B144" s="57" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C144" s="105" t="inlineStr">
+      <c r="C144" s="57" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D144" s="105" t="inlineStr">
+      <c r="D144" s="57" t="inlineStr">
         <is>
           <t>Pendiente definir si se expone una API única con filtrado por perfil o múltiples APIs por actor.</t>
         </is>
       </c>
       <c r="E144" s="54" t="n"/>
-      <c r="F144" s="105">
+      <c r="F144" s="53">
         <f>IF($E144="",0,INDEX($M$5:$M$8,MATCH($E144,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G144" s="105">
+      <c r="G144" s="53">
         <f>IF($F144=0,0,$F144/10)</f>
         <v/>
       </c>
-      <c r="H144" s="105">
+      <c r="H144" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C144,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I144" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I144" s="53" t="n"/>
     </row>
     <row r="145" ht="30" customHeight="1">
-      <c r="A145" s="105" t="inlineStr">
+      <c r="A145" s="53" t="inlineStr">
         <is>
           <t>RT-033</t>
         </is>
       </c>
-      <c r="B145" s="105" t="inlineStr">
+      <c r="B145" s="53" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C145" s="105" t="inlineStr">
+      <c r="C145" s="53" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D145" s="105" t="inlineStr">
+      <c r="D145" s="53" t="inlineStr">
         <is>
           <t>Reto de integración en tiempo real con prestadores — hoy no existe (solo portal con interacción manual).</t>
         </is>
       </c>
       <c r="E145" s="54" t="n"/>
-      <c r="F145" s="105">
+      <c r="F145" s="53">
         <f>IF($E145="",0,INDEX($M$5:$M$8,MATCH($E145,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G145" s="105">
+      <c r="G145" s="53">
         <f>IF($F145=0,0,$F145/10)</f>
         <v/>
       </c>
-      <c r="H145" s="105">
+      <c r="H145" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C145,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I145" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I145" s="53" t="n"/>
     </row>
     <row r="146" ht="30" customHeight="1">
-      <c r="A146" s="105" t="inlineStr">
+      <c r="A146" s="57" t="inlineStr">
         <is>
           <t>RT-034</t>
         </is>
       </c>
-      <c r="B146" s="105" t="inlineStr">
+      <c r="B146" s="57" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C146" s="105" t="inlineStr">
+      <c r="C146" s="57" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D146" s="105" t="inlineStr">
+      <c r="D146" s="57" t="inlineStr">
         <is>
           <t>Datalake de autorizaciones como entregable técnico del Release 3 (feb-abr 2027), con apoyo del arquitecto de datos.</t>
         </is>
       </c>
       <c r="E146" s="54" t="n"/>
-      <c r="F146" s="105">
+      <c r="F146" s="53">
         <f>IF($E146="",0,INDEX($M$5:$M$8,MATCH($E146,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G146" s="105">
+      <c r="G146" s="53">
         <f>IF($F146=0,0,$F146/10)</f>
         <v/>
       </c>
-      <c r="H146" s="105">
+      <c r="H146" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C146,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I146" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I146" s="53" t="n"/>
     </row>
     <row r="147" ht="30" customHeight="1">
       <c r="A147" s="53" t="inlineStr">
@@ -7590,84 +7362,76 @@
       </c>
     </row>
     <row r="151" ht="30" customHeight="1">
-      <c r="A151" s="105" t="inlineStr">
+      <c r="A151" s="53" t="inlineStr">
         <is>
           <t>RT-039</t>
         </is>
       </c>
-      <c r="B151" s="105" t="inlineStr">
+      <c r="B151" s="53" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C151" s="105" t="inlineStr">
+      <c r="C151" s="53" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D151" s="105" t="inlineStr">
+      <c r="D151" s="53" t="inlineStr">
         <is>
           <t>El modelo de eventos de interoperabilidad de historia clínica migra hacia una arquitectura 2.0 orientada a eventos (colas por suscripción/webhooks), desde la arquitectura tradicional de microservicios; hoy conecta 6 prestadores de ayuda diagnóstica externa.</t>
         </is>
       </c>
       <c r="E151" s="54" t="n"/>
-      <c r="F151" s="105">
+      <c r="F151" s="53">
         <f>IF($E151="",0,INDEX($M$5:$M$8,MATCH($E151,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G151" s="105">
+      <c r="G151" s="53">
         <f>IF($F151=0,0,$F151/10)</f>
         <v/>
       </c>
-      <c r="H151" s="105">
+      <c r="H151" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C151,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I151" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I151" s="53" t="n"/>
     </row>
     <row r="152" ht="30" customHeight="1">
-      <c r="A152" s="105" t="inlineStr">
+      <c r="A152" s="57" t="inlineStr">
         <is>
           <t>RT-040</t>
         </is>
       </c>
-      <c r="B152" s="105" t="inlineStr">
+      <c r="B152" s="57" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C152" s="105" t="inlineStr">
+      <c r="C152" s="57" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D152" s="105" t="inlineStr">
+      <c r="D152" s="57" t="inlineStr">
         <is>
           <t>No existe hoy interoperabilidad de agenda por barreras de mercado (ningún prestador ni aseguradora quiere ser el centralizador); una propuesta de mercado con un tercero integrador está en etapa muy temprana.</t>
         </is>
       </c>
       <c r="E152" s="54" t="n"/>
-      <c r="F152" s="105">
+      <c r="F152" s="53">
         <f>IF($E152="",0,INDEX($M$5:$M$8,MATCH($E152,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G152" s="105">
+      <c r="G152" s="53">
         <f>IF($F152=0,0,$F152/10)</f>
         <v/>
       </c>
-      <c r="H152" s="105">
+      <c r="H152" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C152,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I152" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I152" s="53" t="n"/>
     </row>
     <row r="153" ht="30" customHeight="1">
       <c r="A153" s="53" t="inlineStr">
@@ -7934,84 +7698,76 @@
       <c r="I159" s="53" t="n"/>
     </row>
     <row r="160" ht="30" customHeight="1">
-      <c r="A160" s="105" t="inlineStr">
+      <c r="A160" s="57" t="inlineStr">
         <is>
           <t>RT-048</t>
         </is>
       </c>
-      <c r="B160" s="105" t="inlineStr">
+      <c r="B160" s="57" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C160" s="105" t="inlineStr">
+      <c r="C160" s="57" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
         </is>
       </c>
-      <c r="D160" s="105" t="inlineStr">
+      <c r="D160" s="57" t="inlineStr">
         <is>
           <t>El módulo de interoperabilidad de autorizaciones no parte de cero: reutiliza la infraestructura ya construida de interoperabilidad; se tomará como pivote de esfuerzo el costo de la interoperabilidad de ayudas diagnósticas (la más comparable), reconociendo que autorizaciones tiene casuística y costos propios.</t>
         </is>
       </c>
       <c r="E160" s="54" t="n"/>
-      <c r="F160" s="105">
+      <c r="F160" s="53">
         <f>IF($E160="",0,INDEX($M$5:$M$8,MATCH($E160,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G160" s="105">
+      <c r="G160" s="53">
         <f>IF($F160=0,0,$F160/10)</f>
         <v/>
       </c>
-      <c r="H160" s="105">
+      <c r="H160" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C160,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I160" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo no incluye la interoperabilidad de autorizaciones con prestadores. El único principio que sí entra es el acceso al dato vía el core (RF-070).</t>
-        </is>
-      </c>
+      <c r="I160" s="53" t="n"/>
     </row>
     <row r="161" ht="30" customHeight="1">
-      <c r="A161" s="105" t="inlineStr">
+      <c r="A161" s="53" t="inlineStr">
         <is>
           <t>RT-049</t>
         </is>
       </c>
-      <c r="B161" s="105" t="inlineStr">
+      <c r="B161" s="53" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C161" s="105" t="inlineStr">
+      <c r="C161" s="53" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
         </is>
       </c>
-      <c r="D161" s="105" t="inlineStr">
+      <c r="D161" s="53" t="inlineStr">
         <is>
           <t>Se evalúa como insumo de referencia (no de adopción literal) una propuesta de arquitectura agéntica mundial para torres de control de salud, compuesta por 9 agentes especializados (radar, riesgo operacional, capacidad, predictor, director del tráfico, marcos de actuación, anomalías, explicador, recomendación) más un agente “comandante de operaciones” a futuro con capacidad de ejecución directa.</t>
         </is>
       </c>
       <c r="E161" s="54" t="n"/>
-      <c r="F161" s="105">
+      <c r="F161" s="53">
         <f>IF($E161="",0,INDEX($M$5:$M$8,MATCH($E161,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G161" s="105">
+      <c r="G161" s="53">
         <f>IF($F161=0,0,$F161/10)</f>
         <v/>
       </c>
-      <c r="H161" s="105">
+      <c r="H161" s="53">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C161,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I161" s="105" t="inlineStr">
-        <is>
-          <t>Fuera del MVP: el dibujo acota la torre a las capas 1 (ingesta y consolidación) y 2 (correlación y contexto). Medición, alertamiento, decisión y exposición son capas 3 a 5.</t>
-        </is>
-      </c>
+      <c r="I161" s="53" t="n"/>
     </row>
     <row r="162" ht="30" customHeight="1">
       <c r="A162" s="57" t="inlineStr">

</xml_diff>

<commit_message>
corrige la leyenda y deja la estimación real, sin margen
el bloque de resultado declara la suma tal cual: 74 requisitos del mvp, 500 días
hábiles, 50 sprints de un frente, con el reparto por épica y sin margen de
incertidumbre, por decisión del equipo. rt-037 queda en alerta con esa decisión
escrita en observaciones.

rf-054 corrige su salvedad: la talla cubre solo la detección de solicitudes
repetidas, porque el flujo de rescate que invoca (rf-019) y la notificación al
asegurado quedan fuera del mvp.

la leyenda se reescribe con los colores que quedaron en uso y suma tres avisos de
lectura: la tabla de tallaje dice s = 2 días y la nota de al lado dice 3, y se usó
la tabla porque es la que alimenta la fórmula; funcionales y técnicos se tallan
por separado y hay cinco pares que describen la misma capacidad; y los mínimos
del acta del 21 de agosto se cumplen, 59 días en solicitud y 52 en siniestro
integral.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SURA/gestores-sura/estimacin mvp/2 Gestores_Seguimiento_Requerimientos_2026.xlsx
+++ b/SURA/gestores-sura/estimacin mvp/2 Gestores_Seguimiento_Requerimientos_2026.xlsx
@@ -29,7 +29,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="33">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -230,6 +230,7 @@
       <name val="Sura Sans"/>
       <sz val="9"/>
     </font>
+    <font/>
   </fonts>
   <fills count="31">
     <fill>
@@ -616,7 +617,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -900,6 +901,22 @@
     <xf numFmtId="0" fontId="30" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="30" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2810,7 +2827,7 @@
       </c>
       <c r="I30" s="53" t="n"/>
     </row>
-    <row r="31" ht="30" customHeight="1">
+    <row r="31">
       <c r="A31" s="53" t="inlineStr">
         <is>
           <t>RF-027</t>
@@ -2849,8 +2866,14 @@
         <v/>
       </c>
       <c r="I31" s="53" t="n"/>
-    </row>
-    <row r="32" ht="30" customHeight="1">
+      <c r="L31" s="115" t="n"/>
+      <c r="M31" s="115" t="n"/>
+      <c r="N31" s="115" t="n"/>
+      <c r="O31" s="115" t="n"/>
+      <c r="P31" s="115" t="n"/>
+      <c r="Q31" s="115" t="n"/>
+    </row>
+    <row r="32">
       <c r="A32" s="57" t="inlineStr">
         <is>
           <t>RF-028</t>
@@ -2891,9 +2914,14 @@
       <c r="I32" s="53" t="n"/>
       <c r="L32" s="108" t="inlineStr">
         <is>
-          <t>Leyenda de esta revisión (Tech and Solve)</t>
-        </is>
-      </c>
+          <t>Leyenda y criterio de esta estimación (Tech and Solve)</t>
+        </is>
+      </c>
+      <c r="M32" s="115" t="n"/>
+      <c r="N32" s="115" t="n"/>
+      <c r="O32" s="115" t="n"/>
+      <c r="P32" s="115" t="n"/>
+      <c r="Q32" s="115" t="n"/>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="53" t="inlineStr">
@@ -2934,14 +2962,14 @@
         <v/>
       </c>
       <c r="I33" s="53" t="n"/>
-      <c r="L33" s="109" t="inlineStr">
+      <c r="L33" s="116" t="inlineStr">
         <is>
           <t>Fila adicionada</t>
         </is>
       </c>
       <c r="M33" s="110" t="inlineStr">
         <is>
-          <t>Requisito funcional nuevo (RF-109 a RF-129): elementos que el dibujo del MVP y la vista de tecnología exigen y que la hoja no tenía.</t>
+          <t>Requisito funcional nuevo, RF-109 a RF-129. Elementos que el dibujo del MVP y la vista de tecnología exigen y que la hoja no tenía.</t>
         </is>
       </c>
     </row>
@@ -2980,14 +3008,14 @@
         <v/>
       </c>
       <c r="I34" s="53" t="n"/>
-      <c r="L34" s="111" t="inlineStr">
-        <is>
-          <t>Fila modificada</t>
+      <c r="L34" s="117" t="inlineStr">
+        <is>
+          <t>Alerta · sin tallar</t>
         </is>
       </c>
       <c r="M34" s="110" t="inlineStr">
         <is>
-          <t>Fila existente a la que se le agregó una observación: entra al MVP con una salvedad, o queda fuera y se explica por qué.</t>
+          <t>Requisito que no se pudo estimar. La duda concreta queda escrita en Observaciones. Son 13.</t>
         </is>
       </c>
     </row>
@@ -3026,14 +3054,14 @@
         <v/>
       </c>
       <c r="I35" s="53" t="n"/>
-      <c r="L35" s="112" t="inlineStr">
-        <is>
-          <t>Alerta · sin tallar</t>
+      <c r="L35" s="118" t="inlineStr">
+        <is>
+          <t>Fila modificada</t>
         </is>
       </c>
       <c r="M35" s="110" t="inlineStr">
         <is>
-          <t>Requisito que no se pudo estimar. La duda concreta queda escrita en Observaciones.</t>
+          <t>Requisito que entra al MVP con una salvedad sobre qué cubre la talla; la salvedad está en Observaciones. Son 7.</t>
         </is>
       </c>
     </row>
@@ -3072,7 +3100,7 @@
         <v/>
       </c>
       <c r="I36" s="53" t="n"/>
-      <c r="L36" s="113" t="inlineStr">
+      <c r="L36" s="119" t="inlineStr">
         <is>
           <t>Talla diligenciada</t>
         </is>
@@ -3118,18 +3146,18 @@
         <v/>
       </c>
       <c r="I37" s="53" t="n"/>
-      <c r="L37" s="114" t="inlineStr">
+      <c r="L37" s="120" t="inlineStr">
         <is>
           <t>Sin color y sin talla</t>
         </is>
       </c>
       <c r="M37" s="110" t="inlineStr">
         <is>
-          <t>Requisito fuera del MVP en una épica que esta misma hoja ya marca «No» o «N/A».</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1">
+          <t>Requisito fuera del MVP. No se modificó ninguna de estas filas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
       <c r="A38" s="57" t="inlineStr">
         <is>
           <t>RF-034</t>
@@ -3164,8 +3192,14 @@
         <v/>
       </c>
       <c r="I38" s="53" t="n"/>
-    </row>
-    <row r="39" ht="60" customHeight="1">
+      <c r="L38" s="115" t="n"/>
+      <c r="M38" s="115" t="n"/>
+      <c r="N38" s="115" t="n"/>
+      <c r="O38" s="115" t="n"/>
+      <c r="P38" s="115" t="n"/>
+      <c r="Q38" s="115" t="n"/>
+    </row>
+    <row r="39">
       <c r="A39" s="53" t="inlineStr">
         <is>
           <t>RF-035</t>
@@ -3200,18 +3234,18 @@
         <v/>
       </c>
       <c r="I39" s="53" t="n"/>
-      <c r="L39" s="114" t="inlineStr">
-        <is>
-          <t>Criterio de alcance</t>
-        </is>
-      </c>
-      <c r="M39" s="110" t="inlineStr">
-        <is>
-          <t>La pertenencia al MVP se decidió requisito por requisito contra «resumen-arquitectura-gestores — Arquitectura MVP» y «arquitectura-tecnologia», no contra la columna «¿En MVP?», que se deriva por épica y por eso marca «Sí» a épicas donde solo una parte entra. Entran Solicitud, Evaluación, Siniestro Integral, los canales que el MVP habilita, las capas 1 y 2 de la torre, el acceso al dato vía el core y los transversales del ciclo de mejora y del plano de control. Suma: 500 días hábiles con la escala de la propia hoja.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="30" customHeight="1">
+      <c r="L39" s="108" t="inlineStr">
+        <is>
+          <t>Resultado</t>
+        </is>
+      </c>
+      <c r="M39" s="115" t="n"/>
+      <c r="N39" s="115" t="n"/>
+      <c r="O39" s="115" t="n"/>
+      <c r="P39" s="115" t="n"/>
+      <c r="Q39" s="115" t="n"/>
+    </row>
+    <row r="40" ht="46" customHeight="1">
       <c r="A40" s="57" t="inlineStr">
         <is>
           <t>RF-036</t>
@@ -3246,8 +3280,18 @@
         <v/>
       </c>
       <c r="I40" s="53" t="n"/>
-    </row>
-    <row r="41" ht="30" customHeight="1">
+      <c r="L40" s="120" t="inlineStr">
+        <is>
+          <t>Suma y margen</t>
+        </is>
+      </c>
+      <c r="M40" s="110" t="inlineStr">
+        <is>
+          <t>74 requisitos del MVP tallados: 500 días hábiles, 50 sprints de un frente, con la escala de la propia hoja. La suma va sin margen de incertidumbre. Reparto: Gestor de Evaluación 138 d · Gestor de Monitoreo 97 d · Gestor de Solicitud 59 d · Transversal (principios) 59 d · Siniestro Integral 52 d · Transversal 50 d · Canales / Front Externos 43 d · Interoperabilidad (Prestadores) 2 d.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
       <c r="A41" s="53" t="inlineStr">
         <is>
           <t>RF-037</t>
@@ -3282,8 +3326,14 @@
         <v/>
       </c>
       <c r="I41" s="53" t="n"/>
-    </row>
-    <row r="42" ht="30" customHeight="1">
+      <c r="L41" s="115" t="n"/>
+      <c r="M41" s="115" t="n"/>
+      <c r="N41" s="115" t="n"/>
+      <c r="O41" s="115" t="n"/>
+      <c r="P41" s="115" t="n"/>
+      <c r="Q41" s="115" t="n"/>
+    </row>
+    <row r="42">
       <c r="A42" s="57" t="inlineStr">
         <is>
           <t>RF-038</t>
@@ -3318,8 +3368,18 @@
         <v/>
       </c>
       <c r="I42" s="53" t="n"/>
-    </row>
-    <row r="43" ht="30" customHeight="1">
+      <c r="L42" s="108" t="inlineStr">
+        <is>
+          <t>Criterio de alcance</t>
+        </is>
+      </c>
+      <c r="M42" s="115" t="n"/>
+      <c r="N42" s="115" t="n"/>
+      <c r="O42" s="115" t="n"/>
+      <c r="P42" s="115" t="n"/>
+      <c r="Q42" s="115" t="n"/>
+    </row>
+    <row r="43" ht="60" customHeight="1">
       <c r="A43" s="53" t="inlineStr">
         <is>
           <t>RF-039</t>
@@ -3360,8 +3420,18 @@
         <v/>
       </c>
       <c r="I43" s="53" t="n"/>
-    </row>
-    <row r="44" ht="30" customHeight="1">
+      <c r="L43" s="120" t="inlineStr">
+        <is>
+          <t>Qué entra</t>
+        </is>
+      </c>
+      <c r="M43" s="110" t="inlineStr">
+        <is>
+          <t>La pertenencia al MVP se decidió requisito por requisito contra «resumen-arquitectura-gestores — Arquitectura MVP» y «arquitectura-tecnologia», no contra la columna «¿En MVP?», que se deriva por épica y por eso marca «Sí» a épicas donde solo una parte entra. Entran Solicitud, Evaluación, Siniestro Integral, los canales que el MVP habilita, las capas 1 y 2 de la torre, el acceso al dato vía el core y los transversales del ciclo de mejora y del plano de control. Quedan fuera Coordinación, Prestación, Finalización, Asignación, Nexo, AVA, la interoperabilidad de autorizaciones y las capas 3, 4 y 5 de la torre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
       <c r="A44" s="57" t="inlineStr">
         <is>
           <t>RF-040</t>
@@ -3396,8 +3466,14 @@
         <v/>
       </c>
       <c r="I44" s="53" t="n"/>
-    </row>
-    <row r="45" ht="30" customHeight="1">
+      <c r="L44" s="115" t="n"/>
+      <c r="M44" s="115" t="n"/>
+      <c r="N44" s="115" t="n"/>
+      <c r="O44" s="115" t="n"/>
+      <c r="P44" s="115" t="n"/>
+      <c r="Q44" s="115" t="n"/>
+    </row>
+    <row r="45">
       <c r="A45" s="53" t="inlineStr">
         <is>
           <t>RF-041</t>
@@ -3432,8 +3508,18 @@
         <v/>
       </c>
       <c r="I45" s="53" t="n"/>
-    </row>
-    <row r="46" ht="30" customHeight="1">
+      <c r="L45" s="108" t="inlineStr">
+        <is>
+          <t>Tres cosas que conviene saber antes de leer el total</t>
+        </is>
+      </c>
+      <c r="M45" s="115" t="n"/>
+      <c r="N45" s="115" t="n"/>
+      <c r="O45" s="115" t="n"/>
+      <c r="P45" s="115" t="n"/>
+      <c r="Q45" s="115" t="n"/>
+    </row>
+    <row r="46" ht="32" customHeight="1">
       <c r="A46" s="57" t="inlineStr">
         <is>
           <t>RF-042</t>
@@ -3468,8 +3554,18 @@
         <v/>
       </c>
       <c r="I46" s="53" t="n"/>
-    </row>
-    <row r="47" ht="30" customHeight="1">
+      <c r="L46" s="120" t="inlineStr">
+        <is>
+          <t>La escala se contradice</t>
+        </is>
+      </c>
+      <c r="M46" s="110" t="inlineStr">
+        <is>
+          <t>La tabla de tallaje dice S = 2 días y la nota de al lado dice S ≈ 3 días. Se usó la tabla, porque es la que alimenta la fórmula de la columna F. Si el equipo confirma los 3 días, el total sube 15 días (hay 15 requisitos en S).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="32" customHeight="1">
       <c r="A47" s="53" t="inlineStr">
         <is>
           <t>RF-043</t>
@@ -3504,8 +3600,18 @@
         <v/>
       </c>
       <c r="I47" s="53" t="n"/>
-    </row>
-    <row r="48" ht="30" customHeight="1">
+      <c r="L47" s="120" t="inlineStr">
+        <is>
+          <t>Funcionales y técnicos se suman</t>
+        </is>
+      </c>
+      <c r="M47" s="110" t="inlineStr">
+        <is>
+          <t>La hoja talla por separado el requisito funcional y el técnico, y así se respetó. Hay pares que describen la misma capacidad —RF-021 con RT-018, RF-024 con RT-020, RF-025 con RT-021, RF-001 con RT-011, RF-011 con RT-017—. Si el equipo decide contarlos una sola vez, el total baja hasta 32 días.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="26" customHeight="1">
       <c r="A48" s="57" t="inlineStr">
         <is>
           <t>RF-044</t>
@@ -3540,8 +3646,18 @@
         <v/>
       </c>
       <c r="I48" s="53" t="n"/>
-    </row>
-    <row r="49" ht="30" customHeight="1">
+      <c r="L48" s="120" t="inlineStr">
+        <is>
+          <t>Mínimos del acta</t>
+        </is>
+      </c>
+      <c r="M48" s="110" t="inlineStr">
+        <is>
+          <t>El acta del 21-ago-2026 fija talla mínima L para el Gestor de Solicitud y mínimo 1 sprint para Siniestro Integral. Ambos se cumplen: 59 y 52 días.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
       <c r="A49" s="53" t="inlineStr">
         <is>
           <t>RF-045</t>
@@ -3576,6 +3692,12 @@
         <v/>
       </c>
       <c r="I49" s="53" t="n"/>
+      <c r="L49" s="115" t="n"/>
+      <c r="M49" s="115" t="n"/>
+      <c r="N49" s="115" t="n"/>
+      <c r="O49" s="115" t="n"/>
+      <c r="P49" s="115" t="n"/>
+      <c r="Q49" s="115" t="n"/>
     </row>
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="57" t="inlineStr">
@@ -3913,7 +4035,7 @@
       </c>
       <c r="I58" s="105" t="inlineStr">
         <is>
-          <t>Entra la detección de solicitudes repetidas, que el dibujo resuelve en la capa de duplicidad. La notificación al asegurado depende de la capa de exposición de la torre, que no está en el MVP.</t>
+          <t>Entra la detección de solicitudes repetidas, que el dibujo resuelve en la capa de duplicidad. La talla cubre solo eso: el flujo de rescate que el requisito invoca (RF-019) y la notificación al asegurado quedan fuera del MVP, así que el requisito no se cumple completo con esta talla.</t>
         </is>
       </c>
     </row>
@@ -7317,7 +7439,7 @@
       </c>
       <c r="I149" s="106" t="inlineStr">
         <is>
-          <t>🟥 No es un entregable de construcción: es la regla de presentación de la estimación (declarar 30% de incertidumbre). Aplica a este ejercicio, no se talla.</t>
+          <t>🟥 No es un entregable de construcción: es la regla de presentación de la estimación (declarar un 30% de incertidumbre ante patrocinadores). El equipo decidió estimar sin aplicar ese margen, así que la suma de esta hoja va sin él. No se talla.</t>
         </is>
       </c>
     </row>
@@ -8811,18 +8933,22 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:Q187"/>
-  <mergeCells count="11">
+  <mergeCells count="15">
+    <mergeCell ref="M48:Q48"/>
+    <mergeCell ref="M40:Q40"/>
     <mergeCell ref="M35:Q35"/>
+    <mergeCell ref="M43:Q43"/>
     <mergeCell ref="M34:Q34"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="M47:Q47"/>
     <mergeCell ref="M37:Q37"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="L9:N12"/>
     <mergeCell ref="L13:Q13"/>
     <mergeCell ref="M33:Q33"/>
+    <mergeCell ref="M46:Q46"/>
     <mergeCell ref="M36:Q36"/>
     <mergeCell ref="L3:N3"/>
-    <mergeCell ref="M39:Q39"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="E5:E187" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
cierra la respuesta pendiente del front: angular
rt-008 y rt-045 eran los dos únicos requisitos que quedaban sin tallar por la
tecnología del front. con angular confirmado el conflicto se cierra, porque es lo
que ya fijaba el lineamiento: static web app con angular spa.

rt-008 queda en xl: el front nuevo embebido en los dos canales del mvp, portal
proveedor y svp; ava es 2027 y no entra. rt-045 queda en m: solo la
diferenciación por rol del web component, porque la decisión del front único ya
está tallada en rt-006 y no se cuenta dos veces.

las alertas bajan de 13 a 11 y el total del mvp pasa de 500 a 525 días hábiles,
52 sprints de un frente. gestor de solicitud pasa de 59 a 84 días.

dentro del mvp no hay front de la torre de control: sus capas 1 y 2 no tienen
interfaz, y la vista de exposición es capa 5, fuera del alcance.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SURA/gestores-sura/estimacin mvp/2 Gestores_Seguimiento_Requerimientos_2026.xlsx
+++ b/SURA/gestores-sura/estimacin mvp/2 Gestores_Seguimiento_Requerimientos_2026.xlsx
@@ -3015,7 +3015,7 @@
       </c>
       <c r="M34" s="110" t="inlineStr">
         <is>
-          <t>Requisito que no se pudo estimar. La duda concreta queda escrita en Observaciones. Son 13.</t>
+          <t>Requisito que no se pudo estimar. La duda concreta queda escrita en Observaciones. Son 11.</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="M35" s="110" t="inlineStr">
         <is>
-          <t>Requisito que entra al MVP con una salvedad sobre qué cubre la talla; la salvedad está en Observaciones. Son 7.</t>
+          <t>Requisito que entra al MVP con una salvedad sobre qué cubre la talla, o cuya duda ya se cerró con una decisión del equipo; en ambos casos queda escrita en Observaciones. Son 9.</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="M40" s="110" t="inlineStr">
         <is>
-          <t>74 requisitos del MVP tallados: 500 días hábiles, 50 sprints de un frente, con la escala de la propia hoja. La suma va sin margen de incertidumbre. Reparto: Gestor de Evaluación 138 d · Gestor de Monitoreo 97 d · Gestor de Solicitud 59 d · Transversal (principios) 59 d · Siniestro Integral 52 d · Transversal 50 d · Canales / Front Externos 43 d · Interoperabilidad (Prestadores) 2 d.</t>
+          <t>76 requisitos del MVP tallados: 525 días hábiles, 52 sprints de un frente, con la escala de la propia hoja. La suma va sin margen de incertidumbre. Reparto: Gestor de Evaluación 138 d · Gestor de Monitoreo 97 d · Gestor de Solicitud 84 d · Transversal (principios) 59 d · Siniestro Integral 52 d · Transversal 50 d · Canales / Front Externos 43 d · Interoperabilidad (Prestadores) 2 d.</t>
         </is>
       </c>
     </row>
@@ -6300,42 +6300,46 @@
       <c r="I119" s="53" t="n"/>
     </row>
     <row r="120" ht="30" customHeight="1">
-      <c r="A120" s="106" t="inlineStr">
+      <c r="A120" s="105" t="inlineStr">
         <is>
           <t>RT-008</t>
         </is>
       </c>
-      <c r="B120" s="106" t="inlineStr">
+      <c r="B120" s="105" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C120" s="106" t="inlineStr">
+      <c r="C120" s="105" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D120" s="106" t="inlineStr">
+      <c r="D120" s="105" t="inlineStr">
         <is>
           <t>Front nuevo (Flutter), embebido en Sucursal Virtual Personas, AVA y Portal de Prestadores; reutiliza el back/orquestador de Siniestro Integral.</t>
         </is>
       </c>
-      <c r="E120" s="107" t="n"/>
-      <c r="F120" s="106">
+      <c r="E120" s="99" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="F120" s="105">
         <f>IF($E120="",0,INDEX($M$5:$M$8,MATCH($E120,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G120" s="106">
+      <c r="G120" s="105">
         <f>IF($F120=0,0,$F120/10)</f>
         <v/>
       </c>
-      <c r="H120" s="106">
+      <c r="H120" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C120,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I120" s="106" t="inlineStr">
-        <is>
-          <t>🟥 Conflicto con el lineamiento. El requisito dice front en Flutter; el lineamiento AI First fija la experiencia en Azure Static Web App con Angular SPA (Arquitectura de implementación, página 6243680318). Resolver la tecnología del front antes de tallar.</t>
+      <c r="I120" s="105" t="inlineStr">
+        <is>
+          <t>El equipo confirmó Angular, con lo que se cierra el conflicto: coincide con lo que fija el lineamiento AI First, «La experiencia conversacional se materializa en una Static Web App basada en Angular SPA» (Arquitectura de implementación, página 6243680318). La talla cubre el front nuevo embebido en los dos canales del MVP, Portal Proveedor y SVP; AVA es 2027 y no está incluida.</t>
         </is>
       </c>
     </row>
@@ -7708,42 +7712,46 @@
       <c r="I156" s="53" t="n"/>
     </row>
     <row r="157" ht="30" customHeight="1">
-      <c r="A157" s="106" t="inlineStr">
+      <c r="A157" s="105" t="inlineStr">
         <is>
           <t>RT-045</t>
         </is>
       </c>
-      <c r="B157" s="106" t="inlineStr">
+      <c r="B157" s="105" t="inlineStr">
         <is>
           <t>Técnico</t>
         </is>
       </c>
-      <c r="C157" s="106" t="inlineStr">
+      <c r="C157" s="105" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
         </is>
       </c>
-      <c r="D157" s="106" t="inlineStr">
+      <c r="D157" s="105" t="inlineStr">
         <is>
           <t>Confirmado: un único web component (Flutter), agnóstico de canal y con funcionalidades diferenciadas por rol (prestador suma 2-3 campos adicionales frente a cliente), embebido en app móvil, Sucursal Virtual Personas y Portal de Prestador/Proveedor — se descarta un front independiente por canal.</t>
         </is>
       </c>
-      <c r="E157" s="107" t="n"/>
-      <c r="F157" s="106">
+      <c r="E157" s="99" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F157" s="105">
         <f>IF($E157="",0,INDEX($M$5:$M$8,MATCH($E157,$L$5:$L$8,0)))</f>
         <v/>
       </c>
-      <c r="G157" s="106">
+      <c r="G157" s="105">
         <f>IF($F157=0,0,$F157/10)</f>
         <v/>
       </c>
-      <c r="H157" s="106">
+      <c r="H157" s="105">
         <f>IFERROR(INDEX($O$15:$O$29,MATCH($C157,$L$15:$L$29,0)),"🟨 validar")</f>
         <v/>
       </c>
-      <c r="I157" s="106" t="inlineStr">
-        <is>
-          <t>🟥 Mismo conflicto de RT-008: el web component se declara en Flutter y el lineamiento fija Angular sobre Static Web App. La decisión de un único web component agnóstico de canal sí es la del MVP; falta cerrar la tecnología.</t>
+      <c r="I157" s="105" t="inlineStr">
+        <is>
+          <t>El equipo confirmó Angular. La talla cubre solo la diferenciación por rol del web component único —el prestador suma 2 o 3 campos frente al cliente—, porque la decisión del front único reutilizable ya está tallada en RT-006 y no se cuenta dos veces.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
agrega el filtro de capacidad agéntica sobre los requisitos del mvp
columna j nueva, «capacidad agéntica», con lista desplegable y dentro del
autofiltro de la hoja. clasifica solo los 76 requisitos del mvp con la convención
del propio dibujo; las filas fuera del mvp quedan en blanco.

agéntica, 16 requisitos y 124 días: clasificador, enrutador, request builder,
llm-as-a-judge, extractores, pertinencia médica, duplicidad y auditor.
habilitadora, 16 y 106 días: golden set, compuerta de promoción, umbrales y
techos, traza de la decisión y calibración del juez. determinística, 44 y 295
días: reglas duras, apis, integraciones, almacenamiento, front y contrato de
eventos.

el resumen va con countif y sumif sobre la columna, no con números fijos, así que
se mueve si alguien cambia una talla o una clasificación.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SURA/gestores-sura/estimacin mvp/2 Gestores_Seguimiento_Requerimientos_2026.xlsx
+++ b/SURA/gestores-sura/estimacin mvp/2 Gestores_Seguimiento_Requerimientos_2026.xlsx
@@ -617,7 +617,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="123">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -917,6 +917,8 @@
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1187,6 +1189,7 @@
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="8"/>
     <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="15"/>
@@ -1261,6 +1264,11 @@
           <t>Observaciones</t>
         </is>
       </c>
+      <c r="J4" s="51" t="inlineStr">
+        <is>
+          <t>Capacidad agéntica</t>
+        </is>
+      </c>
       <c r="L4" s="52" t="inlineStr">
         <is>
           <t>Talla</t>
@@ -1316,6 +1324,11 @@
         <v/>
       </c>
       <c r="I5" s="55" t="n"/>
+      <c r="J5" s="55" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
       <c r="L5" s="56" t="inlineStr">
         <is>
           <t>S</t>
@@ -1368,6 +1381,11 @@
         <v/>
       </c>
       <c r="I6" s="53" t="n"/>
+      <c r="J6" s="53" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
+        </is>
+      </c>
       <c r="L6" s="56" t="inlineStr">
         <is>
           <t>M</t>
@@ -1422,6 +1440,11 @@
       <c r="I7" s="105" t="inlineStr">
         <is>
           <t>Estimado acotado a los canales que el MVP habilita. La omnicanalidad sobre los ocho canales dibujados exige AVA y Nexo, que son de 2027.</t>
+        </is>
+      </c>
+      <c r="J7" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
         </is>
       </c>
       <c r="L7" s="56" t="inlineStr">
@@ -1479,6 +1502,11 @@
         <v/>
       </c>
       <c r="I8" s="53" t="n"/>
+      <c r="J8" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
       <c r="L8" s="56" t="inlineStr">
         <is>
           <t>XL</t>
@@ -1532,6 +1560,7 @@
           <t>🟥 No estimable como está redactado. Pide habilitar los cinco canales (Portal Prestador, SVP, AVA/Nexo, Super App, WhatsApp) para los tres públicos, pero el MVP 2026 habilita Portal Proveedor y SVP; AVA y Nexo son épicas de 2027. Acotar el requisito a los canales del MVP y volver a tallar.</t>
         </is>
       </c>
+      <c r="J9" s="53" t="n"/>
       <c r="L9" s="91" t="inlineStr">
         <is>
           <t>🟨 Escala de referencia (no oficial para todas las tallas): M ≈ 5 días (medio sprint) y L ≈ 10 días (1 sprint) están tomados literalmente del Acta de Estimación de Costo y Releases (21-ago-2026). S (≈3 días) y XL (≈20 días, el doble de L, por la regla de coherencia de tallaje de Víctor Martínez) son un supuesto para completar la escala — ajústelos si el equipo define otro valor. 1 sprint = 10 días hábiles (estándar SuraHis).</t>
@@ -1573,6 +1602,7 @@
         <v/>
       </c>
       <c r="I10" s="53" t="n"/>
+      <c r="J10" s="53" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="53" t="inlineStr">
@@ -1613,6 +1643,11 @@
         <v/>
       </c>
       <c r="I11" s="53" t="n"/>
+      <c r="J11" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="57" t="inlineStr">
@@ -1653,6 +1688,11 @@
         <v/>
       </c>
       <c r="I12" s="53" t="n"/>
+      <c r="J12" s="53" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="53" t="inlineStr">
@@ -1693,6 +1733,11 @@
         <v/>
       </c>
       <c r="I13" s="53" t="n"/>
+      <c r="J13" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
       <c r="L13" s="90" t="inlineStr">
         <is>
           <t>Referencia de Épicas (usada por la columna "¿En MVP?")</t>
@@ -1738,6 +1783,11 @@
         <v/>
       </c>
       <c r="I14" s="53" t="n"/>
+      <c r="J14" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
       <c r="L14" s="52" t="inlineStr">
         <is>
           <t>Épica / Gestor-Frente</t>
@@ -1812,6 +1862,11 @@
           <t>El dibujo del MVP ubica los extractores en la capa de agentes expertos del Gestor de Solicitud, no en Evaluación; RT-017 confirma que Evaluación consume lo ya extraído. La talla cubre los dos extractores del MVP (historia clínica y orden).</t>
         </is>
       </c>
+      <c r="J15" s="53" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
+        </is>
+      </c>
       <c r="L15" s="58" t="inlineStr">
         <is>
           <t>Gestor de Monitoreo (Torre de Control)</t>
@@ -1880,6 +1935,11 @@
         <v/>
       </c>
       <c r="I16" s="53" t="n"/>
+      <c r="J16" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
       <c r="L16" s="58" t="inlineStr">
         <is>
           <t>Interoperabilidad (Prestadores)</t>
@@ -1948,6 +2008,11 @@
         <v/>
       </c>
       <c r="I17" s="53" t="n"/>
+      <c r="J17" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
       <c r="L17" s="60" t="inlineStr">
         <is>
           <t>Gestor de Evaluación</t>
@@ -2016,6 +2081,11 @@
         <v/>
       </c>
       <c r="I18" s="53" t="n"/>
+      <c r="J18" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
       <c r="L18" s="60" t="inlineStr">
         <is>
           <t>Gestor de Solicitud</t>
@@ -2084,6 +2154,11 @@
         <v/>
       </c>
       <c r="I19" s="53" t="n"/>
+      <c r="J19" s="53" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
+        </is>
+      </c>
       <c r="L19" s="62" t="inlineStr">
         <is>
           <t>Gestor de Coordinación</t>
@@ -2148,6 +2223,7 @@
         <v/>
       </c>
       <c r="I20" s="53" t="n"/>
+      <c r="J20" s="53" t="n"/>
       <c r="L20" s="60" t="inlineStr">
         <is>
           <t>Canales / Front Externos</t>
@@ -2212,6 +2288,7 @@
         <v/>
       </c>
       <c r="I21" s="53" t="n"/>
+      <c r="J21" s="53" t="n"/>
       <c r="L21" s="60" t="inlineStr">
         <is>
           <t>Transversal / Principios generales</t>
@@ -2280,6 +2357,7 @@
           <t>🟥 No estimable: está redactado como una validación pendiente («Validar si se debe publicar eventos antes de generar la solicitud oficial»). El dibujo del MVP sí exige un evento por cada cambio de estado; falta decidir si se emite antes o después de la creación en el core.</t>
         </is>
       </c>
+      <c r="J22" s="53" t="n"/>
       <c r="L22" s="58" t="inlineStr">
         <is>
           <t>Gestor de Asignación</t>
@@ -2344,6 +2422,7 @@
         <v/>
       </c>
       <c r="I23" s="53" t="n"/>
+      <c r="J23" s="53" t="n"/>
       <c r="L23" s="60" t="inlineStr">
         <is>
           <t>Siniestro Integral</t>
@@ -2412,6 +2491,11 @@
         <v/>
       </c>
       <c r="I24" s="53" t="n"/>
+      <c r="J24" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
       <c r="L24" s="62" t="inlineStr">
         <is>
           <t>NEXO (Asesores)</t>
@@ -2482,6 +2566,11 @@
         <v/>
       </c>
       <c r="I25" s="53" t="n"/>
+      <c r="J25" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
       <c r="L25" s="62" t="inlineStr">
         <is>
           <t>Gestor de Prestación</t>
@@ -2554,6 +2643,11 @@
           <t>El dibujo lo resuelve: el dato se pide primero a SuraHis y la conexión directa solo se justifica si el core no lo tiene. La talla cubre el ajuste de la integración, no la decisión.</t>
         </is>
       </c>
+      <c r="J26" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
       <c r="L26" s="62" t="inlineStr">
         <is>
           <t>AVA (Asesores — AVA)</t>
@@ -2622,6 +2716,11 @@
         <v/>
       </c>
       <c r="I27" s="53" t="n"/>
+      <c r="J27" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
       <c r="L27" s="60" t="inlineStr">
         <is>
           <t>Transversal</t>
@@ -2690,6 +2789,11 @@
         <v/>
       </c>
       <c r="I28" s="53" t="n"/>
+      <c r="J28" s="53" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
+        </is>
+      </c>
       <c r="L28" s="62" t="inlineStr">
         <is>
           <t>Gestor de Finalización</t>
@@ -2758,6 +2862,11 @@
         <v/>
       </c>
       <c r="I29" s="53" t="n"/>
+      <c r="J29" s="53" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
       <c r="L29" s="62" t="inlineStr">
         <is>
           <t>Surahis</t>
@@ -2826,6 +2935,11 @@
         <v/>
       </c>
       <c r="I30" s="53" t="n"/>
+      <c r="J30" s="53" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="53" t="inlineStr">
@@ -2866,6 +2980,11 @@
         <v/>
       </c>
       <c r="I31" s="53" t="n"/>
+      <c r="J31" s="53" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
+        </is>
+      </c>
       <c r="L31" s="115" t="n"/>
       <c r="M31" s="115" t="n"/>
       <c r="N31" s="115" t="n"/>
@@ -2912,6 +3031,11 @@
         <v/>
       </c>
       <c r="I32" s="53" t="n"/>
+      <c r="J32" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
       <c r="L32" s="108" t="inlineStr">
         <is>
           <t>Leyenda y criterio de esta estimación (Tech and Solve)</t>
@@ -2962,6 +3086,11 @@
         <v/>
       </c>
       <c r="I33" s="53" t="n"/>
+      <c r="J33" s="53" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
+        </is>
+      </c>
       <c r="L33" s="116" t="inlineStr">
         <is>
           <t>Fila adicionada</t>
@@ -3008,6 +3137,7 @@
         <v/>
       </c>
       <c r="I34" s="53" t="n"/>
+      <c r="J34" s="53" t="n"/>
       <c r="L34" s="117" t="inlineStr">
         <is>
           <t>Alerta · sin tallar</t>
@@ -3054,6 +3184,7 @@
         <v/>
       </c>
       <c r="I35" s="53" t="n"/>
+      <c r="J35" s="53" t="n"/>
       <c r="L35" s="118" t="inlineStr">
         <is>
           <t>Fila modificada</t>
@@ -3100,6 +3231,7 @@
         <v/>
       </c>
       <c r="I36" s="53" t="n"/>
+      <c r="J36" s="53" t="n"/>
       <c r="L36" s="119" t="inlineStr">
         <is>
           <t>Talla diligenciada</t>
@@ -3146,6 +3278,7 @@
         <v/>
       </c>
       <c r="I37" s="53" t="n"/>
+      <c r="J37" s="53" t="n"/>
       <c r="L37" s="120" t="inlineStr">
         <is>
           <t>Sin color y sin talla</t>
@@ -3192,6 +3325,7 @@
         <v/>
       </c>
       <c r="I38" s="53" t="n"/>
+      <c r="J38" s="53" t="n"/>
       <c r="L38" s="115" t="n"/>
       <c r="M38" s="115" t="n"/>
       <c r="N38" s="115" t="n"/>
@@ -3234,6 +3368,7 @@
         <v/>
       </c>
       <c r="I39" s="53" t="n"/>
+      <c r="J39" s="53" t="n"/>
       <c r="L39" s="108" t="inlineStr">
         <is>
           <t>Resultado</t>
@@ -3280,6 +3415,7 @@
         <v/>
       </c>
       <c r="I40" s="53" t="n"/>
+      <c r="J40" s="53" t="n"/>
       <c r="L40" s="120" t="inlineStr">
         <is>
           <t>Suma y margen</t>
@@ -3326,6 +3462,7 @@
         <v/>
       </c>
       <c r="I41" s="53" t="n"/>
+      <c r="J41" s="53" t="n"/>
       <c r="L41" s="115" t="n"/>
       <c r="M41" s="115" t="n"/>
       <c r="N41" s="115" t="n"/>
@@ -3368,6 +3505,7 @@
         <v/>
       </c>
       <c r="I42" s="53" t="n"/>
+      <c r="J42" s="53" t="n"/>
       <c r="L42" s="108" t="inlineStr">
         <is>
           <t>Criterio de alcance</t>
@@ -3420,6 +3558,7 @@
         <v/>
       </c>
       <c r="I43" s="53" t="n"/>
+      <c r="J43" s="53" t="n"/>
       <c r="L43" s="120" t="inlineStr">
         <is>
           <t>Qué entra</t>
@@ -3466,6 +3605,7 @@
         <v/>
       </c>
       <c r="I44" s="53" t="n"/>
+      <c r="J44" s="53" t="n"/>
       <c r="L44" s="115" t="n"/>
       <c r="M44" s="115" t="n"/>
       <c r="N44" s="115" t="n"/>
@@ -3508,6 +3648,7 @@
         <v/>
       </c>
       <c r="I45" s="53" t="n"/>
+      <c r="J45" s="53" t="n"/>
       <c r="L45" s="108" t="inlineStr">
         <is>
           <t>Tres cosas que conviene saber antes de leer el total</t>
@@ -3554,6 +3695,7 @@
         <v/>
       </c>
       <c r="I46" s="53" t="n"/>
+      <c r="J46" s="53" t="n"/>
       <c r="L46" s="120" t="inlineStr">
         <is>
           <t>La escala se contradice</t>
@@ -3600,6 +3742,7 @@
         <v/>
       </c>
       <c r="I47" s="53" t="n"/>
+      <c r="J47" s="53" t="n"/>
       <c r="L47" s="120" t="inlineStr">
         <is>
           <t>Funcionales y técnicos se suman</t>
@@ -3646,6 +3789,7 @@
         <v/>
       </c>
       <c r="I48" s="53" t="n"/>
+      <c r="J48" s="53" t="n"/>
       <c r="L48" s="120" t="inlineStr">
         <is>
           <t>Mínimos del acta</t>
@@ -3692,6 +3836,7 @@
         <v/>
       </c>
       <c r="I49" s="53" t="n"/>
+      <c r="J49" s="53" t="n"/>
       <c r="L49" s="115" t="n"/>
       <c r="M49" s="115" t="n"/>
       <c r="N49" s="115" t="n"/>
@@ -3699,7 +3844,7 @@
       <c r="P49" s="115" t="n"/>
       <c r="Q49" s="115" t="n"/>
     </row>
-    <row r="50" ht="30" customHeight="1">
+    <row r="50">
       <c r="A50" s="57" t="inlineStr">
         <is>
           <t>RF-046</t>
@@ -3734,8 +3879,19 @@
         <v/>
       </c>
       <c r="I50" s="53" t="n"/>
-    </row>
-    <row r="51" ht="30" customHeight="1">
+      <c r="J50" s="53" t="n"/>
+      <c r="L50" s="108" t="inlineStr">
+        <is>
+          <t>Reparto por tipo de capacidad — solo requisitos del MVP</t>
+        </is>
+      </c>
+      <c r="M50" s="115" t="n"/>
+      <c r="N50" s="115" t="n"/>
+      <c r="O50" s="115" t="n"/>
+      <c r="P50" s="115" t="n"/>
+      <c r="Q50" s="115" t="n"/>
+    </row>
+    <row r="51">
       <c r="A51" s="53" t="inlineStr">
         <is>
           <t>RF-047</t>
@@ -3770,8 +3926,35 @@
         <v/>
       </c>
       <c r="I51" s="53" t="n"/>
-    </row>
-    <row r="52" ht="30" customHeight="1">
+      <c r="J51" s="53" t="n"/>
+      <c r="L51" s="51" t="inlineStr">
+        <is>
+          <t>Tipo de capacidad</t>
+        </is>
+      </c>
+      <c r="M51" s="51" t="inlineStr">
+        <is>
+          <t># Requisitos</t>
+        </is>
+      </c>
+      <c r="N51" s="51" t="inlineStr">
+        <is>
+          <t>Días</t>
+        </is>
+      </c>
+      <c r="O51" s="51" t="inlineStr">
+        <is>
+          <t>Sprints</t>
+        </is>
+      </c>
+      <c r="P51" s="51" t="inlineStr">
+        <is>
+          <t>% del MVP</t>
+        </is>
+      </c>
+      <c r="Q51" s="115" t="n"/>
+    </row>
+    <row r="52">
       <c r="A52" s="57" t="inlineStr">
         <is>
           <t>RF-048</t>
@@ -3810,8 +3993,35 @@
         <v/>
       </c>
       <c r="I52" s="53" t="n"/>
-    </row>
-    <row r="53" ht="30" customHeight="1">
+      <c r="J52" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="L52" s="114" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
+        </is>
+      </c>
+      <c r="M52" s="121">
+        <f>COUNTIF($J$5:$J$187,$L52)</f>
+        <v/>
+      </c>
+      <c r="N52" s="121">
+        <f>SUMIF($J$5:$J$187,$L52,$F$5:$F$187)</f>
+        <v/>
+      </c>
+      <c r="O52" s="121">
+        <f>IF($N52=0,0,$N52/10)</f>
+        <v/>
+      </c>
+      <c r="P52" s="122">
+        <f>IF($N$55=0,"",$N52/$N$55)</f>
+        <v/>
+      </c>
+      <c r="Q52" s="115" t="n"/>
+    </row>
+    <row r="53">
       <c r="A53" s="53" t="inlineStr">
         <is>
           <t>RF-049</t>
@@ -3846,8 +4056,31 @@
         <v/>
       </c>
       <c r="I53" s="53" t="n"/>
-    </row>
-    <row r="54" ht="30" customHeight="1">
+      <c r="J53" s="53" t="n"/>
+      <c r="L53" s="114" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
+      <c r="M53" s="121">
+        <f>COUNTIF($J$5:$J$187,$L53)</f>
+        <v/>
+      </c>
+      <c r="N53" s="121">
+        <f>SUMIF($J$5:$J$187,$L53,$F$5:$F$187)</f>
+        <v/>
+      </c>
+      <c r="O53" s="121">
+        <f>IF($N53=0,0,$N53/10)</f>
+        <v/>
+      </c>
+      <c r="P53" s="122">
+        <f>IF($N$55=0,"",$N53/$N$55)</f>
+        <v/>
+      </c>
+      <c r="Q53" s="115" t="n"/>
+    </row>
+    <row r="54">
       <c r="A54" s="57" t="inlineStr">
         <is>
           <t>RF-050</t>
@@ -3886,8 +4119,35 @@
         <v/>
       </c>
       <c r="I54" s="53" t="n"/>
-    </row>
-    <row r="55" ht="30" customHeight="1">
+      <c r="J54" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="L54" s="114" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
+      <c r="M54" s="121">
+        <f>COUNTIF($J$5:$J$187,$L54)</f>
+        <v/>
+      </c>
+      <c r="N54" s="121">
+        <f>SUMIF($J$5:$J$187,$L54,$F$5:$F$187)</f>
+        <v/>
+      </c>
+      <c r="O54" s="121">
+        <f>IF($N54=0,0,$N54/10)</f>
+        <v/>
+      </c>
+      <c r="P54" s="122">
+        <f>IF($N$55=0,"",$N54/$N$55)</f>
+        <v/>
+      </c>
+      <c r="Q54" s="115" t="n"/>
+    </row>
+    <row r="55">
       <c r="A55" s="53" t="inlineStr">
         <is>
           <t>RF-051</t>
@@ -3922,8 +4182,28 @@
         <v/>
       </c>
       <c r="I55" s="53" t="n"/>
-    </row>
-    <row r="56" ht="30" customHeight="1">
+      <c r="J55" s="53" t="n"/>
+      <c r="L55" s="114" t="inlineStr">
+        <is>
+          <t>Total MVP</t>
+        </is>
+      </c>
+      <c r="M55" s="114">
+        <f>SUM($M$52:$M$54)</f>
+        <v/>
+      </c>
+      <c r="N55" s="114">
+        <f>SUM($N$52:$N$54)</f>
+        <v/>
+      </c>
+      <c r="O55" s="114">
+        <f>IF($N$55=0,0,$N$55/10)</f>
+        <v/>
+      </c>
+      <c r="P55" s="115" t="n"/>
+      <c r="Q55" s="115" t="n"/>
+    </row>
+    <row r="56">
       <c r="A56" s="57" t="inlineStr">
         <is>
           <t>RF-052</t>
@@ -3958,8 +4238,15 @@
         <v/>
       </c>
       <c r="I56" s="53" t="n"/>
-    </row>
-    <row r="57" ht="30" customHeight="1">
+      <c r="J56" s="53" t="n"/>
+      <c r="L56" s="115" t="n"/>
+      <c r="M56" s="115" t="n"/>
+      <c r="N56" s="115" t="n"/>
+      <c r="O56" s="115" t="n"/>
+      <c r="P56" s="115" t="n"/>
+      <c r="Q56" s="115" t="n"/>
+    </row>
+    <row r="57" ht="64" customHeight="1">
       <c r="A57" s="53" t="inlineStr">
         <is>
           <t>RF-053</t>
@@ -3994,6 +4281,17 @@
         <v/>
       </c>
       <c r="I57" s="53" t="n"/>
+      <c r="J57" s="53" t="n"/>
+      <c r="L57" s="114" t="inlineStr">
+        <is>
+          <t>Cómo leer el filtro</t>
+        </is>
+      </c>
+      <c r="M57" s="110" t="inlineStr">
+        <is>
+          <t>La columna J clasifica cada requisito del MVP con la convención del propio dibujo. «Agéntica»: el requisito construye o define el comportamiento de un agente que razona con un modelo —clasificador, enrutador, request builder, LLM-as-a-judge, extractores, pertinencia médica, duplicidad, auditor—. «Habilitadora»: no es un agente, pero sin ella no hay autonomía gobernada —golden set, compuerta de promoción, umbrales y techos, traza de la decisión, calibración del juez—. «Determinística»: reglas duras, APIs, integraciones, almacenamiento, front y contrato de eventos. Las filas sin talla quedan en blanco porque están fuera del MVP. Filtre por la columna «Capacidad agéntica» en el encabezado.</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="105" t="inlineStr">
@@ -4036,6 +4334,11 @@
       <c r="I58" s="105" t="inlineStr">
         <is>
           <t>Entra la detección de solicitudes repetidas, que el dibujo resuelve en la capa de duplicidad. La talla cubre solo eso: el flujo de rescate que el requisito invoca (RF-019) y la notificación al asegurado quedan fuera del MVP, así que el requisito no se cumple completo con esta talla.</t>
+        </is>
+      </c>
+      <c r="J58" s="53" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
         </is>
       </c>
     </row>
@@ -4074,6 +4377,7 @@
         <v/>
       </c>
       <c r="I59" s="53" t="n"/>
+      <c r="J59" s="53" t="n"/>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="57" t="inlineStr">
@@ -4110,6 +4414,7 @@
         <v/>
       </c>
       <c r="I60" s="53" t="n"/>
+      <c r="J60" s="53" t="n"/>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="53" t="inlineStr">
@@ -4150,6 +4455,11 @@
         <v/>
       </c>
       <c r="I61" s="53" t="n"/>
+      <c r="J61" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="105" t="inlineStr">
@@ -4192,6 +4502,11 @@
       <c r="I62" s="105" t="inlineStr">
         <is>
           <t>Entra la parte del front: no exigir la selección de prestador en la solicitud inicial. Sugerir el prestador es del Gestor de Coordinación, que queda fuera del MVP.</t>
+        </is>
+      </c>
+      <c r="J62" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
         </is>
       </c>
     </row>
@@ -4230,6 +4545,7 @@
         <v/>
       </c>
       <c r="I63" s="53" t="n"/>
+      <c r="J63" s="53" t="n"/>
     </row>
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="57" t="inlineStr">
@@ -4266,6 +4582,7 @@
         <v/>
       </c>
       <c r="I64" s="53" t="n"/>
+      <c r="J64" s="53" t="n"/>
     </row>
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="53" t="inlineStr">
@@ -4302,6 +4619,7 @@
         <v/>
       </c>
       <c r="I65" s="53" t="n"/>
+      <c r="J65" s="53" t="n"/>
     </row>
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="57" t="inlineStr">
@@ -4338,6 +4656,7 @@
         <v/>
       </c>
       <c r="I66" s="53" t="n"/>
+      <c r="J66" s="53" t="n"/>
     </row>
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="53" t="inlineStr">
@@ -4374,6 +4693,7 @@
         <v/>
       </c>
       <c r="I67" s="53" t="n"/>
+      <c r="J67" s="53" t="n"/>
     </row>
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="57" t="inlineStr">
@@ -4410,6 +4730,7 @@
         <v/>
       </c>
       <c r="I68" s="53" t="n"/>
+      <c r="J68" s="53" t="n"/>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="53" t="inlineStr">
@@ -4446,6 +4767,7 @@
         <v/>
       </c>
       <c r="I69" s="53" t="n"/>
+      <c r="J69" s="53" t="n"/>
     </row>
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="57" t="inlineStr">
@@ -4482,6 +4804,7 @@
         <v/>
       </c>
       <c r="I70" s="53" t="n"/>
+      <c r="J70" s="53" t="n"/>
     </row>
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="53" t="inlineStr">
@@ -4518,6 +4841,7 @@
         <v/>
       </c>
       <c r="I71" s="53" t="n"/>
+      <c r="J71" s="53" t="n"/>
     </row>
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="57" t="inlineStr">
@@ -4554,6 +4878,7 @@
         <v/>
       </c>
       <c r="I72" s="53" t="n"/>
+      <c r="J72" s="53" t="n"/>
     </row>
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="53" t="inlineStr">
@@ -4590,6 +4915,7 @@
         <v/>
       </c>
       <c r="I73" s="53" t="n"/>
+      <c r="J73" s="53" t="n"/>
     </row>
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="105" t="inlineStr">
@@ -4632,6 +4958,11 @@
       <c r="I74" s="105" t="inlineStr">
         <is>
           <t>Entra el principio de acceso al dato vía el core, que el dibujo del MVP recoge explícitamente. La interoperabilidad de autorizaciones como tal queda fuera.</t>
+        </is>
+      </c>
+      <c r="J74" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
         </is>
       </c>
     </row>
@@ -4670,6 +5001,7 @@
         <v/>
       </c>
       <c r="I75" s="53" t="n"/>
+      <c r="J75" s="53" t="n"/>
     </row>
     <row r="76" ht="30" customHeight="1">
       <c r="A76" s="57" t="inlineStr">
@@ -4706,6 +5038,7 @@
         <v/>
       </c>
       <c r="I76" s="53" t="n"/>
+      <c r="J76" s="53" t="n"/>
     </row>
     <row r="77" ht="30" customHeight="1">
       <c r="A77" s="53" t="inlineStr">
@@ -4742,6 +5075,7 @@
         <v/>
       </c>
       <c r="I77" s="53" t="n"/>
+      <c r="J77" s="53" t="n"/>
     </row>
     <row r="78" ht="30" customHeight="1">
       <c r="A78" s="57" t="inlineStr">
@@ -4778,6 +5112,7 @@
         <v/>
       </c>
       <c r="I78" s="53" t="n"/>
+      <c r="J78" s="53" t="n"/>
     </row>
     <row r="79" ht="30" customHeight="1">
       <c r="A79" s="53" t="inlineStr">
@@ -4814,6 +5149,7 @@
         <v/>
       </c>
       <c r="I79" s="53" t="n"/>
+      <c r="J79" s="53" t="n"/>
     </row>
     <row r="80" ht="30" customHeight="1">
       <c r="A80" s="57" t="inlineStr">
@@ -4850,6 +5186,7 @@
         <v/>
       </c>
       <c r="I80" s="53" t="n"/>
+      <c r="J80" s="53" t="n"/>
     </row>
     <row r="81" ht="30" customHeight="1">
       <c r="A81" s="106" t="inlineStr">
@@ -4890,6 +5227,7 @@
           <t>🟥 No estimable: las reglas de visibilidad entre prestadores están señaladas en la propia hoja como decisión importante sin dueño. Definir la regla antes de tallar.</t>
         </is>
       </c>
+      <c r="J81" s="53" t="n"/>
     </row>
     <row r="82" ht="30" customHeight="1">
       <c r="A82" s="57" t="inlineStr">
@@ -4926,6 +5264,7 @@
         <v/>
       </c>
       <c r="I82" s="53" t="n"/>
+      <c r="J82" s="53" t="n"/>
     </row>
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="53" t="inlineStr">
@@ -4962,6 +5301,7 @@
         <v/>
       </c>
       <c r="I83" s="53" t="n"/>
+      <c r="J83" s="53" t="n"/>
     </row>
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="57" t="inlineStr">
@@ -4998,6 +5338,7 @@
         <v/>
       </c>
       <c r="I84" s="53" t="n"/>
+      <c r="J84" s="53" t="n"/>
     </row>
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="53" t="inlineStr">
@@ -5034,6 +5375,7 @@
         <v/>
       </c>
       <c r="I85" s="53" t="n"/>
+      <c r="J85" s="53" t="n"/>
     </row>
     <row r="86" ht="30" customHeight="1">
       <c r="A86" s="57" t="inlineStr">
@@ -5070,6 +5412,7 @@
         <v/>
       </c>
       <c r="I86" s="53" t="n"/>
+      <c r="J86" s="53" t="n"/>
     </row>
     <row r="87" ht="30" customHeight="1">
       <c r="A87" s="53" t="inlineStr">
@@ -5106,6 +5449,7 @@
         <v/>
       </c>
       <c r="I87" s="53" t="n"/>
+      <c r="J87" s="53" t="n"/>
     </row>
     <row r="88" ht="30" customHeight="1">
       <c r="A88" s="57" t="inlineStr">
@@ -5142,6 +5486,7 @@
         <v/>
       </c>
       <c r="I88" s="53" t="n"/>
+      <c r="J88" s="53" t="n"/>
     </row>
     <row r="89" ht="30" customHeight="1">
       <c r="A89" s="53" t="inlineStr">
@@ -5178,6 +5523,7 @@
         <v/>
       </c>
       <c r="I89" s="53" t="n"/>
+      <c r="J89" s="53" t="n"/>
     </row>
     <row r="90" ht="30" customHeight="1">
       <c r="A90" s="57" t="inlineStr">
@@ -5218,6 +5564,11 @@
         <v/>
       </c>
       <c r="I90" s="53" t="n"/>
+      <c r="J90" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="30" customHeight="1">
       <c r="A91" s="53" t="inlineStr">
@@ -5254,6 +5605,7 @@
         <v/>
       </c>
       <c r="I91" s="53" t="n"/>
+      <c r="J91" s="53" t="n"/>
     </row>
     <row r="92" ht="30" customHeight="1">
       <c r="A92" s="57" t="inlineStr">
@@ -5290,6 +5642,7 @@
         <v/>
       </c>
       <c r="I92" s="53" t="n"/>
+      <c r="J92" s="53" t="n"/>
     </row>
     <row r="93" ht="30" customHeight="1">
       <c r="A93" s="53" t="inlineStr">
@@ -5326,6 +5679,7 @@
         <v/>
       </c>
       <c r="I93" s="53" t="n"/>
+      <c r="J93" s="53" t="n"/>
     </row>
     <row r="94" ht="30" customHeight="1">
       <c r="A94" s="57" t="inlineStr">
@@ -5362,6 +5716,7 @@
         <v/>
       </c>
       <c r="I94" s="53" t="n"/>
+      <c r="J94" s="53" t="n"/>
     </row>
     <row r="95" ht="30" customHeight="1">
       <c r="A95" s="53" t="inlineStr">
@@ -5398,6 +5753,7 @@
         <v/>
       </c>
       <c r="I95" s="53" t="n"/>
+      <c r="J95" s="53" t="n"/>
     </row>
     <row r="96" ht="30" customHeight="1">
       <c r="A96" s="57" t="inlineStr">
@@ -5434,6 +5790,7 @@
         <v/>
       </c>
       <c r="I96" s="53" t="n"/>
+      <c r="J96" s="53" t="n"/>
     </row>
     <row r="97" ht="30" customHeight="1">
       <c r="A97" s="53" t="inlineStr">
@@ -5470,6 +5827,7 @@
         <v/>
       </c>
       <c r="I97" s="53" t="n"/>
+      <c r="J97" s="53" t="n"/>
     </row>
     <row r="98" ht="30" customHeight="1">
       <c r="A98" s="57" t="inlineStr">
@@ -5506,6 +5864,7 @@
         <v/>
       </c>
       <c r="I98" s="53" t="n"/>
+      <c r="J98" s="53" t="n"/>
     </row>
     <row r="99" ht="30" customHeight="1">
       <c r="A99" s="53" t="inlineStr">
@@ -5542,6 +5901,7 @@
         <v/>
       </c>
       <c r="I99" s="53" t="n"/>
+      <c r="J99" s="53" t="n"/>
     </row>
     <row r="100" ht="30" customHeight="1">
       <c r="A100" s="57" t="inlineStr">
@@ -5578,6 +5938,7 @@
         <v/>
       </c>
       <c r="I100" s="53" t="n"/>
+      <c r="J100" s="53" t="n"/>
     </row>
     <row r="101" ht="30" customHeight="1">
       <c r="A101" s="105" t="inlineStr">
@@ -5620,6 +5981,11 @@
       <c r="I101" s="105" t="inlineStr">
         <is>
           <t>Entra el agente auditor dentro de cada gestor, que el dibujo del MVP incluye en Solicitud y en Evaluación. El auditor de la torre es capa 3 y queda fuera.</t>
+        </is>
+      </c>
+      <c r="J101" s="53" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
         </is>
       </c>
     </row>
@@ -5658,6 +6024,7 @@
         <v/>
       </c>
       <c r="I102" s="53" t="n"/>
+      <c r="J102" s="53" t="n"/>
     </row>
     <row r="103" ht="30" customHeight="1">
       <c r="A103" s="53" t="inlineStr">
@@ -5694,6 +6061,7 @@
         <v/>
       </c>
       <c r="I103" s="53" t="n"/>
+      <c r="J103" s="53" t="n"/>
     </row>
     <row r="104" ht="30" customHeight="1">
       <c r="A104" s="57" t="inlineStr">
@@ -5730,6 +6098,7 @@
         <v/>
       </c>
       <c r="I104" s="53" t="n"/>
+      <c r="J104" s="53" t="n"/>
     </row>
     <row r="105" ht="30" customHeight="1">
       <c r="A105" s="53" t="inlineStr">
@@ -5766,6 +6135,7 @@
         <v/>
       </c>
       <c r="I105" s="53" t="n"/>
+      <c r="J105" s="53" t="n"/>
     </row>
     <row r="106" ht="30" customHeight="1">
       <c r="A106" s="57" t="inlineStr">
@@ -5802,6 +6172,7 @@
         <v/>
       </c>
       <c r="I106" s="53" t="n"/>
+      <c r="J106" s="53" t="n"/>
     </row>
     <row r="107" ht="30" customHeight="1">
       <c r="A107" s="53" t="inlineStr">
@@ -5838,6 +6209,7 @@
         <v/>
       </c>
       <c r="I107" s="53" t="n"/>
+      <c r="J107" s="53" t="n"/>
     </row>
     <row r="108" ht="30" customHeight="1">
       <c r="A108" s="57" t="inlineStr">
@@ -5874,6 +6246,7 @@
         <v/>
       </c>
       <c r="I108" s="53" t="n"/>
+      <c r="J108" s="53" t="n"/>
     </row>
     <row r="109" ht="30" customHeight="1">
       <c r="A109" s="53" t="inlineStr">
@@ -5910,6 +6283,7 @@
         <v/>
       </c>
       <c r="I109" s="53" t="n"/>
+      <c r="J109" s="53" t="n"/>
     </row>
     <row r="110" ht="30" customHeight="1">
       <c r="A110" s="57" t="inlineStr">
@@ -5946,6 +6320,7 @@
         <v/>
       </c>
       <c r="I110" s="53" t="n"/>
+      <c r="J110" s="53" t="n"/>
     </row>
     <row r="111" ht="30" customHeight="1">
       <c r="A111" s="53" t="inlineStr">
@@ -5982,6 +6357,7 @@
         <v/>
       </c>
       <c r="I111" s="53" t="n"/>
+      <c r="J111" s="53" t="n"/>
     </row>
     <row r="112" ht="30" customHeight="1">
       <c r="A112" s="57" t="inlineStr">
@@ -6018,6 +6394,7 @@
         <v/>
       </c>
       <c r="I112" s="53" t="n"/>
+      <c r="J112" s="53" t="n"/>
     </row>
     <row r="113" ht="30" customHeight="1">
       <c r="A113" s="53" t="inlineStr">
@@ -6058,6 +6435,11 @@
         <v/>
       </c>
       <c r="I113" s="53" t="n"/>
+      <c r="J113" s="53" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="30" customHeight="1">
       <c r="A114" s="57" t="inlineStr">
@@ -6098,6 +6480,11 @@
         <v/>
       </c>
       <c r="I114" s="53" t="n"/>
+      <c r="J114" s="53" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="30" customHeight="1">
       <c r="A115" s="106" t="inlineStr">
@@ -6138,6 +6525,7 @@
           <t>🟥 No es un entregable de construcción sino una premisa de riesgo del proyecto. No se talla; se gestiona como dependencia externa de los cores.</t>
         </is>
       </c>
+      <c r="J115" s="53" t="n"/>
     </row>
     <row r="116" ht="30" customHeight="1">
       <c r="A116" s="57" t="inlineStr">
@@ -6178,6 +6566,11 @@
         <v/>
       </c>
       <c r="I116" s="53" t="n"/>
+      <c r="J116" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="30" customHeight="1">
       <c r="A117" s="53" t="inlineStr">
@@ -6218,6 +6611,11 @@
         <v/>
       </c>
       <c r="I117" s="53" t="n"/>
+      <c r="J117" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="30" customHeight="1">
       <c r="A118" s="57" t="inlineStr">
@@ -6258,6 +6656,11 @@
         <v/>
       </c>
       <c r="I118" s="53" t="n"/>
+      <c r="J118" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="30" customHeight="1">
       <c r="A119" s="53" t="inlineStr">
@@ -6298,6 +6701,11 @@
         <v/>
       </c>
       <c r="I119" s="53" t="n"/>
+      <c r="J119" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="30" customHeight="1">
       <c r="A120" s="105" t="inlineStr">
@@ -6342,6 +6750,11 @@
           <t>El equipo confirmó Angular, con lo que se cierra el conflicto: coincide con lo que fija el lineamiento AI First, «La experiencia conversacional se materializa en una Static Web App basada en Angular SPA» (Arquitectura de implementación, página 6243680318). La talla cubre el front nuevo embebido en los dos canales del MVP, Portal Proveedor y SVP; AVA es 2027 y no está incluida.</t>
         </is>
       </c>
+      <c r="J120" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="30" customHeight="1">
       <c r="A121" s="53" t="inlineStr">
@@ -6382,6 +6795,11 @@
         <v/>
       </c>
       <c r="I121" s="53" t="n"/>
+      <c r="J121" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="30" customHeight="1">
       <c r="A122" s="57" t="inlineStr">
@@ -6422,6 +6840,11 @@
         <v/>
       </c>
       <c r="I122" s="53" t="n"/>
+      <c r="J122" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="30" customHeight="1">
       <c r="A123" s="53" t="inlineStr">
@@ -6462,6 +6885,11 @@
         <v/>
       </c>
       <c r="I123" s="53" t="n"/>
+      <c r="J123" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="30" customHeight="1">
       <c r="A124" s="106" t="inlineStr">
@@ -6502,6 +6930,7 @@
           <t>🟥 Conflicto con el lineamiento. El requisito dice que un LLM multimodal interpreta los documentos directamente; el stack v0.5 declara Azure Document Intelligence obligatorio para OCR y extracción estructurada (Diseño Datos RAG/Knowledge/Memory, página 5900140571). El esfuerzo cambia según cuál se adopte.</t>
         </is>
       </c>
+      <c r="J124" s="53" t="n"/>
     </row>
     <row r="125" ht="30" customHeight="1">
       <c r="A125" s="53" t="inlineStr">
@@ -6542,6 +6971,11 @@
         <v/>
       </c>
       <c r="I125" s="53" t="n"/>
+      <c r="J125" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="30" customHeight="1">
       <c r="A126" s="57" t="inlineStr">
@@ -6578,6 +7012,7 @@
         <v/>
       </c>
       <c r="I126" s="53" t="n"/>
+      <c r="J126" s="53" t="n"/>
     </row>
     <row r="127" ht="30" customHeight="1">
       <c r="A127" s="53" t="inlineStr">
@@ -6618,6 +7053,11 @@
         <v/>
       </c>
       <c r="I127" s="53" t="n"/>
+      <c r="J127" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="30" customHeight="1">
       <c r="A128" s="106" t="inlineStr">
@@ -6658,6 +7098,7 @@
           <t>🟥 Riesgo abierto, no entregable: la Super App opera en Google Cloud y el resto del ecosistema en Azure. Afecta a dos canales dibujados en el MVP. Requiere decisión de arquitectura antes de poder tallarlo.</t>
         </is>
       </c>
+      <c r="J128" s="53" t="n"/>
     </row>
     <row r="129" ht="30" customHeight="1">
       <c r="A129" s="53" t="inlineStr">
@@ -6698,6 +7139,11 @@
         <v/>
       </c>
       <c r="I129" s="53" t="n"/>
+      <c r="J129" s="53" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="30" customHeight="1">
       <c r="A130" s="57" t="inlineStr">
@@ -6738,6 +7184,11 @@
         <v/>
       </c>
       <c r="I130" s="53" t="n"/>
+      <c r="J130" s="53" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="30" customHeight="1">
       <c r="A131" s="106" t="inlineStr">
@@ -6778,6 +7229,7 @@
           <t>🟥 Duplicado exacto de RT-018. Se deja sin tallar para no contar dos veces el mismo esfuerzo; conviene eliminarlo o diferenciarlo.</t>
         </is>
       </c>
+      <c r="J131" s="53" t="n"/>
     </row>
     <row r="132" ht="30" customHeight="1">
       <c r="A132" s="57" t="inlineStr">
@@ -6818,6 +7270,11 @@
         <v/>
       </c>
       <c r="I132" s="53" t="n"/>
+      <c r="J132" s="53" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="30" customHeight="1">
       <c r="A133" s="53" t="inlineStr">
@@ -6858,6 +7315,11 @@
         <v/>
       </c>
       <c r="I133" s="53" t="n"/>
+      <c r="J133" s="53" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="30" customHeight="1">
       <c r="A134" s="57" t="inlineStr">
@@ -6894,6 +7356,7 @@
         <v/>
       </c>
       <c r="I134" s="53" t="n"/>
+      <c r="J134" s="53" t="n"/>
     </row>
     <row r="135" ht="30" customHeight="1">
       <c r="A135" s="53" t="inlineStr">
@@ -6930,6 +7393,7 @@
         <v/>
       </c>
       <c r="I135" s="53" t="n"/>
+      <c r="J135" s="53" t="n"/>
     </row>
     <row r="136" ht="30" customHeight="1">
       <c r="A136" s="57" t="inlineStr">
@@ -6966,6 +7430,7 @@
         <v/>
       </c>
       <c r="I136" s="53" t="n"/>
+      <c r="J136" s="53" t="n"/>
     </row>
     <row r="137" ht="30" customHeight="1">
       <c r="A137" s="53" t="inlineStr">
@@ -7002,6 +7467,7 @@
         <v/>
       </c>
       <c r="I137" s="53" t="n"/>
+      <c r="J137" s="53" t="n"/>
     </row>
     <row r="138" ht="30" customHeight="1">
       <c r="A138" s="57" t="inlineStr">
@@ -7038,6 +7504,7 @@
         <v/>
       </c>
       <c r="I138" s="53" t="n"/>
+      <c r="J138" s="53" t="n"/>
     </row>
     <row r="139" ht="30" customHeight="1">
       <c r="A139" s="53" t="inlineStr">
@@ -7074,6 +7541,7 @@
         <v/>
       </c>
       <c r="I139" s="53" t="n"/>
+      <c r="J139" s="53" t="n"/>
     </row>
     <row r="140" ht="30" customHeight="1">
       <c r="A140" s="57" t="inlineStr">
@@ -7110,6 +7578,7 @@
         <v/>
       </c>
       <c r="I140" s="53" t="n"/>
+      <c r="J140" s="53" t="n"/>
     </row>
     <row r="141" ht="30" customHeight="1">
       <c r="A141" s="53" t="inlineStr">
@@ -7146,6 +7615,7 @@
         <v/>
       </c>
       <c r="I141" s="53" t="n"/>
+      <c r="J141" s="53" t="n"/>
     </row>
     <row r="142" ht="30" customHeight="1">
       <c r="A142" s="57" t="inlineStr">
@@ -7186,6 +7656,11 @@
         <v/>
       </c>
       <c r="I142" s="53" t="n"/>
+      <c r="J142" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="30" customHeight="1">
       <c r="A143" s="53" t="inlineStr">
@@ -7226,6 +7701,11 @@
         <v/>
       </c>
       <c r="I143" s="53" t="n"/>
+      <c r="J143" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="144" ht="30" customHeight="1">
       <c r="A144" s="57" t="inlineStr">
@@ -7262,6 +7742,7 @@
         <v/>
       </c>
       <c r="I144" s="53" t="n"/>
+      <c r="J144" s="53" t="n"/>
     </row>
     <row r="145" ht="30" customHeight="1">
       <c r="A145" s="53" t="inlineStr">
@@ -7298,6 +7779,7 @@
         <v/>
       </c>
       <c r="I145" s="53" t="n"/>
+      <c r="J145" s="53" t="n"/>
     </row>
     <row r="146" ht="30" customHeight="1">
       <c r="A146" s="57" t="inlineStr">
@@ -7334,6 +7816,7 @@
         <v/>
       </c>
       <c r="I146" s="53" t="n"/>
+      <c r="J146" s="53" t="n"/>
     </row>
     <row r="147" ht="30" customHeight="1">
       <c r="A147" s="53" t="inlineStr">
@@ -7370,6 +7853,7 @@
         <v/>
       </c>
       <c r="I147" s="53" t="n"/>
+      <c r="J147" s="53" t="n"/>
     </row>
     <row r="148" ht="30" customHeight="1">
       <c r="A148" s="57" t="inlineStr">
@@ -7406,6 +7890,7 @@
         <v/>
       </c>
       <c r="I148" s="53" t="n"/>
+      <c r="J148" s="53" t="n"/>
     </row>
     <row r="149" ht="30" customHeight="1">
       <c r="A149" s="106" t="inlineStr">
@@ -7446,6 +7931,7 @@
           <t>🟥 No es un entregable de construcción: es la regla de presentación de la estimación (declarar un 30% de incertidumbre ante patrocinadores). El equipo decidió estimar sin aplicar ese margen, así que la suma de esta hoja va sin él. No se talla.</t>
         </is>
       </c>
+      <c r="J149" s="53" t="n"/>
     </row>
     <row r="150" ht="30" customHeight="1">
       <c r="A150" s="106" t="inlineStr">
@@ -7486,6 +7972,7 @@
           <t>🟥 No es un entregable: es la propia escala de tallaje que usa esta hoja (M≈5, L≈10, XL≈20). Aplica a este ejercicio, no se talla.</t>
         </is>
       </c>
+      <c r="J150" s="53" t="n"/>
     </row>
     <row r="151" ht="30" customHeight="1">
       <c r="A151" s="53" t="inlineStr">
@@ -7522,6 +8009,7 @@
         <v/>
       </c>
       <c r="I151" s="53" t="n"/>
+      <c r="J151" s="53" t="n"/>
     </row>
     <row r="152" ht="30" customHeight="1">
       <c r="A152" s="57" t="inlineStr">
@@ -7558,6 +8046,7 @@
         <v/>
       </c>
       <c r="I152" s="53" t="n"/>
+      <c r="J152" s="53" t="n"/>
     </row>
     <row r="153" ht="30" customHeight="1">
       <c r="A153" s="53" t="inlineStr">
@@ -7594,6 +8083,7 @@
         <v/>
       </c>
       <c r="I153" s="53" t="n"/>
+      <c r="J153" s="53" t="n"/>
     </row>
     <row r="154" ht="30" customHeight="1">
       <c r="A154" s="57" t="inlineStr">
@@ -7630,6 +8120,7 @@
         <v/>
       </c>
       <c r="I154" s="53" t="n"/>
+      <c r="J154" s="53" t="n"/>
     </row>
     <row r="155" ht="30" customHeight="1">
       <c r="A155" s="106" t="inlineStr">
@@ -7670,6 +8161,7 @@
           <t>🟥 No estimable como desarrollo: es dimensionamiento de infraestructura de Siniestro Integral por crecimiento transaccional. Necesita el volumen esperado para poder dimensionarse.</t>
         </is>
       </c>
+      <c r="J155" s="53" t="n"/>
     </row>
     <row r="156" ht="30" customHeight="1">
       <c r="A156" s="57" t="inlineStr">
@@ -7710,6 +8202,11 @@
         <v/>
       </c>
       <c r="I156" s="53" t="n"/>
+      <c r="J156" s="53" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
     </row>
     <row r="157" ht="30" customHeight="1">
       <c r="A157" s="105" t="inlineStr">
@@ -7752,6 +8249,11 @@
       <c r="I157" s="105" t="inlineStr">
         <is>
           <t>El equipo confirmó Angular. La talla cubre solo la diferenciación por rol del web component único —el prestador suma 2 o 3 campos frente al cliente—, porque la decisión del front único reutilizable ya está tallada en RT-006 y no se cuenta dos veces.</t>
+        </is>
+      </c>
+      <c r="J157" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
         </is>
       </c>
     </row>
@@ -7790,6 +8292,7 @@
         <v/>
       </c>
       <c r="I158" s="53" t="n"/>
+      <c r="J158" s="53" t="n"/>
     </row>
     <row r="159" ht="30" customHeight="1">
       <c r="A159" s="53" t="inlineStr">
@@ -7826,6 +8329,7 @@
         <v/>
       </c>
       <c r="I159" s="53" t="n"/>
+      <c r="J159" s="53" t="n"/>
     </row>
     <row r="160" ht="30" customHeight="1">
       <c r="A160" s="57" t="inlineStr">
@@ -7862,6 +8366,7 @@
         <v/>
       </c>
       <c r="I160" s="53" t="n"/>
+      <c r="J160" s="53" t="n"/>
     </row>
     <row r="161" ht="30" customHeight="1">
       <c r="A161" s="53" t="inlineStr">
@@ -7898,6 +8403,7 @@
         <v/>
       </c>
       <c r="I161" s="53" t="n"/>
+      <c r="J161" s="53" t="n"/>
     </row>
     <row r="162" ht="30" customHeight="1">
       <c r="A162" s="57" t="inlineStr">
@@ -7938,6 +8444,11 @@
         <v/>
       </c>
       <c r="I162" s="53" t="n"/>
+      <c r="J162" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="163" ht="30" customHeight="1">
       <c r="A163" s="106" t="inlineStr">
@@ -7978,6 +8489,7 @@
           <t>🟥 El propio requisito dice que el nivel de autonomía de cada agente está «pendiente de definir antes de dimensionar el desarrollo». Se respeta: no se talla hasta que se defina.</t>
         </is>
       </c>
+      <c r="J163" s="53" t="n"/>
     </row>
     <row r="164" ht="30" customHeight="1">
       <c r="A164" s="57" t="inlineStr">
@@ -8018,6 +8530,11 @@
         <v/>
       </c>
       <c r="I164" s="53" t="n"/>
+      <c r="J164" s="53" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
     </row>
     <row r="165" ht="30" customHeight="1">
       <c r="A165" s="53" t="inlineStr">
@@ -8058,6 +8575,11 @@
         <v/>
       </c>
       <c r="I165" s="53" t="n"/>
+      <c r="J165" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="166" ht="30" customHeight="1">
       <c r="A166" s="57" t="inlineStr">
@@ -8098,6 +8620,11 @@
         <v/>
       </c>
       <c r="I166" s="53" t="n"/>
+      <c r="J166" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="167" ht="30" customHeight="1">
       <c r="A167" s="98" t="inlineStr">
@@ -8138,6 +8665,11 @@
         <v/>
       </c>
       <c r="I167" s="98" t="n"/>
+      <c r="J167" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="168" ht="30" customHeight="1">
       <c r="A168" s="98" t="inlineStr">
@@ -8178,6 +8710,11 @@
         <v/>
       </c>
       <c r="I168" s="98" t="n"/>
+      <c r="J168" s="53" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
+        </is>
+      </c>
     </row>
     <row r="169" ht="30" customHeight="1">
       <c r="A169" s="98" t="inlineStr">
@@ -8218,6 +8755,11 @@
         <v/>
       </c>
       <c r="I169" s="98" t="n"/>
+      <c r="J169" s="53" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
+        </is>
+      </c>
     </row>
     <row r="170" ht="30" customHeight="1">
       <c r="A170" s="98" t="inlineStr">
@@ -8258,6 +8800,11 @@
         <v/>
       </c>
       <c r="I170" s="98" t="n"/>
+      <c r="J170" s="53" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
+        </is>
+      </c>
     </row>
     <row r="171" ht="30" customHeight="1">
       <c r="A171" s="98" t="inlineStr">
@@ -8298,6 +8845,11 @@
         <v/>
       </c>
       <c r="I171" s="98" t="n"/>
+      <c r="J171" s="53" t="inlineStr">
+        <is>
+          <t>Agéntica</t>
+        </is>
+      </c>
     </row>
     <row r="172" ht="30" customHeight="1">
       <c r="A172" s="98" t="inlineStr">
@@ -8338,6 +8890,11 @@
         <v/>
       </c>
       <c r="I172" s="98" t="n"/>
+      <c r="J172" s="53" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
     </row>
     <row r="173" ht="30" customHeight="1">
       <c r="A173" s="98" t="inlineStr">
@@ -8378,6 +8935,11 @@
         <v/>
       </c>
       <c r="I173" s="98" t="n"/>
+      <c r="J173" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="174" ht="30" customHeight="1">
       <c r="A174" s="98" t="inlineStr">
@@ -8418,6 +8980,11 @@
         <v/>
       </c>
       <c r="I174" s="98" t="n"/>
+      <c r="J174" s="53" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
     </row>
     <row r="175" ht="30" customHeight="1">
       <c r="A175" s="98" t="inlineStr">
@@ -8458,6 +9025,11 @@
         <v/>
       </c>
       <c r="I175" s="98" t="n"/>
+      <c r="J175" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="176" ht="30" customHeight="1">
       <c r="A176" s="98" t="inlineStr">
@@ -8498,6 +9070,11 @@
         <v/>
       </c>
       <c r="I176" s="98" t="n"/>
+      <c r="J176" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="177" ht="30" customHeight="1">
       <c r="A177" s="98" t="inlineStr">
@@ -8538,6 +9115,11 @@
         <v/>
       </c>
       <c r="I177" s="98" t="n"/>
+      <c r="J177" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="178" ht="30" customHeight="1">
       <c r="A178" s="98" t="inlineStr">
@@ -8578,6 +9160,11 @@
         <v/>
       </c>
       <c r="I178" s="98" t="n"/>
+      <c r="J178" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="179" ht="30" customHeight="1">
       <c r="A179" s="98" t="inlineStr">
@@ -8618,6 +9205,11 @@
         <v/>
       </c>
       <c r="I179" s="98" t="n"/>
+      <c r="J179" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="180" ht="30" customHeight="1">
       <c r="A180" s="98" t="inlineStr">
@@ -8658,6 +9250,11 @@
         <v/>
       </c>
       <c r="I180" s="98" t="n"/>
+      <c r="J180" s="53" t="inlineStr">
+        <is>
+          <t>Determinística</t>
+        </is>
+      </c>
     </row>
     <row r="181" ht="30" customHeight="1">
       <c r="A181" s="98" t="inlineStr">
@@ -8698,6 +9295,11 @@
         <v/>
       </c>
       <c r="I181" s="98" t="n"/>
+      <c r="J181" s="53" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
     </row>
     <row r="182" ht="30" customHeight="1">
       <c r="A182" s="98" t="inlineStr">
@@ -8738,6 +9340,11 @@
         <v/>
       </c>
       <c r="I182" s="98" t="n"/>
+      <c r="J182" s="53" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
     </row>
     <row r="183" ht="30" customHeight="1">
       <c r="A183" s="98" t="inlineStr">
@@ -8778,6 +9385,11 @@
         <v/>
       </c>
       <c r="I183" s="98" t="n"/>
+      <c r="J183" s="53" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
     </row>
     <row r="184" ht="30" customHeight="1">
       <c r="A184" s="98" t="inlineStr">
@@ -8818,6 +9430,11 @@
         <v/>
       </c>
       <c r="I184" s="98" t="n"/>
+      <c r="J184" s="53" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
     </row>
     <row r="185" ht="30" customHeight="1">
       <c r="A185" s="98" t="inlineStr">
@@ -8858,6 +9475,11 @@
         <v/>
       </c>
       <c r="I185" s="98" t="n"/>
+      <c r="J185" s="53" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
     </row>
     <row r="186" ht="30" customHeight="1">
       <c r="A186" s="98" t="inlineStr">
@@ -8898,6 +9520,11 @@
         <v/>
       </c>
       <c r="I186" s="98" t="n"/>
+      <c r="J186" s="53" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
     </row>
     <row r="187" ht="30" customHeight="1">
       <c r="A187" s="98" t="inlineStr">
@@ -8938,16 +9565,22 @@
         <v/>
       </c>
       <c r="I187" s="98" t="n"/>
+      <c r="J187" s="53" t="inlineStr">
+        <is>
+          <t>Habilitadora</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:Q187"/>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="M48:Q48"/>
     <mergeCell ref="M40:Q40"/>
     <mergeCell ref="M35:Q35"/>
     <mergeCell ref="M43:Q43"/>
     <mergeCell ref="M34:Q34"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="M57:Q57"/>
     <mergeCell ref="M47:Q47"/>
     <mergeCell ref="M37:Q37"/>
     <mergeCell ref="A1:I1"/>
@@ -8958,9 +9591,12 @@
     <mergeCell ref="M36:Q36"/>
     <mergeCell ref="L3:N3"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="E5:E187" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>$L$5:$L$8</formula1>
+    </dataValidation>
+    <dataValidation sqref="J5:J187" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Agéntica,Habilitadora,Determinística"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>